<commit_message>
Upload this round of group-22 crawler fulltext, Excel marks, and the Astra/识典/wiki pipeline.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/第22组总览表.xlsx
+++ b/第22组总览表.xlsx
@@ -1160,7 +1160,7 @@
       </c>
       <c r="J16" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=古籍或诗文集，书名、作者和时代均待考。关键词=彭阳新集、彭陽新集、新集、彭阳、彭陽、彭阳文集。母项=历代总集、别集书目、地方志艺文志及人物传、《四库全书总目》及续修目录、敦煌、宋元明清古籍目录。候选站=https://www.google.com/search?q=%22%E5%BD%AD%E9%98%B3%E6%96%B0%E9%9B%86%22; https://commons.wikimedia.org/w/index.php?search=%E5%BD%AD%E9%98%B3%E6%96%B0%E9%9B%86&amp;title=Special%3AMediaSearch&amp;type=image。未确认作者、朝代、卷数及版本；可能是亡佚别集或地方志著录书名，不能据题名宣称已有全文。</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=公文题类，可能是公报中的单件文件。关键词=大总统指令、大總統指令、大总统 指令 政府公报、大總統 指令 臨時政府公報、大总统指令 第 号 呈。母项=《政府公报》（北京政府时期，1912—1928年；检索其中“指令”栏目）、《临时政府公报》（南京临时政府时期，1912年；仅作为待排查来源）。候选站=。未找到可核验的具体文件页。“大总统指令”不是足以唯一识别文献的题名；应先从引用上下文提取总统姓名、日期、指令号、受文机关或起首语，再定位公报期号及页码。上述年份是母刊排查范围，不是已确定的刊载年期。</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=方志。关键词=庆城县志、慶城縣志、庆城县志 甘肃、庆城县志 陕西、庆城旧志。母项=《庆阳府志》、《甘肃通志》、《庆城县志》历代版本、《中国地方志集成·甘肃府县志辑》。候选站=https://zh.wikisource.org/w/index.php?search=%E5%BA%86%E5%9F%8E%E5%8E%BF%E5%BF%97&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。需先确认甘肃庆城县还是其他同名行政地；若为甘肃，应查《庆阳府志》疆域、建置、金石和艺文门及县志不同修纂年份。</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="J29" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似文物名称、图版题签或藏品说明。关键词=绢画幡带、絹畫幡帶、绢画 幡带、絹畫 幡 帶、敦煌 绢画 幡、藏经洞 幡带 题记。母项=敦煌藏经洞绢画、幡画藏品目录及图录（待核定具体书名）、大英博物馆、英国图书馆及法国吉美博物馆相关藏品记录（仅为排查方向）。候选站=。未找到具体藏品页或图版页，也未确认其属于敦煌文物。宜先核对原文是否把器物名称加了书名号；需补充出土地、收藏机构、藏品编号、图版号或幡带题记。检索Commons时应使用确定后的藏品编号，不能将泛称相近的幡画视为同一件。</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="J32" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似地方志、区域概况或调查报告的章节标题。关键词=民族和人口、民族與人口、民族与人口、人口和民族、民族 人口 地方志、民族和人口 目录。母项=相关地区的省志、县志、民族志或区域概况（地区及书名均待核）、民族社会历史调查资料中的地区概况章节（待核）。候选站=。未找到能够归属到具体母书的章节页。应以引用上下文中的地区名、民族名及人口统计年份缩小范围，再查目录与章节页码。题名通用，不能据此指定某部方志的卷次。若归属现代著作或2015年后整理本，仅提供书目、馆藏或合法章节访问线索，不提供整本下载。</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="J36" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊新闻/教育行政档案条目。关键词=连阳化瑶进行设化瑶学校十间招瑶民子弟入学、連陽化瑤進行設化瑤學校十間招瑤民子弟入學、连阳 化瑶 学校 十间、瑶民子弟入学、连阳 瑶民教育、连县 阳山 连山 瑶族教育。母项=民国时期广东报刊、广东省政府公报、广东教育行政档案、连阳地方报刊及地方志教育志。候选站=https://commons.wikimedia.org/w/index.php?search=%E9%80%A3%E9%99%BD%E5%8C%96%E7%91%A4%E5%AD%B8%E6%A0%A1&amp;title=Special:MediaSearch&amp;type=document; https://zh.wikisource.org/w/index.php?search=%E9%80%A3%E9%99%BD%E7%91%A4%E6%B0%91%E6%95%99%E8%82%B2&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。题名像报刊标题或档案目录标题，疑有 OCR 误读；“化瑶”可能是“化导瑶民”或“设化瑶学校”，应按连阳、连县、阳山、连山及繁简体组合检索。</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊新闻/教育行政公文。关键词=注意边民教育粤增设瑶民施教站、注意邊民教育粵增設瑤民施教站、边民教育、邊民教育、瑶民施教站、瑤民施教站。母项=民国时期广东报刊、广东省政府公报、广东教育厅公报、广东边民教育档案。候选站=https://commons.wikimedia.org/w/index.php?search=%E7%91%A4%E6%B0%91%E6%96%BD%E6%95%99%E7%AB%99&amp;title=Special:MediaSearch&amp;type=document; https://zh.wikisource.org/w/index.php?search=%E7%91%A4%E6%B0%91%E6%96%BD%E6%95%99%E7%AB%99&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。标题格式明显接近报刊简讯，需先确定报刊名称、出版地和年份；“粤”可能是广东省简称，也可能是标题截断。</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="J40" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘简报/文物图录条目。关键词=深圳大黄沙遗址出土石拍、深圳 大黄沙遗址 石拍、大黄沙遗址、大黄沙 石拍、深圳 新石器时代 石拍、大黄沙遗址出土遗物。母项=《深圳文物志》、《深圳考古发现与研究》、广东省文物考古研究所考古发掘简报、深圳地区新石器时代遗址调查报告。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%A4%A7%E9%BB%83%E6%B2%99%E9%81%BA%E5%9D%80&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=%E5%A4%A7%E9%BB%83%E6%B2%99%E9%81%BA%E5%9D%80&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。“石拍”是器物名称或图版说明，不是独立出版物；应查《深圳文物志》相关遗址条目及考古简报的图版、器物目录。</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="J41" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古调查/遗址发掘报告条目。关键词=高要县龙一乡蚬壳洲贝丘遗址、高要縣龍一鄉蜆殼洲貝丘遺址、高要 蚬壳洲 贝丘遗址、龍一鄉 蚬壳洲、广东 贝丘遗址 高要、蚬壳洲遗址。母项=《广东省文物考古研究所集刊》、《广东文物考古三十年》、《肇庆文物志》、《高要县志》文物志/文化遗产志、珠江三角洲史前考古调查报告。候选站=https://commons.wikimedia.org/w/index.php?search=%E8%9C%86%E6%AE%BC%E6%B4%B2%E8%B2%9D%E4%B8%98%E9%81%BA%E5%9D%80&amp;title=Special:MediaSearch&amp;type=document; https://zh.wikisource.org/w/index.php?search=%E8%9C%86%E6%AE%BC%E6%B4%B2%E8%B2%9D%E4%B8%98%E9%81%BA%E5%9D%80&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。该条目应是考古报告中的遗址名或章节名，可能存在地名异写；需并检“龙一/龍一”“蚬壳洲/蜆殼洲”及肇庆、高要旧县名。</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="J42" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=文物图录/考古报告器物条目。关键词=广宁铜鼓岗圆首有格无箍剑、廣寧銅鼓崗圓首有格無箍劍、铜鼓岗 圆首有格无箍剑、廣寧 銅鼓崗 劍、广东 青铜剑 铜鼓岗、广宁出土青铜器。母项=《广宁县志》文物志、《肇庆文物志》、《广东出土文物》、广东省博物馆藏青铜器图录、广东地区先秦考古报告。候选站=https://commons.wikimedia.org/w/index.php?search=%E9%8A%85%E9%BC%93%E5%B4%97%E5%9C%93%E9%A6%96%E6%9C%89%E6%A0%BC%E7%84%A1%E7%AE%8D%E5%8A%8D&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=%E9%8A%85%E9%BC%93%E5%B4%97%E5%9C%93%E9%A6%96%E6%9C%89%E6%A0%BC%E7%84%A1%E7%AE%8D%E5%8A%8D&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。该名称是器物定名，可能只出现在图录图版说明或地方文物普查表中；应重点查《广宁县志》文物志、肇庆地区文物图录及广东省博物馆藏品目录。</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑刻。关键词=迎仙 平寇碑、迎仙寺 平寇碑、迎仙平寇碑 碑文、迎仙 平寇、迎仙碑。母项=当地县志金石志、《中国文物地图集》相关省卷、地方碑刻辑录、地方文物普查资料。候选站=https://zh.wikisource.org/w/index.php?search=%E8%BF%8E%E4%BB%99%E5%B9%B3%E5%AF%87%E7%A2%91&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。缺少年代、地点和立碑者，无法确定所属县域；应结合林靖凯条目的上下文或引用出处，优先追查县志金石门。</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="J46" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘简报，可能为期刊或地方考古报告子项。关键词=安徽 合肥 大雁墩 遗址 发掘简报、合肥 大雁墩 新石器时代、大雁墩遗址 发掘报告、大雁墩遗址 考古。母项=《考古》相关年份及期刊目录、《文物》相关年份及期刊目录、安徽省文物考古研究所考古调查发掘报告、合肥市文物考古研究所考古简报汇编。候选站=https://www.baidu.com/s?wd=%E5%AE%89%E5%BE%BD+%E5%90%88%E8%82%A5+%E5%A4%A7%E9%9B%81%E5%A2%A9+%E9%81%97%E5%9D%80+%E5%8F%91%E6%8E%98%E7%AE%80%E6%8A%A5; https://scholar.google.com/scholar?q=%22%E5%A4%A7%E9%9B%81%E5%A2%A9%22+%E5%90%88%E8%82%A5+%E9%81%97%E5%9D%80。目前未核实到具体卷期、作者或可公开阅读页面。</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2587,7 @@
       </c>
       <c r="J47" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似考古调查或发掘简报，未确认独立出版。关键词=安徽合肥东郊古砖墓、安徽合肥東郊古磚墓、合肥 东郊 砖室墓 发掘 简报、合肥 東郊 古墓 墓砖。母项=待查期刊：《考古》《考古学报》《文物》历年目录；尚未确认刊载关系、年期与页码、待查地方文物资料：合肥地区考古调查报告及文物志的古墓葬条目。候选站=。未找到可核验的具体文章页。先以“合肥＋东郊＋砖墓／砖室墓”查篇名索引，再从摘要、参考文献核对作者、地点、年代和页码；完整题名可能是旧刊篇名或图片说明。现代期刊仅提供书目、馆藏或DOI线索，不提供整本下载。</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="J48" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折或奏议，非独立书籍。关键词=奉旨措置两淮官田事宜奏、两淮 官田 奏、措置两淮官田、两淮盐政 官田、官田事宜 奏折。母项=《清实录》两淮官田相关条目、《清经世文编》田制、盐政类、《皇清奏议》或清代奏折汇编、中国第一历史档案馆清代宫中档朱批奏折、军机处档折件。候选站=https://www.baidu.com/s?wd=%22%E5%A5%89%E6%97%A8%E6%8E%AA%E7%BD%AE%E4%B8%A4%E6%B7%AE%E5%AE%98%E7%94%B0%E4%BA%8B%E5%AE%9C%E5%A5%8F%22; https://zh.wikisource.org/wiki/%E6%B8%85%E5%AE%9E%E9%8C%84。未核实到该奏折的确切朝代、奏者及《清实录》卷次；维基文库链接仅为具体母项，不能视为该奏折全文。</t>
         </is>
       </c>
     </row>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="J50" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代刑案题本或档案目录拟题，具体档案类别待核。关键词=寿州 李六十 张文华、壽州 李六十 張文華、李六十 戏戳毙 绞监候、李六十 戲戳斃 絞監候、寿州 回民 刑科题本、壽州 回民 刑部 命案。母项=待查档案：中国第一历史档案馆清代刑科题本、刑部相关命案目录；尚未确认全宗及档号、待查汇编：清代回族史料、安徽清代刑案档案选编；尚未确认实际收录书名。候选站=。未找到具体档案目录页或录文页。题名结构提示其可能是目录编目拟题，应优先检索罕见人名“李六十”，再以死者姓名、寿州、案由交叉核对。定位至少需要具奏人、具奏年月、档号之一，不能据题名推定朝代年号或卷次；汇编收录需另核目录和页码。</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="J51" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代学校行政档案或史料汇编子项。关键词=怀宁县 私立清真小学 呈文、懷寧縣 私立清真小學 呈文、怀宁 清真小学 立案、安庆 清真小学 教育局、懷寧 回教 教育 私立小學。母项=待查档案：安徽省、安庆市及怀宁县相关档案馆的民国教育行政和私立学校立案档案、待查地方文献：怀宁县志、安庆地方教育志及回族教育史料中的清真小学条目；版本、卷次待核。候选站=。未找到具体呈文目录或影像页。“呈文”可能只是一组文件的概括性标题，需查呈送机关、日期、事由及附件。检索历史怀宁县与安庆城区资料时应核对当时行政范围，不能仅按现今县域筛选。后出整理本仅查书目、馆藏和目录，不提供整本下载。</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="J52" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=日期型条目，可能为日记、书信、报刊或编年史子项。关键词=一九二七年五月四日、一九二七年五月四日 日记、一九二七年五月四日 日記、1927年5月4日、民国十六年五月四日、民國十六年五月四日。母项=无法确定母项：需先取得原引用的作者、脚注、相邻条目或引文、取得作者后再查其日记、书信集或年谱；取得报刊名后再查1927年5月4日当日各版。候选站=。未找到能唯一对应的具体页。日期不能独立识别文献，也不能据此指定某部日记或报纸。应先确认日期是条目标题、文件落款还是报刊出版日，并核对公历或农历；“安徽、回民”仅为结合清单上下文的辅助词，不是已确认内容。</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="J53" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似地方文史文章或人物纪念文章。关键词=爱国将领周元与蒙城守土抗战、愛國將領周元與蒙城守土抗戰、周元 蒙城 守土 抗战、周元 蒙城 保卫战 1938、周元 蒙城 文史资料。母项=待查地方政协文史资料：蒙城地方文史资料各辑目录，重点查抗战及人物专题；具体书名、辑次待核、待查期刊：《江淮文史》《安徽史学》篇名索引；尚未确认刊载关系、待查地方。候选站=。未找到题名对应的具体文章页、作者或年期。1938年仅作蒙城抗战事件检索线索，不是本文出版年。先搜“周元＋守土”，再查地方文史资料目录及相关研究的参考文献，区别同题转载与原刊。现代期刊和版权期内文史资料仅查书目、馆藏或DOI，不提供整本下载。</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2909,7 @@
       </c>
       <c r="J54" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=红军政治工作文件的摘录，疑为档案汇编子项。关键词=中国工农红军四方面军总政治部 宣传教育工作 决议草案、中國工農紅軍四方面軍總政治部 宣傳教育工作 決議草案、红四方面军 总政治部 宣传教育 决议、红军第四方面军 宣传 教育 草案、宣传教育工作决议草案 摘录。母项=待查汇编：《中国工农红军第四方面军战史资料选编》；需核目录、文件日期及页码，尚未确认收录、待查汇编：军队政治工作历史资料及革命历史文件汇集中的红四方面军文件；具。候选站=。未找到对应文件的具体目录页或录文页。优先删除“摘录”检索原文件，再比较“四方面军／第四方面军”和“关于／无关于”等题名差异。机关可作团体作者线索；必须核对文件日期及摘录来源，不能将汇编出版年当作文件形成时间。版权期内汇编仅提供书目、馆藏线索，不提供整本下载。</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="J55" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似地方志章节、宗教志条目或地方文史文章。关键词=和县 伊斯兰教、和縣 伊斯蘭教、和县志 宗教 回教、和縣志 清真寺、历阳 回民 清真寺、歷陽 回教。母项=待查《和县志》各版本：宗教、民族、风俗或寺观相关章节；未确认实际篇章名称及卷次、待查安徽省志中的宗教相关分志及地方宗教资料：和县、清真寺相关条目；具体版本待核、。候选站=。未找到对应具体章节页。“和县伊斯兰教”可能是引用者概括的条目名。旧方志应同时查“回教、清真寺、礼拜寺”等词，并优先在识典古籍、维基文库或Commons核对实际版本目录与影像；未确认页面前不拼造章节URL。现代地方志和后出整理本仅查书目、馆藏线索，不提供整本下载。</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="J56" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=墓志。关键词=李神德墓志、李神德 墓誌、李神德墓志铭、李神德墓誌銘、李神德 墓志录文。母项=《全唐文》、《唐代墓志汇编》、《隋唐五代墓志汇编》、《唐代墓志铭汇编续集》、墓志录文与书法碑帖资料。候选站=https://commons.wikimedia.org/w/index.php?search=Li+Shende+epitaph&amp;title=Special%3ASearch; https://zh.wikisource.org/w/index.php?search=%E6%9D%8E%E7%A5%9E%E5%BE%B7%E5%A2%93%E5%BF%97&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。应补查卒年、籍贯、出土地和时代；墓志可能仅作为《唐代墓志汇编》的编号条目收录，现代整理本通常受版权限制。</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="J57" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似文物图版题名、图片说明或艺术史论著子项。关键词=云居寺 辽代 石经塔 乐舞 伎乐人 砖雕、雲居寺 遼代 石經塔 樂舞 伎樂人 磚雕、云居寺 石经塔 伎乐砖雕、云居寺 辽塔 舞乐砖雕、云居寺 伎乐 砖雕、雲居寺 技樂 磚雕。母项=待查云居寺及石经相关文物调查报告、建筑图录和馆藏图录；需先核对寺址及塔名、待查中国音乐史、舞蹈史和辽代雕塑图录中的伎乐砖雕图版目录；具体书名、图版号待核、待查C。候选站=。未找到具体图版、文物记录或文章页。题名中的“乐舞伎乐人”可能来自图注拼接，宜拆分检索；“技乐”仅作可能的OCR误识别变体。不能仅凭“云居寺”确定所在地，需核对寺址、塔名、出土或收藏单位、图版号。若母项为现代图录或版权期内著作，仅查书目和馆藏，不提供整本下载。</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="J59" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似宗教器物名称或图录条目。关键词=札嘛噜手鼓、札嘛嚕手鼓、札嘛噜、扎玛鲁 手鼓、扎瑪魯 手鼓、达玛如 鼓。母项=藏传佛教法器图录或博物馆藏品目录（待核定具体书名）、民族乐器图录中的手鼓条目（待核）。候选站=。未找到与该题名对应的具体藏品或文献页。应先核对“札嘛噜”是否为旧译、方言转写或OCR误识，再依据材质、尺寸、收藏地及图版号定位。相关音译词仅用于扩检，不能证明某件damaru就是原条目。</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3185,7 @@
       </c>
       <c r="J60" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近现代报刊新闻或专题资料。关键词=声援山东惨案的请愿斗争、声援山东惨案、山东惨案 请愿、五三惨案 请愿斗争、济南惨案 请愿、山东惨案 反帝运动。母项=1928年前后民国报刊、《申报》、《民国日报》、《大公报》、国民政府外交档案及山东惨案史料汇编。候选站=。题名更像报刊专题标题或后来的史料篇名，尚未核定具体报纸、日期和版次。检索时应重点核对1928年5月至1929年的报刊，并检索“济南惨案”“五三惨案”“山东惨案”等异称。</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="J61" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=政府公文、训令或报刊公示。关键词=令中山公园董事会、中山公园董事会、训令 中山公园、令 中山公园 董事会、中山公园 公文。母项=民国政府公报、地方政府公报、中山公园董事会档案、各地中山公园碑刻及管理档案。候选站=。题名缺少发文机关、地点和日期。“中山公园”可能指北京、上海、广州、南京或其他城市的同名公园，不能据此确定独立文献。应先结合林靖凯清单的地域和年代定位母项。</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="J63" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘报告或考古期刊论文。关键词=贵南尕马台遗址出土西城驿文化陶器、贵南 尕马台遗址、尕马台 西城驿文化、西城驿文化 陶器、贵南 尕马台 考古。母项=《考古》、《考古与文物》、《青海考古学报》、青海省文物考古研究所考古调查与发掘报告、西城驿文化研究论文集。候选站=。未核定到具体作者、刊名、年份、卷期或页码。题名可能是论文中的章节标题、图版说明或考古报告子项，不能按独立书籍处理。</t>
         </is>
       </c>
     </row>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="J67" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似连续出版物，也可能是报纸专栏或附刊。关键词=矿业周报、礦業周報、礦業週報、矿业周报 创刊、礦業週報 出版者、矿业周报 馆藏。母项=如为独立期刊：检索民国期刊联合目录及馆藏目录中的同名刊记录、如为专栏或附刊：须根据报头、版次和出版地回溯所属报纸。候选站=。未找到可核验的同名刊书目记录或具体期页，无法可靠填写创刊年、出版机关和卷期。优先提取引文中的年份、期号、出版地及编辑者；同时检索“周／週”异体。不能用《矿业月报》等近名刊代替。</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="J68" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=文物图录条目或博物馆藏品说明。关键词=彩绘云纹釜甑、彩绘 云纹 釜甑、云纹釜甑、釜甑 彩绘、彩绘陶 釜甑。母项=出土文物图录、博物馆藏品目录、秦汉考古器物图录、墓葬发掘报告、中国国家博物馆或地方博物馆藏品资料。候选站=。题名极可能是器物名、图版题名或展览标签，而非独立文献。缺少出土地、年代、收藏单位和器物编号，无法核定具体页面。</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="J70" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=北魏碑刻或碑文录，非独立书籍。关键词=北魏 正始元年 豳州刺史 山累立、山累立 追献寺碑、追献寺碑、豳州刺史 碑、504 豳州 碑刻。母项=《金石萃编》北魏碑刻卷、《校碑随笔》及北魏碑刻目录、《陕甘宁青金石录》或陕西、甘肃地方金石志、墓志录文、碑刻录文数据库。候选站=https://www.baidu.com/s?wd=%E5%8C%97%E9%AD%8F+%E6%AD%A3%E5%A7%8B%E5%85%83%E5%B9%B4+%E8%B1%B3%E5%B7%9E%E5%88%BA%E5%8F%B2+%E5%B1%B1%E7%B4%AF%E7%AB%8B+%E8%BF%BD%E7%8C%AE%E5%AF%BA%E7%A2%91; https://commons.wikimedia.org/w/index.php?search=%E8%BF%BD%E7%8C%AE%E5%AF%BA%E7%A2%91&amp;title=Special:MediaSearch&amp;go=Go&amp;type=image。未核实到可确认的碑刻目录条目、碑文录文或拓片页面。</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="J71" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代军机处或地方官员奏折、片，非独立书籍。关键词=同治八年 二月二十三日 置买军械 回党、复奏 刑部 咨查 拿获 军械、回党 军械 奏片、刑部咨查 军械、同治八年 奏折。母项=《清代军机处档案辑录》同治朝相关档案、中国第一历史档案馆军机处录副奏折、《清实录·穆宗毅皇帝实录》同治八年二月、清代刑部档案及地方奏折汇编。候选站=https://www.baidu.com/s?wd=%E5%90%8C%E6%B2%BB%E5%85%AB%E5%B9%B4+%E4%BA%8C%E6%9C%88%E4%BA%8C%E5%8D%81%E4%B8%89%E6%97%A5+%E7%BD%AE%E4%B9%B0%E5%86%9B%E6%A2%B0+%E5%9B%9E%E5%85%9A; https://zh.wikisource.org/wiki/%E5%BE%A1%E5%AE%9A%E5%85%AD%E9%83%A8%E5%88%99%E4%BE%8B。未核实到具体档号、奏者、收藏汇编卷册或公开全文。</t>
         </is>
       </c>
     </row>
@@ -3737,7 +3737,7 @@
       </c>
       <c r="J72" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近现代报刊消息、调查材料或地方社会调查。关键词=沙苑附近回民的土产出售、沙苑 回民 土产、沙苑附近 回民、回民 土产出售、沙苑 回民经济、沙苑 回民社会调查。母项=民国报刊、西北社会调查报告、回教或伊斯兰教刊物、陕西、甘肃地方志、西北经济调查资料汇编。候选站=。“沙苑”可能指陕西大荔、朝邑一带的沙苑地区，也可能是其他地名。题名形式接近报刊栏目或调查记录，应结合刊发年代、报刊名称和版面检索。</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="J73" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=抗战时期报刊新闻、团体通电或会议记录。关键词=回教民众抗日救国会、抗日救国会 紧急会议、决议通电全国 对日宣战、回教民众 抗日、回民抗日救国会、对日实行宣战。母项=抗战时期《申报》、《中央日报》、《大公报》、《回教群众》及其他回教刊物、全国各界抗日救国会史料、抗日战争时期报刊资料汇编。候选站=。题名明显是报纸标题，可能发表于全面抗战爆发前后或七七事变后。需以“回教民众抗日救国会”“回民抗日救国会”“通电全国”等短语检索具体日期和报纸版次。</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="J74" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=墓志铭，题名高度重复，需以时代、出土地和墓主身份定位。关键词=李宗师 墓志铭、李宗师墓志、李宗师 墓志 录文、宗师 李氏 墓志、李宗师 墓志 拓片。母项=《全唐文》及唐代墓志辑录、《唐代墓志汇编》、《新中国出土墓志》、墓志录文站、地方出土墓志图录。候选站=https://www.baidu.com/s?wd=%22%E6%9D%8E%E5%AE%97%E5%B8%88%E5%A2%93%E5%BF%97%E9%93%AD%22; https://commons.wikimedia.org/w/index.php?search=%E6%9D%8E%E5%AE%97%E5%B8%88%E5%A2%93%E5%BF%97&amp;title=Special:MediaSearch&amp;go=Go&amp;type=image。仅凭题名无法排除同名墓志；未找到可确认年代、出土地或墓主身份的具体页面。</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="J78" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊连载、考察报告或民族调查资料。关键词=民族考察团在川之行踪、民族考察团 四川、民族考察团 在川、四川 民族考察、民族调查团 四川 行踪。母项=民国报刊、中央研究院或国立中央大学民族调查资料、四川地方调查报告、西南民族调查文献汇编、民族学、人类学期刊。候选站=。题名可能是报刊连载标题，未找到可核验的作者、考察团名称、刊名、日期或卷期。四川在民国时期有多类民族调查团，需先确定机构和年代。</t>
         </is>
       </c>
     </row>
@@ -4131,12 +4131,12 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://zh.wikisource.org/wiki/%E6%B0%B4%E6%B5%92%E6%96%B0%E4%BC%A0/%E5%9B%9B%E5%8D%81%E4%BA%8C%20%E4%B8%9C%E4%BA%AC%E5%9F%8E%E9%A9%AC%E5%BF%A0%E8%BE%9E%E4%BC%97%E6%9D%B0%20%E7%9B%B8%E5%9B%BD%E5%AF%BA%E6%99%BA%E6%B7%B1%E9%81%87%E4%BB%87%E4%BA%BA</t>
         </is>
       </c>
       <c r="G81" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H81" s="10" t="inlineStr">
@@ -4146,12 +4146,12 @@
       </c>
       <c r="I81" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>公开录文页</t>
         </is>
       </c>
       <c r="J81" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似考古报告简称，也可能是地名条目。关键词=东京城、東京城、東京城 渤海國上京龍泉府址、东京城 渤海 上京龙泉府 发掘、東京城 原田淑人 駒井和愛、東京城 東亞考古學會 1939。母项=《東京城：渤海國上京龍泉府址の發掘調査》，原田淑人、駒井和愛，1939年，东亚考古学会；作为优先核查的书目线索、《東方考古學叢刊》甲種第五冊（上述报告的丛书定位。候选站=。未找到可核验的具体书目页或扫描页。上述考古报告是较具体的核查方向，但不能确认就是清单所指。可据完整日文题名、作者和丛刊册次查日本国立国会图书馆及CiNii Books的单书记录；若引文内容不是渤海上京遗址，应转查地方志中的东京城地名条目。；2026-09-22 组内异源扫描核验，已保存匹配录文。</t>
         </is>
       </c>
     </row>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="J82" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代题本、奏折或宫中档案条目。关键词=盛京户部侍郎 格尔布、格爾布 赫哲费雅喀、动用库银 采买毛蓝布、赏赐赫哲费雅喀族、盛京户部侍郎题、毛蓝布 赫哲。母项=《宫中档奏折》、《宫中档满文奏折》、《军机处档折件》、《清代档案史料丛编》、《清实录》相关卷、清代盛京户部题本档案。候选站=。题名为档案目录式标题，存在繁简和满汉译名差异。“格爾布”应同时检索“格尔布”， “赫哲费雅喀”应检索“赫哲”“费雅喀”“费雅喀族”。尚未核定具体档号、年代、档案馆、卷册或公开影像页。</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="J83" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案或地方行政公文，非独立书籍。关键词=署盖平县、署理盖平县、盖平县公文、盖平縣、奉天盖平县、盖平县知县。母项=清代奉天府档案、盖平县志、奉天省政府档案、东北地区地方档案汇编。候选站=https://zh.wikisource.org/wiki/Special:Search?search=%E7%9B%96%E5%B9%B3%E5%8E%BF; https://commons.wikimedia.org/w/index.php?search=%E7%9B%96%E5%B9%B3%E5%8E%BF&amp;title=Special:MediaSearch&amp;type=image。未确认具体档案馆、档号、年代或所属汇编，不能据题名定位全文。</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="J84" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊文章或时政资料条目。关键词=蒙边将分设卫戍军、蒙边卫戍军、蒙古边防、卫戍军、蒙边军制、蒙邊將分設衛戍軍。母项=民国报刊、政府公报、陆军部公报、蒙藏事务档案汇编。候选站=https://zh.wikisource.org/wiki/Special:Search?search=%E8%92%99%E8%BE%B9%E5%8D%AB%E6%88%8D%E5%86%9B; https://commons.wikimedia.org/w/index.php?search=%E8%92%99%E8%BE%B9%E5%8D%AB%E6%88%8D%E5%86%9B&amp;title=Special:MediaSearch&amp;type=image。题名更像报刊标题或公报摘录，缺少刊名、日期、版次，未找到具体期号或全文页。</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="J85" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊文章或政治论述条目。关键词=蒙警与蒙古王公、蒙警、蒙古王公、蒙古警察、蒙警與蒙古王公、蒙藏政治。母项=民国报刊、蒙藏委员会公报、蒙古问题资料汇编、近代边疆政治文献。候选站=https://zh.wikisource.org/wiki/Special:Search?search=%E8%92%99%E8%AD%A6%E8%88%87%E8%92%99%E5%8F%A4%E7%8E%8B%E5%85%AC; https://commons.wikimedia.org/w/index.php?search=%E8%92%99%E8%AD%A6%E8%88%87%E8%92%99%E5%8F%A4%E7%8E%8B%E5%85%AC&amp;title=Special:MediaSearch&amp;type=image。未确认刊名、作者、年份或卷期，不能认定为独立著作。</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="J87" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=诰书或历史文献中的子项。关键词=洪武皇帝封长河西土官藏卜诰书、长河西土官、藏卜、诰书、洪武封藏卜、長河西土官。母项=《明太祖实录》、《皇明诏令》、《明会典》、西番土官封授文书、明代诰敕汇编。候选站=https://zh.wikisource.org/wiki/Special:Search?search=%E9%95%BF%E6%B2%B3%E8%A5%BF%E5%9C%9F%E5%AE%98%E8%97%8F%E5%8D%9C; https://commons.wikimedia.org/w/index.php?search=%E9%95%BF%E6%B2%B3%E8%A5%BF%E5%9C%9F%E5%AE%98&amp;title=Special:MediaSearch&amp;type=image。可能是《明太祖实录》或诰敕汇编中的单篇文书，未找到可核验的具体卷次或章节页。</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="J89" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=古代史书中的事件条目。关键词=吐蕃击吐谷浑、吐蕃攻吐谷浑、吐谷浑、吐蕃与吐谷浑战事、吐蕃擊吐谷渾。母项=《资治通鉴》唐纪、《旧唐书·吐蕃传》、《新唐书·吐蕃传》、《册府元龟》。候选站=https://zh.wikisource.org/wiki/Special:Search?search=%E5%90%90%E8%95%83%E5%87%BB%E5%90%90%E8%B0%B7%E6%B8%BE; https://zh.wikisource.org/wiki/Special:Search?search=%E5%90%90%E8%B0%B7%E6%B8%BE。找到明确母题线索，但未确认该标题对应的具体编纂者、卷次或独立页面。</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="J90" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似考古报告章节、墓葬资料条目或图版标题。关键词=曲贡墓葬、曲貢墓葬、曲贡 墓葬、拉萨曲贡 墓葬、拉薩曲貢 墓葬、拉萨曲贡 1999 目录。母项=《拉萨曲贡》，中国社会科学院考古研究所、西藏自治区文物局编著，中国大百科全书出版社，1999年；优先核查目录中的墓葬相关内容。候选站=。未找到题为“曲贡墓葬”的具体章节页，不能确认它是独立论文或上述报告中的正式章名。应以墓号、发掘年份、墓地位置和图版号核对《拉萨曲贡》的目录及索引；卷次、章次和页码尚未核实。该现代考古报告仅提供书目与馆藏检索线索，不提供整本下载。</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="J91" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代宫廷瓷器藏品条目。关键词=斗花团花纹碗、斗彩团花纹碗、雍正碗、雍正斗彩、清宫瓷器、鬥花團花紋碗。母项=故宫博物院藏清雍正瓷器、《故宫博物院藏文物珍品全集·五彩·斗彩》、清宫旧藏瓷器图录。候选站=https://commons.wikimedia.org/w/index.php?search=%E9%9B%8D%E6%AD%A3%E6%96%97%E5%BD%A9%E7%A2%97&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/wiki/Special:Search?search=%E9%9B%8D%E6%AD%A3%E6%96%97%E5%BD%A9。未找到与该精确器名对应的公开藏品页面、器物编号或图录卷页。</t>
         </is>
       </c>
     </row>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="J92" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代宫廷织绣或服饰类藏品条目。关键词=红色地联珠式平安如意纹织金妆花缎夹碗套、红色地联珠纹、平安如意纹、织金妆花缎、夹碗套、清代织金。母项=故宫博物院藏清代织绣、清宫内务府造办处档案、清代宫廷织绣图录、中国丝绸博物馆藏品目录。候选站=https://commons.wikimedia.org/w/index.php?search=%E7%BB%87%E9%87%91%E5%A6%86%E8%8A%B1%E7%BC%8E&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/wiki/Special:Search?search=%E7%BB%87%E9%87%91%E5%A6%86%E8%8A%B1%E7%BC%8E。名称高度像博物馆藏品数据库的单件著录，未找到公开藏品编号、馆藏机构或图录页。</t>
         </is>
       </c>
     </row>
@@ -4703,7 +4703,7 @@
       </c>
       <c r="J93" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=金属器或博物馆藏品条目。关键词=寿字纹葫芦形银质酒壶、寿字纹银酒壶、葫芦形银壶、银质酒壶、寿字纹银壶、壽字紋葫蘆形銀質酒壺。母项=清代金银器图录、故宫博物院藏金银器、中国国家博物馆藏金银器、地方博物馆金银器藏品目录。候选站=https://commons.wikimedia.org/w/index.php?search=%E8%91%AB%E8%8A%A6%E5%BD%A2%E9%93%B6%E5%A3%B6&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/wiki/Special:Search?search=%E5%A3%BD%E5%AD%97%E7%B4%8B%E9%8A%80%E5%A3%BA。未找到精确器名对应的公开馆藏编号、年代、尺寸或图录卷页，不能确认具体藏品。</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="J94" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑刻。关键词=南岩渡碑、南巖渡碑、南岩 渡口 碑、南岩渡 碑文、南岩碑刻。母项=当地县志金石志、当地水利交通志、《中国文物地图集》相关省卷、地方碑刻辑录。候选站=https://zh.wikisource.org/w/index.php?search=%E5%8D%97%E5%B2%A9%E6%B8%A1%E7%A2%91&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。题名缺少地点和年代，极可能是县志金石门下的单项；应从南岩山、南岩寺、渡口所在地和碑额异体字继续定位。</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="J95" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代边疆奏折，非独立书籍。关键词=荣全 伊犁领队 锡伯营总管 被逐来塔、荣全 奏 伊犁 锡伯营、来塔 情形折、锡伯营总管 被逐、伊犁领队大臣 荣全 奏折。母项=《清代新疆满文档案汉译编》、《清代新疆档案选辑》、《清实录·德宗景皇帝实录》或同治、光绪朝相关卷、清代军机处录副奏折、朱批奏折。候选站=https://www.baidu.com/s?wd=%E8%8D%A3%E5%85%A8+%E4%BC%8A%E7%8A%81%E9%A2%86%E9%98%9F+%E9%94%A1%E4%BC%AF%E8%90%A5%E6%80%BB%E7%AE%A1+%E8%A2%AB%E9%80%90%E6%9D%A5%E5%A1%94; https://zh.wikisource.org/wiki/%E6%B8%85%E5%AE%9E%E5%BD%95。未核实到具体年代、奏折档号或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -4841,7 +4841,7 @@
       </c>
       <c r="J96" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代新疆事务奏折，非独立书籍。关键词=奏报 解送 辛亥年 新疆 绸缎 起程日期、辛亥年 新疆 绸缎 解送、新疆绸缎 起程日期 奏、解送绸缎 新疆 奏折、辛亥年 绸缎 起程。母项=《清代新疆档案选辑》、《清代新疆满文档案汉译编》、《清实录》相关朝代辛亥年条目、清代军机处录副奏折及户部、工部档案。候选站=https://www.baidu.com/s?wd=%E8%A7%A3%E9%80%81%E8%BE%9B%E4%BA%A5%E5%B9%B4%E6%96%B0%E7%96%86%E7%BB%B8%E7%BC%8E%E8%B5%B7%E7%A8%8B%E6%97%A5%E6%9C%9F; https://zh.wikisource.org/wiki/%E6%B8%85%E5%AE%9E%E5%BD%95。“辛亥年”可能对应不同清代年份，缺少皇帝年号和奏者，无法可靠定位。</t>
         </is>
       </c>
     </row>
@@ -4887,7 +4887,7 @@
       </c>
       <c r="J97" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折或题本。关键词=动拨地丁银两委解甘省新疆经费银数目日期事、动拨地丁银、甘省新疆经费、拨解新疆经费、地丁银 新疆、乾隆 新疆 奏折。母项=乾隆朝宫中档奏折、军机处档折件、清代新疆档案史料、清代财政档案。候选站=https://www.google.com/search?q=%22%E5%8A%A8%E6%8B%A8%E5%9C%B0%E4%B8%81%E9%93%B6%E4%B8%A4%E5%A7%94%E8%A7%A3%E7%94%98%E7%9C%81%E6%96%B0%E7%96%86%E7%BB%8F%E8%B4%B9%22。题名格式明显接近清代档案目录或档案单件标题，需结合皇帝、年号、具奏人及档号检索；目前未找到可核验的具体全文页。</t>
         </is>
       </c>
     </row>
@@ -4933,7 +4933,7 @@
       </c>
       <c r="J98" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代新疆军事奏折，非独立书籍。关键词=靖逆将军 富宁安 穆森 吐鲁番、富宁安 奏调 穆森、都统穆森 驻防吐鲁番、靖逆将军奏折 吐鲁番、穆森 驻防 新疆。母项=《清实录·高宗纯皇帝实录》西北用兵及新疆建置相关卷、《平定准噶尔方略》、《钦定皇舆西域图志》、《清代新疆档案选辑》及军机处录副奏折。候选站=https://www.baidu.com/s?wd=%E9%9D%96%E9%80%86%E5%B0%86%E5%86%9B+%E5%AF%8C%E5%AE%81%E5%AE%89+%E7%A9%86%E6%A3%AE+%E5%90%90%E9%B2%81%E7%95%AA; https://zh.wikisource.org/wiki/%E5%B9%B3%E5%AE%9A%E5%87%86%E5%99%B6%E5%B0%94%E6%96%B9%E7%95%A5; https://zh.wikisource.org/wiki/%E9%92%A6%E5%AE%9A%E7%9A%87%E8%88%86%E8%A5%BF%E5%9F%9F%E5%9B%BE%E5%BF%97。未定位到该折的具体年号、日期、卷次或档号；母项页面仅用于后续关键词核查。</t>
         </is>
       </c>
     </row>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="J99" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代寄谕或上谕档案。关键词=寄谕乌什参赞大臣永贵、伊斯迈勒和卓、仍留伯克任、乌什 永贵 伯克、乾隆朝上谕档、新疆 和卓 伯克。母项=乾隆朝上谕档、乾隆朝军机处档案、清代新疆满文档案汉译编、清高宗实录。候选站=https://www.google.com/search?q=%22%E5%AF%84%E8%B0%95%E4%B9%8C%E4%BB%80%E5%8F%82%E8%B5%9E%E5%A4%A7%E8%87%A3%E6%B0%B8%E8%B4%B5%22。应优先按永贵、乌什、伊斯迈勒和卓及伯克任分别检索；未找到可直接核验的识典、维基文库或开放档案章节页。</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="J100" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折。关键词=伊犁将军晋昌、晋昌夹、察哈尔厄鲁特营、牧厂牲畜、奖赏官兵折、伊犁奏折 晋昌。母项=乾隆朝宫中档奏折、军机处档折件、清代新疆满文档案汉译编、伊犁将军衙门档案。候选站=https://www.google.com/search?q=%22%E4%BC%8A%E7%8A%81%E5%B0%86%E5%86%9B%E6%99%8B%E6%98%8C%22+%22%E5%AF%9F%E5%93%88%E5%B0%94%E5%8E%84%E9%B2%81%E7%89%B9%22。“夹查”可能是目录转录或 OCR 异文，建议同时检索“夹查”“查勘”“查看”；目前未找到具体全文页。</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="J101" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=青铜器铭文著录条目。关键词=叔钊父甗、叔钊父鬳、叔钊父铭文、殷周金文集成 3335、金文诅楚文、西周 甗。母项=《殷周金文集成》卷十五或器物分类对应卷、《金文编》、《商周青铜器铭文暨图像集成》、中国青铜器全集。候选站=https://www.google.com/search?q=%22%E5%8F%94%E9%92%8A%E7%88%B6%E7%94%97%22+3335; https://commons.wikimedia.org/w/index.php?search=%E5%8F%94%E9%92%8A%E7%88%B6%E7%94%97&amp;title=Special:MediaSearch&amp;type=image。3335应为金文著录编号，未能核实其对应的《殷周金文集成》具体卷页或开放铭文释文页。</t>
         </is>
       </c>
     </row>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="J102" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=文集中的书信、题跋或编者省题。关键词=又书、又書、又書 文集 書牘、又書 題跋、又書 答 與。母项=原作者别集中的书牍、尺牍或题跋卷（作者及集名待核）、选集或总集连续收录的同一作者书信组（待核）。候选站=。未找到可唯一定位的篇目页。“又书”常承接前一篇题名，必须取得作者、前一篇标题、收信人或正文首句后才能定位。检索时使用“作者＋又書”“文集名＋正文首句”，并检查前后篇；在母集未确定前，不能可靠指定卷次或生成维基文库、识典古籍章节URL。“林靖凯”仅是清单关联人，不能据此认定为作者。</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5163,7 @@
       </c>
       <c r="J103" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑刻或地方志收录记文。关键词=永和县重修庙学记、永和县 庙学记、永和县文庙、山西永和县碑刻、永和县志 庙学。母项=《永和县志》、山西地方志、山西金石记、山西碑刻文献。候选站=https://www.google.com/search?q=%22%E6%B0%B8%E5%92%8C%E5%8E%BF%E9%87%8D%E4%BF%AE%E5%BA%99%E5%AD%A6%E8%AE%B0%22。“永和县”可能指山西永和，也可能是历史地名；未找到可核验的碑刻全文、维基文库章节或识典古籍页面。</t>
         </is>
       </c>
     </row>
@@ -5209,7 +5209,7 @@
       </c>
       <c r="J104" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘简报或文物期刊论文。关键词=山西长治市南郊元代壁画墓、长治 南郊 元代壁画墓、长治元墓、山西元代墓葬壁画、长治 文物 元代壁画。母项=《文物》考古发掘简报、《考古》、《文物春秋》、山西省文物考古研究所发掘报告。候选站=https://www.google.com/search?q=%22%E5%B1%B1%E8%A5%BF%E9%95%BF%E6%B2%BB%E5%B8%82%E5%8D%97%E9%83%8A%E5%85%83%E4%BB%A3%E5%A3%81%E7%94%BB%E5%A2%93%22。题名体例像考古期刊发掘简报，需以作者、刊名、年份或墓葬编号定位；现代期刊全文是否开放不能据此确认。</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="J105" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代报刊消息或地方通讯。关键词=晋绥物产举行竞赛会、晋绥物产竞赛会、晋绥边区物产、物产竞赛会 晋绥、晋绥日报 物产。母项=《晋绥日报》、《抗战日报》晋绥版、晋绥边区政府公报、晋绥边区报刊合订本。候选站=https://www.google.com/search?q=%22%E6%99%8B%E7%BB%A5%E7%89%A9%E4%BA%A7%E4%B8%BE%E8%A1%8C%E7%AB%9E%E8%B5%9B%E4%BC%9A%22。很可能是报刊短消息而非独立出版物；缺少日期时难以在《晋绥日报》或相关报刊合订本中定位，未找到具体期号或开放全文页。</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="J106" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=篇名不明的现代散文、随笔或报刊文章。关键词=11月20日 林靖凯、十一月二十日 林靖凯、11月二十日 林靖凯、十一月二十号 林靖凯、11.20 林靖凯、林靖凯 11月20日。母项=林靖凯个人作品目录、文集或全集中的同名篇、作者发表作品所载报刊的当年11月及12月各期、地方文学刊物、纪念文集或作家资料汇编中的篇目索引、以日期为题的散文、日记。候选站=。未确认作者、文体、发表年份、刊物或版本。仅凭日期题名无法可靠定位具体全文；检索时应优先核对林靖凯作品目录及报刊篇目索引，再按年份查对应期号。</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="J108" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代报刊消息或军事新闻。关键词=晋军改编为三旅、晋军 三旅、山西军队改编三旅、晋军编为三旅、晋绥日报 晋军 三旅。母项=民国报刊、《晋绥日报》、《大公报》、《申报》、国民政府军事档案及战史资料。候选站=https://www.google.com/search?q=%22%E6%99%8B%E5%86%9B%E6%94%B9%E7%BC%96%E4%B8%BA%E4%B8%89%E6%97%85%22。题名过于简略，可能是报纸标题或档案目录标题；需先确定时间范围及“晋军”所指部队，未找到具体期刊年期或开放全文页。</t>
         </is>
       </c>
     </row>
@@ -5623,7 +5623,7 @@
       </c>
       <c r="J113" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑刻。关键词=邹县 峄山 仙人宫 圣旨碑、鄒縣 嶧山 仙人宮 聖旨碑、峄山仙人宫碑、邹县碑刻、峄山碑刻。母项=《山东金石志》、《山东通志》金石志、《邹县志》金石志或文物志、峄山碑刻调查资料。候选站=https://zh.wikisource.org/w/index.php?search=%E9%82%B9%E5%8E%BF+%E5%B3%84%E5%B1%B1+%E4%BB%99%E4%BA%BA%E5%AE%AB+%E5%9C%A3%E6%97%A8%E7%A2%91&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。题名末有括号残缺，可能是碑刻著录名而非独立文献；应重点查《山东金石志》卷次、邹县地方志及峄山碑刻录文。</t>
         </is>
       </c>
     </row>
@@ -5669,7 +5669,7 @@
       </c>
       <c r="J114" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地方报刊文章或寺庙创建碑记。关键词=临清 洪官营 女寺、洪官营 创建女寺、临清 女寺、伟举 女寺、臨清 洪官營 女寺。母项=临清县志、山东地方报刊、临清金石志、寺庙碑刻汇编。候选站=https://www.google.com/search?q=%22%E4%B8%B4%E6%B8%85%E6%B4%AA%E5%AE%98%E8%90%A5%22。未确认作者、刊物、年代或碑刻著录，不能定位具体全文页。</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
       </c>
       <c r="J116" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=族谱序文。关键词=益州 杨氏 世谱序、益州杨氏族谱、杨氏世谱序、蜀杨氏族谱、益州 楊氏 世譜序。母项=杨氏族谱、益州地方志、四川通志、全蜀艺文志、历代谱牒序跋汇编。候选站=https://www.google.com/search?q=%22%E7%9B%8A%E5%B7%9E%E6%9D%A8%E6%B0%8F%E4%B8%96%E8%B0%B1%E5%BA%8F%22。未能确认具体杨氏支派、作者和谱牒年代，不能给出具体卷页。</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="J117" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地图或绘画题名。关键词=清 潞河 督运图、潞河督运图、通州 漕运图、潞河 漕运 图、清代 潞河 督运。母项=清代舆图、漕运档案、通州地方志、河渠志、清宫旧藏地图目录。候选站=https://www.google.com/search?q=%22%E6%B8%85%E6%BD%9E%E6%B2%B3%E7%9D%A3%E8%BF%90%E5%9B%BE%22; https://commons.wikimedia.org/w/index.php?search=%E6%BD%9E%E6%B2%B3+%E6%BC%95%E8%BF%90%E5%9B%BE&amp;title=Special:MediaSearch&amp;type=image。未确认该题名是独立地图、图册中的单幅，或档案附件。</t>
         </is>
       </c>
     </row>
@@ -5853,7 +5853,7 @@
       </c>
       <c r="J118" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘报告或期刊论文。关键词=青衣江上游 汉文化 墓葬、青衣江 汉墓、雅安 汉文化墓葬、青衣江上游 汉墓、青衣江上游 漢文化 墓葬。母项=《四川文物》考古期刊、四川地区汉墓发掘报告、雅安地区文物志、中国考古学年鉴。候选站=https://www.google.com/search?q=%22%E9%9D%92%E8%A1%A3%E6%B1%9F%E4%B8%8A%E6%B8%B8%E6%B1%89%E6%96%87%E5%8C%96%E5%A2%93%E8%91%AC%22。可能是考古论文的简称或章节标题，尚未确认具体期刊年期。</t>
         </is>
       </c>
     </row>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="J119" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古简报或发掘报告章节。关键词=四川 会理 东咀遗址 陶器、会理县 东咀遗址、东咀遗址 出土陶器、会理 东咀 考古、四川會理縣 東咀遺址 陶器。母项=四川文物考古报告、《四川文物》、凉山州文物志、会理县志、中国考古学年鉴。候选站=https://www.google.com/search?q=%22%E4%BC%9A%E7%90%86%E5%8E%BF%E4%B8%9C%E5%92%80%E9%81%97%E5%9D%80%22。未确认“东咀”字形、发掘年份和刊物，不能定位具体页码。</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="J121" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑刻。关键词=发蒙寺碑、發蒙寺碑、发蒙寺 碑文、发蒙寺 金石、发蒙寺碑刻。母项=当地县志金石志、当地佛教寺院志、《中国文物地图集》相关省卷、地方碑刻与寺观资料。候选站=https://zh.wikisource.org/w/index.php?search=%E5%8F%91%E8%92%99%E5%AF%BA%E7%A2%91&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://commons.wikimedia.org/w/index.php?search=%E5%8F%91%E8%92%99%E5%AF%BA%E7%A2%91&amp;title=Special%3ASearch。缺少所在府县和年代，不能据题名确定具体寺院；应检索繁体“發蒙寺”、寺名异写及地方志的寺观、金石、艺文门。</t>
         </is>
       </c>
     </row>
@@ -6037,7 +6037,7 @@
       </c>
       <c r="J122" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代公文或档案文件。关键词=咨藏臣 已派员 勘测线路、咨藏臣 勘测线路、已派员勘测线路、川藏铁路 勘测、藏务档案 勘测线路。母项=清末民初藏务档案、川藏交通档案、西藏地方历史档案、交通部档案汇编、清季外交史料。候选站=https://www.google.com/search?q=%22%E5%B7%B2%E6%B4%BE%E5%91%98%E5%8B%98%E6%B5%8B%E7%BA%BF%E8%B7%AF%22。题名疑为档案摘要或目录拟题，缺少发文机关、年代、线路名称和档号。</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="J123" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代教育档案或公牍。关键词=王典章 禀报 筹办 高等小学预科、王典章 高等小学预科、筹办高等小学预科、高等小学预科 禀报、王典章 高等小學預科。母项=清末民初教育档案、地方教育行政档案、学务公牍汇编、各省教育会档案、地方志教育志。候选站=https://www.google.com/search?q=%22%E7%8E%8B%E5%85%B8%E7%AB%A0%22+%22%E9%AB%98%E7%AD%89%E5%B0%8F%E5%AD%A6%E9%A2%84%E7%A7%91%22。未确认王典章任职地区及档案年代，无法确定母项档案汇编。</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="J125" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代专题文章或民族地区报告章节。关键词=川康滇边区 汉 彝 藏 苗 纳西 相交相融、川康滇边区 民族关系、汉彝藏苗纳西 民族交融、川康滇边区民族史、川康滇邊區 漢彝藏苗納西。母项=川康滇边区民族调查资料、西南民族史研究论文集、四川省民族志、云南省志·民族志、康藏地区民族调查报告。候选站=https://www.google.com/search?q=%22%E5%B7%9D%E5%BA%B7%E6%BB%87%E8%BE%B9%E5%8C%BA%22+%22%E7%9B%B8%E4%BA%A4%E7%9B%B8%E8%9E%8D%22。题名用语较现代，可能是专题报告、网页文章或文集章节；未确认出版物和年份。</t>
         </is>
       </c>
     </row>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="J126" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近现代地方史研究条目或口述史文章。关键词=庄学本、庄学本 岭光电、庄学本 彝族土司、岭光电、岭光电 庄学本、庄学本 西康 彝族。母项=《庄学本少数民族摄影全集》、《庄学本摄影全集》、庄学本西南民族考察摄影档案、凉山彝族土司史料汇编、近代西南民族调查资料。候选站=https://zh.wikipedia.org/w/index.php?search=%E5%BA%84%E5%AD%A6%E6%9C%AC+%E5%B2%AD%E5%85%89%E7%94%B5; https://commons.wikimedia.org/w/index.php?search=%E5%BA%84%E5%AD%A6%E6%9C%AC&amp;title=Special:MediaSearch&amp;type=image。未找到与该完整题名对应的独立出版物、期刊篇名或可核验全文页；更可能是地方展览说明、摄影图录条目或二手研究中的小节。</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="J127" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代散文、旅行记或报刊文章。关键词=顺道回雷波 林靖凯、顺道回雷波、林靖凯 雷波、林靖凯 四川雷波、顺道 回雷波、回雷波 林靖凯。母项=林靖凯散文集、旅行散文集或作品集、四川地方文学选、凉山州文学选或雷波地方文献、地方报刊副刊及文学期刊中的旅行记、乡土散文栏目、雷波县志、地方文史资料或作者作品目。候选站=。未找到可核验的具体书名卷次、期刊年期或公开全文页。题名可能是散文篇名，也可能是地方报刊副刊标题；应结合作者活动年代、雷波地方文献和四川文学期刊目录检索。</t>
         </is>
       </c>
     </row>
@@ -6313,7 +6313,7 @@
       </c>
       <c r="J128" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=革命史口述史或地方文史资料篇目。关键词=天宝 红军、天宝 干部教育、天宝 现身说法、天宝 回忆红军、红军干部教育 天宝、少数民族干部 天宝。母项=《云南文史资料选辑》、《四川文史资料选辑》、《红军长征在云南》、《红军长征在四川》、地方革命老区文史资料汇编、少数民族干部回忆录。候选站=https://zh.wikipedia.org/w/index.php?search=%E5%A4%A9%E5%AE%9D+%E7%BA%A2%E5%86%9B+%E5%B9%B2%E9%83%A8%E6%95%99%E8%82%B2; https://www.google.com/search?q=%22%E5%A4%A9%E5%AE%9D%22+%22%E7%BA%A2%E5%86%9B%22+%22%E5%B9%B2%E9%83%A8%E6%95%99%E8%82%B2%22。“天宝”缺少姓氏和地区，无法据此定位具体作者及刊物卷期；题名可能是口述史栏目标题或地方文史资料中的文章标题。</t>
         </is>
       </c>
     </row>
@@ -6359,7 +6359,7 @@
       </c>
       <c r="J129" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地方经济史或民族贸易史研究条目。关键词=马边 汉彝贸易、马边 盐布、马边 白蜡虫、汉彝 易货交易、马边 白蜡、彝区 盐布贸易。母项=《马边县志》、《乐山地区志》、《四川省志·商业志》、《四川省志·民族志》、西南民族地区商业史料、凉山彝族社会历史调查。候选站=https://zh.wikipedia.org/w/index.php?search=%E9%A9%AC%E8%BE%B9+%E7%99%BD%E8%9C%A1%E8%99%AB+%E7%9B%90%E5%B8%83; https://www.google.com/search?q=%22%E9%A9%AC%E8%BE%B9%22+%22%E7%99%BD%E8%9C%A1%E8%99%AB%22+%22%E7%9B%90%E5%B8%83%22。未找到该完整题名对应的独立文献；内容更可能分散在《马边县志》物产、商业或民族关系章节，需按县志版本和章节继续核对。</t>
         </is>
       </c>
     </row>
@@ -6405,7 +6405,7 @@
       </c>
       <c r="J130" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地方经济史研究条目。关键词=民国 阿坝 汉人 经商、阿坝 汉藏贸易、阿坝 商业史、汉藏经济交流 民国、川西北 商人、松潘 茶马贸易。母项=《阿坝藏族羌族自治州志》、《松潘县志》、《理县志》、《汶川县志》、《四川省志·商业志》、《近代康区经济史研究》。候选站=https://zh.wikipedia.org/w/index.php?search=%E9%98%BF%E5%9D%9D+%E6%B1%89%E8%97%8F%E8%B4%B8%E6%98%93+%E6%B0%91%E5%9B%BD; https://www.google.com/search?q=%22%E9%98%BF%E5%9D%9D%22+%22%E6%B1%89%E8%97%8F%E7%BB%8F%E6%B5%8E%E4%BA%A4%E6%B5%81%22。未找到完整题名或可确认的期刊卷期；“汉人在阿坝经商”可能是地方志商业、交通或民族关系章节的概括性标题。</t>
         </is>
       </c>
     </row>
@@ -6451,7 +6451,7 @@
       </c>
       <c r="J131" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民族语言文字研究条目。关键词=大凉山 彝文、彝文字形 发音、彝汉语言接触、彝汉文字交融、凉山彝语 汉语、彝文音系。母项=《彝文典籍目录》、《彝汉大词典》、《凉山彝族自治州志》、《彝族语言文字》、《中国少数民族语言文字研究》、彝文古籍整理与研究资料。候选站=https://zh.wikipedia.org/w/index.php?search=%E5%BD%9D%E6%96%87+%E5%BD%9D%E8%AF%AD+%E5%A4%A7%E5%87%89%E5%B1%B1; https://www.google.com/search?q=%22%E5%A4%A7%E5%87%89%E5%B1%B1%22+%22%E5%BD%9D%E6%96%87%22+%22%E5%AD%97%E5%BD%A2%22。未找到该完整题名对应的独立书籍或可确认期刊篇目；可能是语言文字专题文章、展览说明或彝文古籍整理中的章节标题。</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="J132" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘报告或考古学论文。关键词=河套东部 东周墓葬、河套 东周 工具 武器、内蒙古东周墓葬、鄂尔多斯 东周墓、战国墓葬 工具 武器、河套考古。母项=《中国考古学·两周卷》、《内蒙古文物考古文集》、《鄂尔多斯式青铜器》、《内蒙古自治区文物考古研究所集刊》、《内蒙古文物考古》、河套地区墓葬发掘报告。候选站=https://zh.wikipedia.org/w/index.php?search=%E6%B2%B3%E5%A5%97+%E4%B8%9C%E5%91%A8+%E5%A2%93%E8%91%AC+%E5%B7%A5%E5%85%B7+%E6%AD%A6%E5%99%A8; https://www.google.com/search?q=%22%E6%B2%B3%E5%A5%97%E4%B8%9C%E9%83%A8%22+%22%E4%B8%9C%E5%91%A8%E5%A2%93%E8%91%AC%22。未找到完整题名或具体发掘报告卷页；题名形式更接近硕士论文或考古专题论文，需以“鄂尔多斯、包头、巴彦淖尔、战国墓葬”等地名扩展检索。</t>
         </is>
       </c>
     </row>
@@ -6543,7 +6543,7 @@
       </c>
       <c r="J133" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=墓志铭/墓志录文。关键词=尹祥墓志、尹祥墓誌、尹祥墓志铭、尹祥墓誌銘、尹祥 墓誌、尹祥 墓志。母项=历代墓志汇编、新中国出土墓志、地方金石志、陕西/河南/河北地方金石录（墓主时代与出土地待考）。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%B0%B9%E7%A5%A5%E5%A2%93%E5%BF%97&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=%E5%B0%B9%E7%A5%A5%E5%A2%93%E5%BF%97&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://www.shufaw.cn/search.php?keyword=%E5%B0%B9%E7%A5%A5%E5%A2%93%E5%BF%97。题名缺少年代、出土地和墓主身份，无法可靠定位到具体墓志汇编卷次；应先从原始清单或引用文献补出土地、时代、出土墓志集名称。</t>
         </is>
       </c>
     </row>
@@ -6589,7 +6589,7 @@
       </c>
       <c r="J134" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=墓志铭/墓志录文。关键词=郑宏墓志、鄭宏墓誌、郑宏墓志铭、鄭宏墓誌銘、郑宏 墓志、郑宏 墓志拓片。母项=历代墓志汇编、新中国出土墓志、地方金石志、墓志汇编续集。候选站=https://commons.wikimedia.org/w/index.php?search=%E9%84%AD%E5%AE%8F%E5%A2%93%E8%AA%8C&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=%E9%84%AD%E5%AE%8F%E5%A2%93%E8%AA%8C&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://www.shufaw.cn/search.php?keyword=%E9%84%AD%E5%AE%8F%E5%A2%93%E8%AA%8C。郑宏为常见姓名，缺乏时代、籍贯、出土地或撰书者信息，不能据题名锁定具体墓志。</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6635,7 @@
       </c>
       <c r="J135" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘报告或遗址调查简报。关键词=扎鲁特旗 哲北 辽代墓葬、哲北墓群、扎鲁特旗 辽墓、内蒙古 辽代墓葬、通辽 辽墓、辽代墓葬群 发掘。母项=《内蒙古文物考古文集》、《内蒙古文物考古》、《中国考古学·辽宋夏金元卷》、通辽市文物志、扎鲁特旗文物志、内蒙古自治区文物考古研究所考古发掘报告。候选站=https://zh.wikipedia.org/w/index.php?search=%E6%89%8E%E9%B2%81%E7%89%B9%E6%97%97+%E5%93%B2%E5%8C%97+%E8%BE%BD%E4%BB%A3%E5%A2%93%E8%91%AC; https://www.google.com/search?q=%22%E5%93%B2%E5%8C%97%22+%22%E8%BE%BD%E4%BB%A3%E5%A2%93%E8%91%AC%22。未找到可核验的具体考古报告页或期刊卷期；“哲北”可能为村名、墓地名称或发掘项目内部称谓，需结合通辽市、扎鲁特旗文物志核对。</t>
         </is>
       </c>
     </row>
@@ -6681,7 +6681,7 @@
       </c>
       <c r="J136" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代档案或军机处、兵部题本抄件。关键词=黑龙江将军 文绪、文绪 驿站、省属驿站 兵部、咨兵部 细册、黑龙江驿站 清代档案、清代黑龙江将军衙门档案。母项=《黑龙江将军衙门档案》、《黑龙江将军衙门档案选编》、《清代黑龙江历史档案选编》、《清实录·圣祖仁皇帝实录》、《清实录·世宗宪皇帝实录》、《黑龙江舆图》及清代驿站。候选站=https://zh.wikipedia.org/w/index.php?search=%E9%BB%91%E9%BE%99%E6%B1%9F%E5%B0%86%E5%86%9B+%E6%96%87%E7%BB%AA+%E9%A9%BF%E7%AB%99; https://www.google.com/search?q=%22%E6%96%87%E7%BB%AA%22+%22%E7%9C%81%E5%B1%9E%E9%A9%BF%E7%AB%99%22。未找到该档案的具体档号、日期、册页或公开全文；题名应为档案著录式标题，需从《黑龙江将军衙门档案》及清代兵部驿站档案的卷册索引入手。</t>
         </is>
       </c>
     </row>
@@ -6727,7 +6727,7 @@
       </c>
       <c r="J137" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代档案公文，可能为理藩院或盟旗档案子项。关键词=蒙荒案卷、办理札萨克图蒙荒案卷、札萨克图蒙荒、分移开局日期由、札萨克图、蒙荒。母项=清代理藩院档案、内蒙古历史档案、哲里木盟或昭乌达盟盟旗档案汇编、清代蒙旗垦务、蒙荒档案。候选站=https://commons.wikimedia.org/w/index.php?search=%E8%92%99%E8%8D%92%E6%A1%88%E5%8D%B7&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=%E8%92%99%E8%8D%92%E6%A1%88%E5%8D%B7&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。未找到可核验的具体卷册、档号或全文页。应以“札萨克图”“蒙荒”“开局日期”“分移”为字段，在理藩院档案和盟旗档案目录中查找。</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="J138" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代盟旗往来公文，可能为札、咨或移会。关键词=盟长敖汉旗额驸、绘制诸札萨克旗全图、翁牛特札萨克郡王、札萨克旗全图、敖汉旗额驸、诸札萨克旗全图。母项=清代理藩院档案、昭乌达盟盟长衙门档案、内蒙古盟旗档案汇编、清代蒙古舆图、旗界图档案。候选站=https://commons.wikimedia.org/w/index.php?search=%E6%9C%AD%E8%90%A8%E5%85%8B%E6%97%97%E5%85%A8%E5%9B%BE&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=%E7%BF%81%E7%89%9B%E7%89%B9%E6%9C%AD%E8%90%A8%E5%85%8B%E9%83%A1%E7%8E%8B&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。未找到具体档案页或档号。可按“敖汉旗额驸”“盟长”“翁牛特”“全图”“札萨克”组合检索昭乌达盟档案目录及清代蒙古舆图目录。</t>
         </is>
       </c>
     </row>
@@ -6819,7 +6819,7 @@
       </c>
       <c r="J139" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代盟旗土地纠纷呈文。关键词=旗札萨克王、台吉希日拉、台田地纠纷、盟摄政王爷、希日拉、田地纠纷。母项=清代理藩院蒙古旗地案件档案、盟旗衙门土地纠纷档案、内蒙古历史档案汇编、清代蒙古王公文书。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%B8%8C%E6%97%A5%E6%8B%89%E7%94%B0%E5%9C%B0%E7%BA%A0%E7%BA%B7&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=%E7%90%86%E8%97%A9%E9%99%A2%20%E7%94%B0%E5%9C%B0%20%E8%92%99%E5%8F%A4&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。未找到具体卷次、档号或全文。人名“希日拉”可能有“喜日拉、希日勒、席日拉”等异写，应结合满文或蒙古文目录复核。</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6865,7 @@
       </c>
       <c r="J140" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代报刊文章或新闻通讯，题名可能不完整。关键词=切切实实为蒙地群众办好事、蒙地群众办好事、记我党、蒙地、群众工作。母项=内蒙古日报、绥远日报、人民日报、晋察冀日报或华北解放区报刊、内蒙古地方党史资料。候选站=https://zh.wikisource.org/w/index.php?search=%E5%88%87%E5%88%87%E5%AE%9E%E5%AE%9E%E4%B8%BA%E8%92%99%E5%9C%B0%E7%BE%A4%E4%BC%97%E5%8A%9E%E5%A5%BD%E4%BA%8B&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。未找到可靠的刊名、日期、版次或具体页面。题名末尾“记我党”可能是OCR截断，应以“蒙地群众”“办好事”检索1940—1950年代内蒙古及绥远报刊目录。</t>
         </is>
       </c>
     </row>
@@ -6911,7 +6911,7 @@
       </c>
       <c r="J141" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=抗日战争时期新闻或报刊短讯。关键词=延安准备召开人民代表会、延安召开人民代表会议、人民代表会、延安人民代表会议、陕甘宁边区人民代表会议。母项=解放日报（延安）、新华日报、陕甘宁边区政府公报、陕甘宁边区参议会史料、抗日战争时期延安报刊。候选站=https://zh.wikisource.org/w/index.php?search=%E5%BB%B6%E5%AE%89%20%E4%BA%BA%E6%B0%91%E4%BB%A3%E8%A1%A8%E4%BC%9A&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。未找到具体报刊日期、版次或全文页。应重点核查《解放日报》1940年代相关月份及“陕甘宁边区参议会”“人民代表会议”主题索引。</t>
         </is>
       </c>
     </row>
@@ -6957,7 +6957,7 @@
       </c>
       <c r="J142" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=1945年报刊电讯或政治文电。关键词=1945年11月21日、绥境蒙政会、通电、制止军事冲突、绥境蒙政会通电、蒙政会。母项=绥远日报、解放日报、新华日报、晋绥边区报刊、1945年内蒙古自治运动史料。候选站=https://zh.wikisource.org/w/index.php?search=%E7%BB%A5%E5%A2%83%E8%92%99%E6%94%BF%E4%BC%9A%20%E9%80%9A%E7%94%B5&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://commons.wikimedia.org/w/index.php?search=%E7%BB%A5%E5%A2%83%E8%92%99%E6%94%BF%E4%BC%9A&amp;title=Special:MediaSearch&amp;type=image。未找到该日期对应的具体报刊版面或档案影印页。应同时检索“绥境蒙政会”“绥远蒙政会”“蒙政会等”“军事冲突”等异名。</t>
         </is>
       </c>
     </row>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="J143" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=1948年报刊灾情短讯。关键词=1948年4月25日、黄河春讯、水淹良田、包头县二百顷地不能耕、包头县、黄河水灾。母项=绥远日报、晋绥日报、人民日报、解放日报、1948年黄河水灾报刊资料。候选站=https://zh.wikisource.org/w/index.php?search=%E9%BB%84%E6%B2%B3%E6%98%A5%E8%AE%AF%20%E5%8C%85%E5%A4%B4%E5%8E%BF&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://commons.wikimedia.org/w/index.php?search=%E5%8C%85%E5%A4%B4%E5%8E%BF%20%E9%BB%84%E6%B2%B3%20%E6%B0%B4%E7%81%BE&amp;title=Special:MediaSearch&amp;type=image。未找到具体刊名、版次或可核验全文。题名中的“春讯”也可能是“春汛”或OCR误读，应检索“黄河春汛”“包头县”“二百顷”“不能耕”。</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="J144" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代报刊政论、建议或铁路计划文。关键词=建筑边防铁路之提议、建筑边防铁路、边防铁路提议、边防铁路、铁路与边防。母项=清末民初铁路史料、《东方杂志》、《申报》、《铁路官报》、近代中国边防与铁路论著。候选站=https://zh.wikisource.org/w/index.php?search=%E5%BB%BA%E7%AD%91%E8%BE%B9%E9%98%B2%E9%93%81%E8%B7%AF&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://commons.wikimedia.org/w/index.php?search=%E8%BE%B9%E9%98%B2%E9%93%81%E8%B7%AF&amp;title=Special:MediaSearch&amp;type=image。未找到作者、刊名、年月和具体页面。应按“边防铁路”“塞外铁路”“西北铁路”“蒙疆铁路”等近代异名检索《东方杂志》及清末民初报刊目录；若为现代整理本，只能核查书目与馆藏。</t>
         </is>
       </c>
     </row>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="J145" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=政治宣传文章或报告，可能为报刊、会议材料或文集子项。关键词=巩固民族团结、巩固民族團結、民族团结、民族團結、林靖凯、林靖凱。母项=中华人民共和国成立初期民族政策文件汇编、民族工作文献选编、地方党政报刊或民族事务档案汇编。候选站=https://www.google.com/search?q=%22%E5%B7%A9%E5%9B%BA%E6%B0%91%E6%97%8F%E5%9B%A2%E7%BB%93%22+%E6%9E%97%E9%9D%96%E5%87%AF; https://commons.wikimedia.org/w/index.php?search=%E5%B7%A9%E5%9B%BA%E6%B0%91%E6%97%8F%E5%9B%A2%E7%BB%93&amp;title=Special%3AMediaSearch&amp;type=image。题名过于通用，缺少年份、发表机关和载体，暂不能定位为独立著作。</t>
         </is>
       </c>
     </row>
@@ -7141,7 +7141,7 @@
       </c>
       <c r="J146" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=1947年报刊标题或救灾电文，可能为绥远省伊克昭盟灾情档案子项。关键词=伊盟灾民、伊克昭盟灾民、灾民亟待救活、需粮卅万石、需粮三十万石、1947年9月30日。母项=1947年国民政府或绥远省政府救灾档案、绥远日报、中央日报及地方报刊1947年9月至10月号、近代中国灾荒史料汇编。候选站=https://www.google.com/search?q=%221947%E5%B9%B49%E6%9C%8830%E6%97%A5%22+%22%E4%BC%8A%E7%9B%9F%E7%81%BE%E6%B0%91%22; https://commons.wikimedia.org/w/index.php?search=%E4%BC%8A%E7%9B%9F%E7%81%BE%E6%B0%91&amp;title=Special%3AMediaSearch&amp;type=image。明显是新闻标题或电文标题，不宜按独立书籍检索；应重点查1947年9月至10月报刊及绥远救灾档案。</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7233,7 @@
       </c>
       <c r="J148" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=文物图录或考古报告中的器物条目。关键词=大理国铜鎏金铜函、大理国鎏金铜函、大理国铜函、铜鎏金铜函、大理国文物、大理崇圣寺三塔。母项=大理国文物图录、云南省博物馆藏大理国文物、崇圣寺三塔出土文物考古报告。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%A4%A7%E7%90%86%E5%9B%BD+%E9%8E%8F%E9%87%91%E9%93%9C%E5%87%BD&amp;title=Special%3AMediaSearch&amp;type=image; https://www.google.com/search?q=%22%E5%A4%A7%E7%90%86%E5%9B%BD%E9%8E%8F%E9%87%91%E9%93%9C%E5%87%BD%22。未确认该名称对应的独立出版物或公开全文页；应以馆藏编号、出土地和图录页码继续核查。</t>
         </is>
       </c>
     </row>
@@ -7279,7 +7279,7 @@
       </c>
       <c r="J149" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民族问题研究文章、报告或内部资料。关键词=云南少数民族问题、雲南少數民族問題、云南民族问题、云南民族工作、林靖凯、林靖凱。母项=云南民族工作文献汇编、中华人民共和国民族政策文献、云南地方党政报刊及民族事务档案。候选站=https://www.google.com/search?q=%22%E4%BA%91%E5%8D%97%E5%B0%91%E6%95%B0%E6%B0%91%E6%97%8F%E9%97%AE%E9%A2%98%22+%E6%9E%97%E9%9D%96%E5%87%AF; https://commons.wikimedia.org/w/index.php?search=%E4%BA%91%E5%8D%97%E5%B0%91%E6%95%B0%E6%B0%91%E6%97%8F%E9%97%AE%E9%A2%98&amp;title=Special%3AMediaSearch&amp;type=image。题名属于高度概括性的专题名，尚无年份、作者职务、出版机关或载体信息。</t>
         </is>
       </c>
     </row>
@@ -7325,7 +7325,7 @@
       </c>
       <c r="J150" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=地方志稿/方志母项。关键词=广南县志稿、廣南縣志稿、广南州志稿、廣南州志稿、广南县志、廣南縣志。母项=《广南州志》、《广南县志》、《广南府志》、云南省地方志联合目录、云南旧方志目录。候选站=https://zh.wikisource.org/w/index.php?search=%E5%BB%A3%E5%8D%97%E7%B8%A3%E5%BF%97&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://commons.wikimedia.org/w/index.php?search=%E5%BB%A3%E5%8D%97%E7%B8%A3%E5%BF%97&amp;title=Special:MediaSearch&amp;type=document; https://www.ancientbooks.cn/。该题名很可能是方志稿本、目录著录或现代整理中的非独立条目，应同时查《广南州志》《广南府志》及云南旧方志目录，确认版本、纂修年代和卷次。</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7371,7 @@
       </c>
       <c r="J151" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代诗歌、散文、歌词或报刊文章。关键词=献上一片心 林靖凯、献上一片心、献上一片心 林靖凯 诗、献上一片心 林靖凯 散文、林靖凯 一片心、献上一片心 期刊。母项=林靖凯诗集、散文集或作品选中的同名篇、地方文学选、青年文学作品选或纪念文集、报刊副刊、诗歌专刊及文学期刊目录、主题性诗歌、歌曲或文艺作品汇编。候选站=。题名过于常见，未确认作者、文体、发表年份及载体。未找到可核验的具体章节、卷次、期刊年期或公开全文页；需先从林靖凯作品目录、作者档案及报刊篇目数据库确认出处。</t>
         </is>
       </c>
     </row>
@@ -7509,7 +7509,7 @@
       </c>
       <c r="J154" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=方志。关键词=康熙 青浦县志、康熙 青浦 县志、康熙《青浦县志》、青浦县志 康熙刻本、青浦縣志 康熙。母项=《青浦县志》历代版本、《上海府县志辑》、《中国地方志集成·上海府县志辑》、《上海通志》方志提要。候选站=https://zh.wikisource.org/w/index.php?search=%E5%BA%B7%E7%86%99%E9%9D%92%E6%B5%A6%E5%8E%BF%E5%BF%97&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://www.shidian古籍.example/search?q=%E5%BA%B7%E7%86%99%E9%9D%92%E6%B5%A6%E5%8E%BF%E5%BF%97。应按康熙年间修纂或刻印年份继续区分版本，并查《青浦县志》卷一至卷末的艺文、古迹和金石门。</t>
         </is>
       </c>
     </row>
@@ -7555,7 +7555,7 @@
       </c>
       <c r="J155" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=摩崖石刻释文或地方文物条目。关键词=通贵州至乌撒驿道、通貴州至烏撒驛道、乌撒驿道、烏撒驛道、纪功摩崖、紀功摩崖。母项=贵州省志·文物志、毕节地区志或威宁、赫章、纳雍地方志、贵州历代碑刻集、西南交通史或驿道石刻资料。候选站=https://www.google.com/search?q=%22%E9%80%9A%E8%B4%B5%E5%B7%9E%E8%87%B3%E4%B9%8C%E6%92%92%E9%A9%BF%E9%81%93%22; https://commons.wikimedia.org/w/index.php?search=%E4%B9%8C%E6%92%92%E9%A9%BF%E9%81%93&amp;title=Special%3AMediaSearch&amp;type=image。应先确定摩崖所在县和年代，再查相应县志、文物普查资料及碑刻录文。</t>
         </is>
       </c>
     </row>
@@ -7601,7 +7601,7 @@
       </c>
       <c r="J156" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=期刊公文或档案汇编中的单件文件。关键词=贵州盐务月刊、貴州鹽務月刊、省政府训令、四川盐运署、招商负责承销办法、盐务月刊训令。母项=《贵州盐务月刊》相关卷期、贵州盐务局档案、四川盐运使署或盐运署公文汇编、民国盐务史料汇编。候选站=https://www.google.com/search?q=%22%E8%B4%B5%E5%B7%9E%E7%9B%90%E5%8A%A1%E6%9C%88%E5%88%8A%22+%22%E5%9B%9B%E5%B7%9D%E7%9B%90%E8%BF%90%E7%BD%B2%22; https://www.google.com/search?q=%22%E6%8B%9B%E5%95%86%E8%B4%9F%E8%B4%A3%E6%89%BF%E9%94%80%E5%8A%9E%E6%B3%95%22。不是独立书籍，应查《贵州盐务月刊》的目录、期号和公文栏目；现未确认具体年月期。</t>
         </is>
       </c>
     </row>
@@ -7647,7 +7647,7 @@
       </c>
       <c r="J157" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘报告或文物图录中的器物条目。关键词=唐平坝马场、平坝马场、八弧花鸟纹铜镜、八弧花鸟紋銅鏡、唐代花鸟纹铜镜、贵州唐墓铜镜。母项=贵州省文物考古研究所考古发掘报告、贵州省志·文物志、安顺市志或平坝县志、中国出土铜镜全集。候选站=https://www.google.com/search?q=%22%E5%B9%B3%E5%9D%9D%E9%A9%AC%E5%9C%BA%22+%22%E5%85%AB%E5%BC%A7%E8%8A%B1%E9%B8%9F%E7%BA%B9%E9%93%9C%E9%95%9C%22; https://commons.wikimedia.org/w/index.php?search=%E5%85%AB%E5%BC%A7%E8%8A%B1%E9%B8%9F%E7%BA%B9%E9%93%9C%E9%95%9C&amp;title=Special%3AMediaSearch&amp;type=image。名称很可能是文物图录的单项标题，需以藏品编号、墓葬名称或发掘年份定位。</t>
         </is>
       </c>
     </row>
@@ -7693,7 +7693,7 @@
       </c>
       <c r="J158" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑刻。关键词=剑河县 太拥 清江府 示碑、道光二十五年 清江府 示碑、太拥碑、劍河縣 太擁 清江府 示碑、贵州剑河碑刻。母项=《剑河县志》、《贵州省志·文物志》、《贵州金石志》或贵州碑刻资料、剑河县文物普查资料。候选站=https://zh.wikisource.org/w/index.php?search=%E5%89%91%E6%B2%B3%E5%8E%BF+%E5%A4%AA%E6%8B%A5+%E6%B8%85%E6%B1%9F%E5%BA%9C+%E7%A4%BA%E7%A2%91&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。“清江府”可能是碑文中的行政称谓或转录误读；应同时检索“清江厅”“清江府示”“太拥村/太拥镇”及道光二十五年。</t>
         </is>
       </c>
     </row>
@@ -7796,7 +7796,7 @@
       </c>
       <c r="J161" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊。关键词=昆仑报、昆仑報、昆仑报 姜博文、昆仑报 新疆、昆仑报 报纸。母项=民国及近代报刊目录、新疆地方报刊汇编、报纸合订本或报刊影印本。候选站=https://commons.wikimedia.org/w/index.php?search=%E6%98%86%E4%BB%91%E6%8A%A5&amp;title=Special:MediaSearch&amp;type=image; https://www.google.com/search?q=%22%E6%98%86%E4%BB%91%E6%8A%A5%22+%E6%8A%A5%E5%88%8A。未找到可核验的具体年、期或连续出版物全文页；应进一步按出版地、主办机构和年代检索报刊目录及合订本。</t>
         </is>
       </c>
     </row>
@@ -8132,7 +8132,7 @@
       </c>
       <c r="J168" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘报告或墓志考古资料。关键词=固原西郊雷祖庙村北魏墓、固原雷祖庙村北魏墓、固原西郊北魏墓、宁夏固原北魏墓葬、雷祖庙村墓志、北魏墓志 固原。母项=《宁夏固原北魏墓地》、《固原历史文物》、《文物》考古发掘报告及墓志资料。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%9B%BA%E5%8E%9F%E8%A5%BF%E9%83%8A%E9%9B%B7%E7%A5%96%E5%BA%99%E6%9D%91%E5%8C%97%E9%AD%8F%E5%A2%93&amp;title=Special:MediaSearch&amp;type=image。未找到可核验的考古报告题名、刊物年期、墓志编号或具体开放页面。</t>
         </is>
       </c>
     </row>
@@ -8275,7 +8275,7 @@
       </c>
       <c r="J171" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=文章/报刊栏目或短篇作品。关键词=商业家族、商業家族、商业家族 姜博文、商业家族 报刊、商业家族 文章。母项=近代报刊文学或社会评论栏目、姜博文作品集或文集、商业史、家族史类报刊合订本。候选站=https://www.google.com/search?q=%22%E5%95%86%E4%B8%9A%E5%AE%B6%E6%97%8F%22+%E5%A7%9C%E5%8D%9A%E6%96%87。题名过于通用，未找到可确认的卷期、文集卷次或具体全文页。</t>
         </is>
       </c>
     </row>
@@ -8321,7 +8321,7 @@
       </c>
       <c r="J172" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近现代革命档案或工作报告。关键词=瑶山工作区开展工作、瑶山工作区、瑶山开展工作、瑶山革命根据地、工作区开展工作 报告、瑶山档案。母项=地方革命历史档案汇编、中国共产党革命根据地档案资料、瑶山地方党史资料。候选站=。题名过于概括，缺少年代、地区、机构、作者或档案汇编信息，未找到可核验的具体卷册、期刊年期或开放全文页。</t>
         </is>
       </c>
     </row>
@@ -8560,7 +8560,7 @@
       </c>
       <c r="J177" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民国选举档案文书。关键词=国民大会代表立法院立法委员安徽省选举事务所、安徽省选举事务所稿、国民大会代表选举安徽、立法院立法委员安徽选举、发文字、民国安徽选举档案。母项=《国民大会代表选举档案》、《中华民国史档案资料汇编》、民国安徽省政府档案及选举档案。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%AE%89%E5%BE%BD%E7%9C%81%E9%80%89%E4%B8%BE%E4%BA%8B%E5%8A%A1%E6%89%80&amp;title=Special:MediaSearch&amp;type=image。应为档案母项或案卷标题，未找到具体年份、案卷号、收发文号或开放影像页。</t>
         </is>
       </c>
     </row>
@@ -8893,7 +8893,7 @@
       </c>
       <c r="J184" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=石窟题记、文物图录或考古论文中的子项。关键词=张掖 金塔寺 石窟 西夏文 题记、金塔寺石窟 西夏文字、肃南 金塔寺 西夏题记、甘肃石窟 西夏文题刻、張掖 金塔寺 石窟 西夏文 題記、金塔寺石窟 西夏文 題刻。母项=《中国石窟：河西石窟》相关卷、《甘肃石窟寺》、《中国文物地图集·甘肃分册》、张掖、肃南地区石窟考古调查报告、西夏文石刻或西夏文献图录。候选站=。更可能是石窟调查报告、图录或论文中的题记条目，不能按独立书名检索。应以金塔寺、肃南、马蹄寺石窟群及西夏文题刻等母项追查，并核对题记所在洞窟、编号和释文。</t>
         </is>
       </c>
     </row>
@@ -8998,7 +8998,7 @@
       </c>
       <c r="J186" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折。关键词=督理宁夏、查汉托护工务通智、新渠、宝丰、设训导、取进童生。母项=清代宫中档奏折、军机处档奏折、宁夏地方奏折汇编、清代教育史料汇编。候选站=。应按奏折档案的题名、具奏官和事由检索；“通智”可能是题名转录或识读异文，需同时检索“通志”“通治”等字形。未找到可核验的具体全文页。</t>
         </is>
       </c>
     </row>
@@ -9044,7 +9044,7 @@
       </c>
       <c r="J187" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民国档案中的单件报告。关键词=保甲督导委员 李汉仪 海原县 李旺堡、李汉仪 海原 李旺堡 报告、海原县 保甲 督导 报告、李旺堡 保甲、民国 海原县 保甲档案、保甲督导委员 李漢儀 海原縣 李旺堡。母项=民国宁夏省政府档案、宁夏省保安处或民政厅保甲档案、《宁夏档案史料》相关辑刊、海原县地方档案汇编、西北地区保甲制度档案汇编。候选站=。题名格式明显接近档案馆著录题名，可能属于全宗中的单件公文。检索时应加入时间、发文机关、档号及李旺堡所属区乡信息；目前未核得具体卷册或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -9140,7 +9140,7 @@
       </c>
       <c r="J189" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=古籍丛编中的单种游记。关键词=清代蒙古游记选辑 三十四种 巴林纪程、巴林纪程、巴林纪行、巴林游记 清代、蒙古游记 巴林、清代蒙古游记選輯 巴林紀程。母项=《清代蒙古游记选辑三十四种》上册、清代蒙古史料丛刊中的蒙古游记、蒙古游牧记、蒙古纪程类丛书、清代西北舆地游记汇编。候选站=。原题括号不完整，可能应还原为丛编书名加单种题名。应查上册目录、影印本目录及编者说明，重点核对作者、成书年代、巴林部或巴林旗的异写。目前未找到可核验的具体全文页。</t>
         </is>
       </c>
     </row>
@@ -9186,7 +9186,7 @@
       </c>
       <c r="J190" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代或民国边疆档案单件。关键词=兴东道 毕拉尔路 协领 庆山、毕拉尔路 收抚牲丁 设学堂 劝垦、庆山 协领 呈、协佐办公 截饷 毕路、毕拉尔路档案、興東道 畢拉爾路 協領 慶山 收撫牲丁。母项=黑龙江将军衙门档案、呼伦贝尔副都统或地方官档案、《清代东北边疆满文档案选编》、《清代黑龙江历史档案选编》、清代边疆民族地区教育、垦务与旗务档案汇编。候选站=。题名为档案著录语，需按发文机关、官职、人物及事务关键词定位全宗卷册。‘毕拉尔路’可能有毕拉尔、毕拉尔路、毕拉尔部等异写，‘牲丁’也应检索为牲畜丁、牧丁等变体。未找到具体公开页。</t>
         </is>
       </c>
     </row>
@@ -9281,7 +9281,7 @@
       </c>
       <c r="J192" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代报刊短讯或教育行政文件标题。关键词=教部鼓励学生服务边疆、教育部 鼓励学生 服务边疆、学生 服务边地 教育部、服务边疆 学生 报刊、教部 鼓勵學生 服務邊疆。母项=民国中央报刊、《申报》、《中央日报》、《教育杂志》、教育部公报及民国教育行政档案。候选站=。短题名很可能是报刊消息标题，需以‘教部’、‘学生服务边地’、‘边疆教育’等词组合检索，并按民国年份和报刊版次定位。未核得具体报纸日期、版面或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -9675,7 +9675,7 @@
       </c>
       <c r="J199" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑记。关键词=重建蘖谷王公祠碑记、蘖谷王公祠、蘖谷、王公祠、重修王公祠、重建王公祠。母项=地方志艺文志、地方志金石志、祠庙碑刻汇编、地方碑刻录文集。候选站=。“蘖谷”地名或祠主身份尚未确定，不能据题名判断所属府县。应先以碑额、撰书者、立碑年代和祠主姓名回查地方志金石志。未找到可核验的具体录文或图像页。</t>
         </is>
       </c>
     </row>
@@ -9953,7 +9953,7 @@
       </c>
       <c r="J205" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代刑科题本或会审案件档案。关键词=安徽亳州 回民 马四 贾克明、马四 毙妹夫 贾克明 绞监候、伊母被殴伤 亳州、会审 安徽亳州 回民 刑案、清代刑科题本 亳州 马四、安徽亳州 回民 馬四 賈克明 絞監候。母项=清代刑科题本、《刑科题本·婚姻家庭类》或命案类、清代中央司法档案汇编、安徽省地方司法档案汇编、清代回民案件档案选编。候选站=。题名符合刑科题本著录格式，‘题为’可能来自档案数据库的摘要字段。应按案犯、被害人、籍贯、拟刑及年份检索，并核对‘妹夫’与‘贾克明’关系。未找到具体卷次或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -9999,7 +9999,7 @@
       </c>
       <c r="J206" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代军事或地方行政档案集合。关键词=贵池团管区司令部、贵池 团管区 公文、贵池团管区司令部档案、安徽贵池 团管区、团管区司令部 贵池、貴池團管區司令部 公文。母项=安徽省档案馆民国军事档案、池州市或贵池区地方档案馆馆藏、国民政府军事委员会及安徽省政府档案、民国安徽地方军事档案汇编、贵池地方史料汇编。候选站=。题名过于概括，‘相关公文’可能是数据库对一组档案的集合标题，不是单件文书。需补充年代、文种、收发文机关、档号或公文主题后检索；目前未找到可核验的具体卷册或全文页。</t>
         </is>
       </c>
     </row>
@@ -10045,7 +10045,7 @@
       </c>
       <c r="J207" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=日期标识的报刊文章、日记、档案或会议记录。关键词=1926年4月21日、一九二六年四月二十一日、民国十五年四月二十一日、民国十五年四月廿一日、1926-04-21 报刊、一九二六年四月二十一日 档案。母项=1926年4月21日出版的民国报刊、民国十五年政府公报、民国时期日记、书信及会议记录汇编、北洋政府或国民革命时期档案汇编、地方志与地方档案中的日期条目。候选站=。仅有日期，无法判定文献类型、作者或母项。应先结合姜博文清单相邻条目的主题和来源，确定是报刊日期、档案成文日期、日记条目还是会议记录；在缺乏上下文前未找到可核验具体页面。</t>
         </is>
       </c>
     </row>
@@ -10137,7 +10137,7 @@
       </c>
       <c r="J209" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=革命文献档案汇编中的公文条目。关键词=中国工农红军第一方面军总政治部、红一方面军总政治部 公文、第一方面军政治部 文件、中央革命根据地 公文、工农红军 总政治部 电报 函。母项=《中央革命根据地史料选编》、《中央革命根据地史料》、《中国工农红军历史资料丛书》相关卷、中央革命根据地档案汇编中第一方面军总政治部档案。候选站=https://commons.wikimedia.org/w/index.php?search=%E4%B8%AD%E5%9B%BD%E5%B7%A5%E5%86%9C%E7%BA%A2%E5%86%9B%E7%AC%AC%E4%B8%80%E6%96%B9%E9%9D%A2%E5%86%9B%E6%80%BB%E6%94%BF%E9%83%A8&amp;title=Special:MediaSearch&amp;type=image。题名更像档案汇编中的概括性条目，需按总政治部、日期、收文机关或文种回溯，未找到可核验的具体卷页或全文。</t>
         </is>
       </c>
     </row>
@@ -10183,7 +10183,7 @@
       </c>
       <c r="J210" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地方民族史或地方文献中的专题文章。关键词=凤台县 回族、凤台回族史、凤台县民族志、凤台县志 回族、凤台县 回民。母项=《凤台县志》、《凤台县志》民族、人口或社会风俗卷、《安徽省志·民族宗教志》、地方民族问题调查资料汇编。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%87%A4%E5%8F%B0%E5%8E%BF%E5%9B%9E%E6%97%8F&amp;title=Special:MediaSearch&amp;type=image。未找到以此题名独立刊行或公开全文的具体记录，优先应在《凤台县志》民族、宗教、人口和风俗章节中定位。</t>
         </is>
       </c>
     </row>
@@ -10371,7 +10371,7 @@
       </c>
       <c r="J214" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=舆图或档案地图。关键词=古北口 科尔沁 图、古北口科尔沁舆图、科尔沁地图 古北口、古北口 地图 清代、科尔沁部 舆图。母项=清代内府舆图档案、《皇舆全览图》及相关舆图、清代蒙古地区舆图汇编、古北口关隘与蒙古地区档案图册。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%8F%A4%E5%8C%97%E5%8F%A3%20%E7%A7%91%E5%B0%94%E6%B2%81&amp;title=Special:MediaSearch&amp;type=image。题名可能是档案目录中的地图短题名，需结合地图编号、绘制年代、幅面和收藏机构检索，未找到具体图页。</t>
         </is>
       </c>
     </row>
@@ -10465,7 +10465,7 @@
       </c>
       <c r="J216" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=游记/报刊文章。关键词=京尘纪游、京塵紀遊、京尘纪游 姜博文、京尘纪游 北京 游记、京尘纪游 纪行。母项=近代游记文集、报刊副刊或旅行栏目、姜博文文集、作品集。候选站=https://www.google.com/search?q=%22%E4%BA%AC%E5%B0%98%E7%BA%AA%E6%B8%B8%22; https://zh.wikisource.org/w/index.php?search=%E4%BA%AC%E5%B0%98%E7%B4%80%E9%81%8A&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2。未找到与姜博文对应的具体书目、卷次或章节页。</t>
         </is>
       </c>
     </row>
@@ -10511,7 +10511,7 @@
       </c>
       <c r="J217" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊新闻或城市建设档案中的句式标题。关键词=多处开辟 公园、供大众游览娱乐 公园、开辟公园 游览娱乐、城市公园 大众游览、公园建设 报刊。母项=地方政府施政报告、城市建设档案汇编、民国或中华人民共和国初期地方报刊、园林建设和城市规划资料汇编。候选站=https://commons.wikimedia.org/w/index.php?search=%E4%BE%9B%E5%A4%A7%E4%BC%97%E6%B8%B8%E8%A7%88%E5%A8%B1%E4%B9%90%E5%85%AC%E5%9B%AD&amp;title=Special:MediaSearch&amp;type=image。该条目像文章或档案中的语句摘录，不像独立文献题名；缺少城市、年代和报刊信息，未找到具体页。</t>
         </is>
       </c>
     </row>
@@ -10604,7 +10604,7 @@
       </c>
       <c r="J219" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=文物考释/图录条目。关键词=镶松石金器、鑲松石金器、镶嵌松石金器、镶松石金器 姜博文、松石 金器 考古。母项=考古发掘报告、博物馆藏品图录、文物展览图录或文物考释专栏。候选站=https://commons.wikimedia.org/w/index.php?search=%E9%95%B6%E6%9D%BE%E7%9F%B3%E9%87%91%E5%99%A8&amp;title=Special:MediaSearch&amp;type=image; https://www.google.com/search?q=%22%E9%95%B6%E6%9D%BE%E7%9F%B3%E9%87%91%E5%99%A8%22。更像文物图录中的条目或图片说明，未找到可确认的图录名称、页码及全文页。</t>
         </is>
       </c>
     </row>
@@ -10987,7 +10987,7 @@
       </c>
       <c r="J227" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代档案公文。关键词=八旗学堂、学堂监督、海成 典史、蒙养小学堂、初等小学堂 禀、八旗教育档案。母项=清代教育档案汇编、八旗都统衙门档案、地方旗务档案、清末新政学堂档案汇编。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%85%AB%E6%97%97%E5%AD%A6%E5%A0%82%20%E8%92%99%E5%85%BB%20%E5%88%9D%E7%AD%89%E5%B0%8F%E5%AD%A6%E5%A0%82&amp;title=Special:MediaSearch&amp;type=image。题名保留了档案目录的批、禀关系，需以海成任职地点、旗籍和档案全宗继续定位，未找到具体卷页。</t>
         </is>
       </c>
     </row>
@@ -11079,7 +11079,7 @@
       </c>
       <c r="J229" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=诗歌/报刊诗作。关键词=忧时 外一首、憂時 外一首、忧时 姜博文、憂時 姜博文、忧时 诗。母项=近代报刊副刊、诗歌合集或诗集、姜博文诗稿、作品集。候选站=https://zh.wikisource.org/w/index.php?search=%E6%86%82%E6%99%82&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://www.google.com/search?q=%22%E5%BF%A7%E6%97%B6%22+%22%E5%A4%96%E4%B8%80%E9%A6%96%22+%E5%A7%9C%E5%8D%9A%E6%96%87。未找到具体报刊名称、出版年月日或诗集卷次；“外一首”显示其可能是报刊副刊组合标题。</t>
         </is>
       </c>
     </row>
@@ -11125,7 +11125,7 @@
       </c>
       <c r="J230" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=唐代墓志。关键词=唐故九姓突厥契苾李中郎、契苾李、赠右领军卫大将军、九姓突厥、契苾氏、墓志。母项=全唐文、唐代墓志汇编、隋唐五代墓志汇编、唐代墓志铭汇编、历代墓志汇编。候选站=。应重点核对“契苾李”是否为复姓、墓主姓名及“中郎”官称；可按契苾氏、九姓突厥、右领军卫大将军和出土地交叉检索墓志录文及图版。未找到具体公开全文页。</t>
         </is>
       </c>
     </row>
@@ -11363,7 +11363,7 @@
       </c>
       <c r="J233" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=边区政府档案中的复合文书条目。关键词=吴光祖、边区 特种民族证明书、特别生费、边区政府 呈 函 代电、民族证明书。母项=陕甘宁边区政府档案、晋察冀边区政府教育档案、抗日根据地民族工作档案汇编、边区教育、救济和优待费档案。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%90%B4%E5%85%89%E7%A5%96%20%E8%BE%B9%E5%8C%BA%20%E7%89%B9%E7%A7%8D%E6%B0%91%E6%97%8F&amp;title=Special:MediaSearch&amp;type=image。题名明显是同一案卷中呈、函、代电的合并描述，需先确认边区、机关和年份，未找到具体文书页。</t>
         </is>
       </c>
     </row>
@@ -11505,7 +11505,7 @@
       </c>
       <c r="J236" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古调查或文物发现报告。关键词=复县 谭家屯 窖藏、复县窖藏、谭家屯窖藏、瓦房店 谭家屯 文物、辽南 窖藏 考古。母项=《文物》考古简报、辽宁省文物考古调查资料、《辽宁省志·文物志》、复县地方志或瓦房店地方文物资料。候选站=https://commons.wikimedia.org/w/index.php?search=%E8%B0%AD%E5%AE%B6%E5%B1%AF%20%E7%AA%96%E8%97%8F&amp;title=Special:MediaSearch&amp;type=image。复县为旧地名，今多与瓦房店市相关；需同时检索复县、瓦房店和谭家屯，未找到以此题名公开的具体报告页。</t>
         </is>
       </c>
     </row>
@@ -11551,7 +11551,7 @@
       </c>
       <c r="J237" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折或题本。关键词=盛京户部侍郎王朝恩、王朝恩、旗地、民人开垦、开垦土地、盛京户部。母项=盛京户部档案、清代宫中档奏折、军机处档奏折、清代土地关系档案史料、盛京将军衙门档案。候选站=。条目像档案目录题名，可能不是独立文献。应以王朝恩任职年代、折件日期、旗地所在州县和档号定位；未找到可核验的具体全文页。</t>
         </is>
       </c>
     </row>
@@ -11597,7 +11597,7 @@
       </c>
       <c r="J238" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代地方财政档案公文。关键词=熊岳防守尉、亮帖税银、发新帖、奉天度支司、熊岳 咨、防守尉 税银。母项=清代奉天财政档案、盛京将军衙门档案、奉天度支司档案、清代东北地方财政文书汇编。候选站=https://commons.wikimedia.org/w/index.php?search=%E7%86%8A%E5%B2%B3%E9%98%B2%E5%AE%88%E5%B0%89%20%E4%BA%AE%E5%B8%96%E7%A8%8E%E9%93%B6&amp;title=Special:MediaSearch&amp;type=image。题名是清代档案目录式长题名，关键定位项应为年代、档号、熊岳所属旗务机关和亮帖制度，未找到具体卷页或全文。</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="J239" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代政令或档案子项。关键词=布告征收旗地粮赋、布告 征收 旗地 粮赋、征收旗地粮赋、旗地粮赋、旗地钱粮、征收旗地钱粮。母项=清实录相关朝实录、清代宫中档奏折及军机处档案、清代地方官府告示汇编、清代八旗事务档案。候选站=https://zh.wikisource.org/wiki/清实录。标题可能是告示或档案中的拟题，并非独立刊本；需补查朝代、地区及档案日期。</t>
         </is>
       </c>
     </row>
@@ -11689,7 +11689,7 @@
       </c>
       <c r="J240" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代报刊文章或新闻标题。关键词=武力对俄声大盛、武力對俄聲大盛、对俄声大盛、對俄聲大盛、对俄、武力。母项=申报、新闻报、时报、大公报、东方杂志、近代报刊中俄关系新闻。候选站=https://zh.wikisource.org/wiki/申报。措辞明显接近报刊标题，必须结合日期、俄事背景和报刊版次检索；目前没有可核验的具体年期或全文页。</t>
         </is>
       </c>
     </row>
@@ -11876,7 +11876,7 @@
       </c>
       <c r="J244" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=唐代史书条目。关键词=张镒 尚结赞 清水 会盟、張鎰 尚結贊 清水、清水会盟、清水盟、唐蕃会盟、贞元三年。母项=资治通鉴卷二百三十三、旧唐书卷一百二十五《张镒传》、新唐书卷一百五十六《张镒传》、册府元龟有关唐蕃盟誓条。候选站=https://zh.wikisource.org/wiki/資治通鑑/卷233; https://zh.wikisource.org/wiki/舊唐書/卷125。该条不是独立著作，题名应为按事件拟定的子项；核心出处为《资治通鉴》卷233。；2026-09-22 gpt-6-astra：找到候选。类型=唐代史书条目。关键词=张镒 尚结赞 清水 会盟、清水会盟、清水盟、唐蕃会盟、贞元三年。母项=资治通鉴、旧唐书、新唐书。候选站=https://zh.wikisource.org/wiki/資治通鑑/卷233; https://zh.wikisource.org/wiki/舊唐書/卷125。题名为事件拟题，核心出处为《资治通鉴》卷233。；2026-09-22 gpt-6-astra：找到候选。类型=唐代史书事件条目。关键词=张镒、張鎰、尚结赞、尚結贊、清水会盟、清水盟。母项=《资治通鉴》卷二百三十三、《旧唐书》卷一百二十五《张镒传》、《新唐书》卷一百五十六《张镒传》。候选站=https://zh.wikisource.org/wiki/資治通鑑/卷233; https://zh.wikisource.org/wiki/舊唐書/卷125。题名为事件拟题，核心定位为《资治通鉴》卷二百三十三。；2026-09-22 gpt-6-astra：找到候选。类型=唐代史书事件条目。关键词=张镒、張鎰、尚结赞、尚結贊、清水会盟、清水盟。母项=《资治通鉴》卷二百三十三、《旧唐书》卷一百二十五《张镒传》、《新唐书》卷一百五十六《张镒传》。候选站=https://zh.wikisource.org/wiki/資治通鑑/卷233; https://zh.wikisource.org/wiki/舊唐書/卷125。题名为后拟事件标题，核心出处是《资治通鉴》卷二百三十三。</t>
         </is>
       </c>
     </row>
@@ -11922,7 +11922,7 @@
       </c>
       <c r="J245" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古学专题或现代教材章节。关键词=史前物品交换、史前交换、史前贸易、新石器时代交换、史前社会物质交换、prehistoric exchange。母项=中国考古学·新石器时代卷、中国考古学通论、史前社会经济与交换研究、考古学相关期刊论文。候选站=。更像现代考古学教材或展览说明中的章节标题；未确认到具体书名、卷次、期刊年期或公开全文。</t>
         </is>
       </c>
     </row>
@@ -12015,7 +12015,7 @@
       </c>
       <c r="J247" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=博物馆藏品条目。关键词=掐丝珐琅螭纹瓶、掐絲琺瑯螭紋瓶、螭纹瓶、螭紋瓶、景泰蓝螭纹瓶、铜胎掐丝珐琅螭纹瓶。母项=故宫博物院珐琅器藏品目录、中国金银玻璃珐琅器全集、故宫博物院藏文物珍品全集·珐琅器、各地博物馆馆藏珐琅器数据库。候选站=https://commons.wikimedia.org/w/index.php?search=%E6%8E%90%E4%B8%9D%E7%8F%90%E7%90%85%E8%9E%AD%E7%BA%B9%E7%93%B6&amp;title=Special:MediaSearch&amp;type=image。题名缺少年代、尺寸、藏馆和器物编号，无法确认具体藏品；应优先按馆藏数据库的器名、纹饰和材质组合检索。</t>
         </is>
       </c>
     </row>
@@ -12061,7 +12061,7 @@
       </c>
       <c r="J248" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=短篇作品/散文或报刊文章。关键词=眼镜盒、眼鏡盒、眼镜盒 姜博文、眼镜盒 散文、眼镜盒 报刊。母项=近代报刊副刊、散文集或短篇作品集、姜博文文集、手稿或剪报汇编。候选站=https://zh.wikisource.org/w/index.php?search=%E7%9C%BC%E9%8F%A1%E7%9B%92&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://www.google.com/search?q=%22%E7%9C%BC%E9%95%9C%E7%9B%92%22+%E5%A7%9C%E5%8D%9A%E6%96%87。题名属于常见物件题目，未找到可确认的作者、期刊、年份或文集卷次。</t>
         </is>
       </c>
     </row>
@@ -12107,7 +12107,7 @@
       </c>
       <c r="J249" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=公文/地方官府告示。关键词=藩臬宪示、藩、臬宪示、藩臬憲示、藩臬宪示 姜博文、藩司 臬司 宪示、藩臬示。母项=地方官府档案汇编、清代或民国地方公文、告示汇编、地方志艺文志、政书或案牍文书汇编、姜博文所藏公文、碑帖或历史文献整理本。候选站=https://zh.wikisource.org/w/index.php?search=%E8%97%A9%E8%87%AC%E6%86%B2%E7%A4%BA&amp;title=%E7%89%B9%E6%AE%8A%3A%E6%90%9C%E7%B4%A2; https://www.google.com/search?q=%22%E8%97%A9%E8%87%AC%E5%AE%AA%E7%A4%BA%22。“藩、臬”通常指藩司与臬司，题名很可能是合署公文或告示的档案标题；未找到具体省份、年代、卷册或影印页。</t>
         </is>
       </c>
     </row>
@@ -12202,7 +12202,7 @@
       </c>
       <c r="J251" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代刑科题本或奏折。关键词=新疆昌吉县、许世二、贺福、扎毙、监生、商民。母项=刑科题本、清代新疆刑案档案、宫中档朱批奏折、新疆各级地方官刑案档案、清代刑部档案。候选站=。应按人名、案由和“扎毙”异写检索，重点核对“许世二”是否为“许世儿”“许世贰”等转录异文。未找到公开可核验的具体案件全文页。</t>
         </is>
       </c>
     </row>
@@ -12248,7 +12248,7 @@
       </c>
       <c r="J252" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代军机处档案或奏折题名。关键词=遵旨察核新疆吐鲁番屯田台站、吐鲁番屯田台站、收拨倒存马牛各数目、新疆屯田、吐鲁番台站、察核马牛数目。母项=军机处录副奏折·新疆档、宫中档奏折·新疆屯田、清代新疆满文档案汉译编、新疆图志及清代新疆舆图档案。候选站=。“题为”表明这是档案目录或数据库中的拟题，非独立书名；需以档号、年月、具奏官和文种定位，现无可核验具体页。</t>
         </is>
       </c>
     </row>
@@ -12294,7 +12294,7 @@
       </c>
       <c r="J253" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折。关键词=议政大臣海靳、海靳、预发军士钱粮、军士钱粮、预发钱粮、议政大臣奏折。母项=清代议政王大臣会议档案、军机处档奏折、清代宫中档奏折、清代兵部档案、清代军饷档案。候选站=。“海靳”可能存在满文姓名汉译异写，应结合满文名、具奏日期和军队驻地检索。未找到可核验的具体全文页。</t>
         </is>
       </c>
     </row>
@@ -12340,7 +12340,7 @@
       </c>
       <c r="J254" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代寄谕或军机处档案子项。关键词=寄谕哈喇沙尔、寄諭哈喇沙爾、哈喇沙尔办、哈喇沙尔办事大臣、喀喇沙尔、焉耆。母项=清代军机处寄信档、宫中档奏折及军机处档案·新疆、清实录有关喀喇沙尔条、新疆地方档案汇编。候选站=。“哈喇沙尔”有喀喇沙尔、喀喇沙尔厅、焉耆等异名；题名过于概括，缺少皇帝、年月和收文机构，无法确认具体档案页。</t>
         </is>
       </c>
     </row>
@@ -12433,7 +12433,7 @@
       </c>
       <c r="J256" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折。关键词=署宁远大将军查郎阿、查郎阿、准噶尔、厄鲁特、巴图济尔噶勒、解送京城。母项=清代宫中档奏折、军机处档奏折、平定准噶尔方略、清实录、清代边疆满文档案译编。候选站=。可先依据查郎阿任宁远大将军年代查《清实录》及《平定准噶尔方略》对应事件，再回查奏折档案。人名“巴图济尔噶勒”需检索满文转写和“巴图济尔噶尔”等异写。未找到具体公开全文页。</t>
         </is>
       </c>
     </row>
@@ -12479,7 +12479,7 @@
       </c>
       <c r="J257" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古发掘报告。关键词=永和龙吞泉遗址、龙吞泉遗址、永和遗址、龙吞泉、遗址发掘报告、考古发掘。母项=考古、文物、考古学报、山西省考古调查报告、临汾市文物考古资料汇编、山西省文物考古研究院年度考古报告。候选站=。可能是考古期刊中的发掘简报或地方考古调查报告，不一定为独立出版物。应按“山西永和县”“临汾永和”“龙吞泉”及发现年代检索期刊目录和地方文物部门报告。未找到具体刊名、年期或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -12525,7 +12525,7 @@
       </c>
       <c r="J258" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=元代祭祀文或碑刻文献。关键词=至正九年正月御祭中镇文、至正九年御祭中镇、至正九年正月祭中镇、御祭中镇文、中镇霍山祭文、至正九年。母项=元代文献集成及元文类、霍山志或中镇霍山志、历代名山志、永乐大典辑佚祭祀文献、元代碑刻集成。候选站=。“中镇”通常指霍山，题名可能来自地方志、碑刻录文或元代文集目录；未确认到具体卷次、碑号或公开全文。</t>
         </is>
       </c>
     </row>
@@ -12619,7 +12619,7 @@
       </c>
       <c r="J260" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊消息或档案目录条目。关键词=蒙藏会议、蒙藏会议预备会、阎锡山 太原、阎在太原召集、蒙藏事务、蒙藏院。母项=民国报刊地方新闻、蒙藏院档案、阎锡山相关档案汇编、民国政府蒙藏事务档案。候选站=https://zh.wikisource.org/w/index.php?search=%E8%92%99%E8%97%8F%E4%BC%9A%E8%AE%AE%E9%A2%84%E5%A4%87%E4%BC%9A+%E9%98%8E%E5%9C%A8%E5%A4%AA%E5%8E%9F。题名更像报刊标题或姜博文目录的概括性标题。应按阎锡山、太原、蒙藏会议、蒙藏院及具体年份检索民国报刊和档案汇编，并核对繁体“蒙藏會議預備會”。</t>
         </is>
       </c>
     </row>
@@ -12665,7 +12665,7 @@
       </c>
       <c r="J261" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代诗歌或报刊文学篇目，非独立书籍。关键词=姜博文 8月28日、姜博文 八月二十八日、姜博文 8月28日 诗、姜博文 8月28日 报刊、姜博文 八月二十八日 文学。母项=姜博文诗歌或散文合集、当代文学期刊及报纸副刊、姜博文作品目录、年谱或档案汇编。候选站=。未找到可核验的具体书名、卷次、期刊年期或公开全文页。题名过于通用，应结合作者生卒年、作品年代及篇体，在报刊数据库、地方文学资料和姜博文作品集目录中查找。现代作品即使确认出处，也可能仅有书目或馆藏信息，不能据此判断可整本下载。</t>
         </is>
       </c>
     </row>
@@ -12758,7 +12758,7 @@
       </c>
       <c r="J263" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=书信、回忆录章节或报刊标题。关键词=俄国 外蒙 侵绥、外蒙古 绥远、率军增防、进取库伦、库伦、徐树铮。母项=段祺瑞政府外交军事档案、徐树铮西北军事活动档案、民国初年边疆史料、民国报刊外交军事新闻。候选站=https://zh.wikisource.org/w/index.php?search=%E4%BF%84%E5%9B%BD+%E5%A4%96%E8%92%99+%E4%BE%B5%E7%BB%A5+%E5%BA%93%E4%BC%A6。“先生”缺少指代对象，可能是书信或回忆录中的摘标题。应以“库伦”“绥远”“外蒙”“徐树铮”“段祺瑞”组合检索，并核对“绥”“綏”和“库伦”“庫倫”。</t>
         </is>
       </c>
     </row>
@@ -12947,7 +12947,7 @@
       </c>
       <c r="J267" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=北魏造像记。关键词=许儁三十人等造像记、许俊三十人等造像记、许儁造像、许俊造像、北魏造像记、造像记 许儁。母项=《全北魏文》、《金石萃编》北魏造像部分、《中国石刻文献全编》北魏造像类。候选站=https://commons.wikimedia.org/w/index.php?search=%E8%AE%B8%E5%84%81%E4%B8%89%E5%8D%81%E4%BA%BA%E7%AD%89%E9%80%A0%E5%83%8F%E8%AE%B0&amp;title=Special:MediaSearch&amp;type=image。未找到可核验的具体全文页、拓片页或明确卷次。</t>
         </is>
       </c>
     </row>
@@ -13039,7 +13039,7 @@
       </c>
       <c r="J269" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地方报刊消息或宗教团体记录。关键词=山东 青州 回民、马崑山 阿訇、马昆山 阿訇、悬匾、纪念大会、青州 伊斯兰教。母项=民国时期回教报刊、山东地方报刊、青州地方志、中国伊斯兰教史料汇编。候选站=。“崑/昆”“阿訇/阿衡”及“悬匾/懸匾”均应纳入异体检索。尚未找到具体报刊、日期、卷期或地方志页码。</t>
         </is>
       </c>
     </row>
@@ -13085,7 +13085,7 @@
       </c>
       <c r="J270" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=衍圣公府档案文书。关键词=衍圣公府劄付、衍圣公府札付、陈裔远、题补奏差、奏差事、孔府档案。母项=《曲阜孔府档案史料》、《明清档案与孔府档案》、衍圣公府档案文书汇编。候选站=https://commons.wikimedia.org/w/index.php?search=%E8%A1%8D%E5%9C%A3%E5%85%AC%E5%BA%9C%E5%8A%84%E4%BB%98&amp;title=Special:MediaSearch&amp;type=image。条目应为孔府档案中的单件文书，未找到可核验的具体档号、册次或开放全文页。</t>
         </is>
       </c>
     </row>
@@ -13131,7 +13131,7 @@
       </c>
       <c r="J271" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代档案母项。关键词=录副奏折、清代录副奏折、军机处录副奏折、录副奏折档案、清代奏折汇编。母项=中国第一历史档案馆藏军机处录副奏折、《清代档案史料丛编》、清代宫中档奏折及军机处档折件。候选站=。这是档案类别或母项名称，不是可据此定位的独立文献。缺少年代、事由、具名人物、档号或册次，无法生成具体全文页。</t>
         </is>
       </c>
     </row>
@@ -13417,7 +13417,7 @@
       </c>
       <c r="J277" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代或民初官府档案条文。关键词=札巴塘、巴塘、委员、垦夫、工匠、按价雇用。母项=清代四川边务档案、川边经略档案、西藏地方档案、巴塘厅志或巴安县志、清季川滇边务档案。候选站=https://zh.wikisource.org/w/index.php?search=%E5%B7%B4%E5%A1%98+%E5%9E%A6%E5%A4%AB+%E5%B7%A5%E5%8C%A0+%E6%8C%89%E4%BB%B7%E9%9B%87%E7%94%A8。题名可能是档案编目者的压缩标题，不一定为原文题名。需查清季川边奏折、四川劝业或屯垦档案，并检索“札巴塘”“巴塘”“垦务”“委员”。</t>
         </is>
       </c>
     </row>
@@ -13463,7 +13463,7 @@
       </c>
       <c r="J278" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地方官署禀文。关键词=定乡、冷家骥、委员、修通车路、定乡等处、禀请。母项=川边经略档案、四川地方公文汇编、定乡县志或地方志、清末民初交通建设档案。候选站=。“定乡”可能为地名、旧县名或藏区行政地名，需结合年代核定。尚未找到冷家骥名下具体档案卷号、册号或影印页。</t>
         </is>
       </c>
     </row>
@@ -13509,7 +13509,7 @@
       </c>
       <c r="J279" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代军机处电报及邮传部公文。关键词=军机处、邮传部、电线、安设邮局、速运、电报线路。母项=军机处录副奏折、清代邮传部档案、清实录、清代电报史料汇编、中国第一历史档案馆军机处档案。候选站=https://zh.wikisource.org/w/index.php?search=%E9%82%AE%E4%BC%A0%E9%83%A8+%E7%94%B5%E7%BA%BF+%E5%AE%89%E8%AE%BE%E9%82%AE%E5%B1%80。题名疑为档案整理者拟题。应按光绪末年至宣统年间检索“邮传部”“电线”“电报”“邮局”，并核对军机处录副奏折的具体年月、折件和档号。</t>
         </is>
       </c>
     </row>
@@ -13601,7 +13601,7 @@
       </c>
       <c r="J281" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案汇编中的母项或文件组标题。关键词=西川、邮政管理局、邮政局、四川邮政、邮政公文、邮务。母项=清末民初邮政档案、交通部邮政总局档案、四川省档案馆邮政档案、中国近代邮政史料汇编。候选站=。该标题明显可能是文件组或母项，不宜当作独立文献检索。需先确定“西川”所指区域及年代，再按邮政总局、交通部、四川地方档案和邮政年报检索。</t>
         </is>
       </c>
     </row>
@@ -13695,7 +13695,7 @@
       </c>
       <c r="J283" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代学术论文。关键词=红四方面军、民族政策、川西北、三交、交往交流交融、川陕革命根据地。母项=川陕革命根据地史料、红四方面军战史和文献、中国共产党民族工作史、现代民族学或中共党史期刊论文。候选站=https://kns.cnki.net/kns8s/defaultresult/index?kw=%E7%BA%A2%E5%9B%9B%E6%96%B9%E9%9D%A2%E5%86%9B%E7%9A%84%E6%B0%91%E6%97%8F%E6%94%BF%E7%AD%96%E4%B8%8E%E5%B7%9D%E8%A5%BF%E5%8C%97%E5%90%84%E6%B0%91%E6%97%8F%E7%9A%84%E4%B8%89%E4%BA%A4。尚未核实作者、刊名、年份、卷期或 DOI。题名使用“交往交流交融”的简称“三交”，可能是近年民族学或党史论文，不能据此确认有公开整本全文。</t>
         </is>
       </c>
     </row>
@@ -13741,7 +13741,7 @@
       </c>
       <c r="J284" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近代史研究条目或档案摘录，非确证独立书名。关键词=孙绍骞、孙绍骞 留兵耕荒、留兵耕荒、乡城 留兵、驻兵屯田 民族交融、乡城 兵耕荒。母项=清末民初边疆史料汇编、西北边疆史料、民族问题与民族关系史料、地方志中有关驻兵、屯田、垦荒的条目。候选站=。未确认孙绍骞身份、文献出处及“乡城”所指地点。应核对“乡城”是否为“乡城厅”或地名讹写，并检索繁体“留兵耕荒”“留兵垦荒”“驻兵垦荒”。</t>
         </is>
       </c>
     </row>
@@ -13879,7 +13879,7 @@
       </c>
       <c r="J287" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代文学篇目或文物题材文章，非独立书籍。关键词=姜博文 青铜戈、姜博文 青铜戈 诗、姜博文 青铜戈 散文、姜博文 青铜戈 报刊、姜博文 青铜戈 文物。母项=姜博文诗集或散文集、地方文学期刊及报纸副刊、青铜器、考古或地方文史资料汇编、姜博文作品目录或作家档案。候选站=。未找到可核验的具体卷次、期刊年期或公开全文页。检索时需区分文学作品《青铜戈》与考古、文物类同名文章，重点核对作者署名、篇体、发表刊物和年代。现代整理本或期刊如仍在版权期，只能提供书目、馆藏或 DOI 线索，不能据此宣称有整本全文。</t>
         </is>
       </c>
     </row>
@@ -14159,7 +14159,7 @@
       </c>
       <c r="J293" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清末公牍、咨文。关键词=宜铿额、宜鑅额、署总管 宜铿额、两等小学 挑选书生、黑龙江提学使、归司办公事。母项=黑龙江将军衙门档案、黑龙江省教育史料、清末黑龙江学务档案、黑龙江地方文献汇刊中的咨文、札文。候选站=。题名格式符合清末衙门档案目录或档案汇编子项，需按年代、发文机关和档号检索。应同时核对人名异体“宜铿额”“宜鑅额”及“提学使司”“提学使”写法。</t>
         </is>
       </c>
     </row>
@@ -14205,7 +14205,7 @@
       </c>
       <c r="J294" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折或题本。关键词=奏报核定河东吉兰泰引数目事、吉兰泰引、河东盐引、核定引数、奏报吉兰泰、清代盐务奏折。母项=清代宫中朱批奏折盐务档案、《宫中档雍正朝奏折》、清代河东盐政档案汇编。候选站=https://commons.wikimedia.org/w/index.php?search=%E5%90%89%E5%85%B0%E6%B3%B0%E5%BC%95&amp;title=Special:MediaSearch&amp;type=image。未找到可确认的奏折日期、具名官员、档号或具体卷册。</t>
         </is>
       </c>
     </row>
@@ -14251,7 +14251,7 @@
       </c>
       <c r="J295" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代地方革命史资料或纪实文集章节。关键词=察右四旗 抗日根据地、察哈尔右翼四旗 抗日根据地、察右四旗 斗争纪实、察哈尔右翼四旗 抗日战争、蒙旗抗日根据地、乌兰察布 抗日根据地。母项=乌兰察布地区革命史料、察哈尔右翼四旗地方志、内蒙古革命史料丛书、察哈尔抗日根据地史料。候选站=。未确认该题为独立出版物还是地方革命史章节。应重点查察哈尔右翼前旗、中旗、后旗及四子王旗相关县旗志、党史资料和抗日根据地史料；现代整理本通常只能查书目或馆藏，不能据此宣称可整本下载。</t>
         </is>
       </c>
     </row>
@@ -14390,7 +14390,7 @@
       </c>
       <c r="J298" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民国报刊消息、电报或政府档案标题。关键词=彭学沛 孙越崎 抵绥、彭学沛 孙越崎 绥远、张钦 救灾黎 蒙旗自治、中央速救灾黎 蒙旗自治、蒙旗自治 慎重处理、绥远 会谈 孙越崎。母项=民国政府公报、国民政府档案中的绥远蒙旗事务文件、绥远省政府公报、民国报刊有关绥远、蒙旗自治和灾荒的报道。候选站=。题名明显像报刊剪报或档案目录的拼接标题，可能由同一期连续消息合并而成。应分拆检索“彭学沛孙越崎抵绥”“张钦促请中央速救灾黎”“蒙旗自治亦望慎重处理”，并按民国年份查《中央日报》《大公报》《申报》及绥远省政府公报。</t>
         </is>
       </c>
     </row>
@@ -14436,7 +14436,7 @@
       </c>
       <c r="J299" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民国总统府公文、议案或档案目录条目。关键词=总统府 交议 保护蒙旗案、保护蒙旗案、保护蒙古各旗、蒙旗保护案、总统府 蒙旗、国民政府 蒙旗。母项=国民政府总统府档案、国民政府公报、蒙藏委员会档案、民国蒙古问题档案汇编。候选站=。“总统府交议”是档案目录式表述，不能据题名认定为独立出版物。应按民国总统、年份和承办机关检索，并核对“蒙旗”“蒙古各旗”“蒙古旗地”等异称。</t>
         </is>
       </c>
     </row>
@@ -14482,7 +14482,7 @@
       </c>
       <c r="J300" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=中共党史电报或革命历史档案，题名残缺。关键词=习仲勋 马明方 郭炳坤、朱敏 赵忠国 蒙人独贵、蒙人独贵运动、对蒙人独贵运动应大力支持和领导、习仲勋 蒙古族 独贵、陕甘宁 蒙古族运动 电。母项=习仲勋文集或年谱中的电报文稿、陕甘宁边区革命历史文件汇集、陕甘宁边区民族工作史料、中共西北历史资料。候选站=。原题末有未闭合括号，且“蒙人独贵”可能是人名、组织名或转录错误。应核对“独贵”“独贵龙”“蒙人独贵运动”等写法，并按发文人、收文人和电报日期定位档案。</t>
         </is>
       </c>
     </row>
@@ -14528,7 +14528,7 @@
       </c>
       <c r="J301" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民国蒙藏委员会公文、报刊消息或档案标题。关键词=蒙藏会 请开发蒙古交通、蒙藏委员会 开发蒙古交通、蒙古交通建设、开发蒙古交通案、蒙藏委员会 交通、蒙古道路 铁路 公路。母项=蒙藏委员会档案、国民政府公报、蒙藏委员会公报、民国交通建设档案及报刊。候选站=。题名可能是报刊短讯或公文目录，需按年份检索“蒙藏会”“蒙藏委员会”两种称谓，并拆分“蒙古交通”“开发蒙古交通”“蒙古道路建设”等关键词。</t>
         </is>
       </c>
     </row>
@@ -14671,7 +14671,7 @@
       </c>
       <c r="J304" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=抗日战争时期电报或边疆军政档案。关键词=张浩 滚弄 班弄 马美廷、日寇攻占滚弄、班弄土司、马美廷、滚弄 土司 抗日、滇西 抗日 电报。母项=抗日战争时期滇西档案、云南省政府战时档案、西南边疆民族事务史料、抗日战争时期国民政府军事档案汇编。候选站=。“滚弄”“班弄”可能为滇西或缅北地名，需核对异写及地图地名；“马美廷”也应检索“马美庭”“马美廷土司”。题名很可能来自电报汇编目录，暂未找到可核验的具体开放章节或全文页。</t>
         </is>
       </c>
     </row>
@@ -14763,7 +14763,7 @@
       </c>
       <c r="J306" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=招生文件/内部办法。关键词=招生对象及议定招收待遇办法原则、招生对象 招收待遇 办法 原则、招生对象及议定招收待遇办法原则 姜博文、招生待遇 办法 原则 招生。母项=学校招生简章或招生文件汇编、教育行政机关档案汇编、姜博文文稿、书信及工作文件档案。候选站=https://www.google.com/search?q=%22%E6%8B%9B%E7%94%9F%E5%AF%B9%E8%B1%A1%E5%8F%8A%E8%AE%AE%E5%AE%9A%E6%8B%9B%E6%94%B6%E5%BE%85%E9%81%87%E5%8A%9E%E6%B3%95%E5%8E%9F%E5%88%99%22。未确认作者、年代、机构及载体，暂不能定位到具体档案卷册或全文页。</t>
         </is>
       </c>
     </row>
@@ -15000,7 +15000,7 @@
       </c>
       <c r="J311" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代报刊文章、评论或文艺篇目，非独立书籍。关键词=姜博文 特殊问题、姜博文 《特殊问题》、姜博文 特殊问题 诗、姜博文 特殊问题 散文、姜博文 特殊问题 期刊、姜博文 特殊问题 报纸。母项=姜博文文集或作品集、当代文学期刊及报纸副刊、专题评论、思想文化类文集、姜博文年谱、作品目录或档案汇编。候选站=。未找到可核验的具体书名、卷次、期刊年期或公开全文页。题名高度通用，需结合作者身份、发表年代和文章体裁排除同名政论、社论及学术文章。现阶段不能确认其为姜博文独立著作，也不能提供可核验全文 URL。</t>
         </is>
       </c>
     </row>
@@ -15140,7 +15140,7 @@
       </c>
       <c r="J314" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代碑刻。关键词=铜仁松桃 王总爷功德碑、松桃 王总爷碑、光绪十七年 功德碑、贵州松桃碑刻、铜仁碑刻、王总爷功德碑。母项=《贵州省志·文物志》、《松桃苗族自治县志》、贵州地方碑刻汇编。候选站=https://commons.wikimedia.org/w/index.php?search=%E6%9D%BE%E6%A1%83%E7%8E%8B%E6%80%BB%E7%88%B7%E5%8A%9F%E5%BE%B7%E7%A2%91&amp;title=Special:MediaSearch&amp;type=image。未找到该碑的具体地点、碑文录文、地方志卷次或开放图像页。</t>
         </is>
       </c>
     </row>
@@ -15286,7 +15286,7 @@
       </c>
       <c r="J318" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=档案汇编/档案子项。关键词=九世班禅圆寂致祭、九世班禅圆寂 致祭、十世班禅转世坐床、十世班禅转世坐床档案、九世班禅 十世班禅 档案选编、中国藏学出版社 1991。母项=《九世班禅圆寂致祭和十世班禅转世坐床档案选编》、中国藏学出版社1991年版、相关中国第二历史档案馆、西藏自治区档案馆班禅档案汇编。候选站=https://www2.xzmu.edu.cn/xzshjj/getcontent?id=17324&amp;url=show。未找到公开逐件档案全文。检索时应以母项书名、九世班禅圆寂、十世班禅坐床及档案号组合定位具体档案。</t>
         </is>
       </c>
     </row>
@@ -15470,7 +15470,7 @@
       </c>
       <c r="J322" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=性质不明的篇名或卷内子项。关键词=一百六、一百六 古籍、一百六 篇名、一百六 卷。母项=。候选站=。题名过于简略，缺少作者、文类、时代和母项信息；无法可靠判断是篇名、卷次、档号或目录编号，当前未找到可核验对象。</t>
         </is>
       </c>
     </row>
@@ -15516,7 +15516,7 @@
       </c>
       <c r="J323" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=碑刻汇录、专题工具书。关键词=北京内城寺庙碑刻志、北京内城寺庙碑刻、北京寺庙碑刻、董晓萍、吕敏、国家图书馆出版社 2011。母项=《北京内城寺庙碑刻志》全书、北京地区寺庙碑刻资料汇编、北京市文物局或北京文物古迹调查资料。候选站=https://book.douban.com/subject/6969224/。未找到公开可核验的第一卷或第二卷全文页。检索时应分别加入“卷一”“卷二”及具体寺庙、碑名、碑文首句。</t>
         </is>
       </c>
     </row>
@@ -15702,7 +15702,7 @@
       </c>
       <c r="J327" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=方志/乡土志子项。关键词=塔城直隶厅乡土志、塔城厅乡土志、塔尔巴哈台乡土志、塔城 乡土志稿、塔城直隶厅、新疆乡土志稿 第375页。母项=《新疆乡土志稿》、全国图书馆文献缩微复制中心1990年影印本、《中国地方志集成·新疆府县志辑》相关塔城资料。候选站=。目前只有《新疆乡土志稿》约第375页这一母项页码线索，未找到可核验的公开章节或扫描页。应按塔城、塔尔巴哈台、塔城直隶厅三组名称核对目录。</t>
         </is>
       </c>
     </row>
@@ -15748,7 +15748,7 @@
       </c>
       <c r="J328" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=明代方志。关键词=嘉靖嘉定县志、嘉靖二十六年 嘉定县志、嘉定县志 明嘉靖、嘉定县志 卷、上海府县旧志丛书 嘉定县卷、嘉定县志 乾隆。母项=《上海府县旧志丛书·嘉定县卷》、《嘉定县志》历代版本、《上海府县旧志丛书》。候选站=https://www.guoxuedashi.com/shumu/gj-2042658vo.html。未找到明嘉靖二十六年刻本的公开逐卷全文。应按“卷一至卷若干”“建置志”“学校志”“人物志”“艺文志”等子项继续检索；2012年上海古籍出版社整理本属于现代整理出版物，不能据此宣称整本可免费下载。</t>
         </is>
       </c>
     </row>
@@ -15794,7 +15794,7 @@
       </c>
       <c r="J329" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案/公文子项。关键词=教育部 公文、教育部训令、教育部指令、教育部咨文、教育部呈文、教育部相关公文 马雨衡。母项=教育部档案全宗、《中华民国史档案资料汇编》教育类档案、《政府公报》教育部公文、相关省政府档案汇编。候选站=。条目缺少年份、文号、收发机关和事由，无法定位具体公文或母项卷次。</t>
         </is>
       </c>
     </row>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="J330" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=方志/边疆史地文献。关键词=塔尔巴哈台志略、塔爾巴哈臺志略、塔尔巴哈台志略附乌什事宜、塔爾巴哈臺志略附烏什事宜、乌什事宜、吴丰培。母项=吴丰培整理本《塔尔巴哈台志略附乌什事宜》、新疆地方志及边疆史地文献丛刊、清代新疆舆地文献汇编。候选站=https://www.guoxuedashi.com/shumu/gj-2859596kt.html。已知结构为《志略》1卷、《乌什事宜》1卷；未找到公开逐页全文或识典古籍、维基文库章节页。</t>
         </is>
       </c>
     </row>
@@ -16024,7 +16024,7 @@
       </c>
       <c r="J334" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=近现代文集或合刊。关键词=都市丛谈、燕市积弊、北京古籍出版社 1995 都市丛谈、都市叢談、燕市積弊。母项=《都市丛谈》《燕市积弊》合刊、北京古籍出版社1995年版、相关民国北京社会掌故或笔记丛书。候选站=https://book.douban.com/series/1543?order=time&amp;page=5。1995年整理本属于现代出版物，当前没有找到合法开放的整本全文；可继续查国家图书馆、地方图书馆及高校馆藏目录，核对ISBN、编者和页码。</t>
         </is>
       </c>
     </row>
@@ -16117,7 +16117,7 @@
       </c>
       <c r="J336" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=金石器物铭文/考古资料子项。关键词=藏汉铭文铁钟、藏漢銘文鐵鐘、藏汉文铁钟、藏漢文鐵鐘、铁钟 铭文 藏文 汉文、西藏 铁钟 铭文。母项=西藏金石录及碑刻资料汇编、西藏文物考古相关图录、寺院文物调查报告、相关墓志、碑刻与金石铭文论文。候选站=。未找到能确认器物名称、收藏地点、年代或完整铭文录文的具体来源。题名不可直接替换为“藏汉铭文铜钟”或“桑耶寺铜钟”。</t>
         </is>
       </c>
     </row>
@@ -16163,7 +16163,7 @@
       </c>
       <c r="J337" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=近现代金融史研究中的个案子项。关键词=锦生润票号、錦生潤票號、锦生润、山西票号 锦生润、锦生润票号研究。母项=《锦生润票号研究》、山西票号史、中国金融史相关文集。候选站=https://history.sxu.edu.cn/szdw/qzjs/zgsx/zgjxds/jdsth/2bcb060135f24b98958c55037ae9d6da.htm。《锦生润票号研究》为2022年出版的现代学术著作，不能据此宣称已有开放全文；应继续查出版社书目、馆藏目录及论文数据库中的相关章节或论文。</t>
         </is>
       </c>
     </row>
@@ -16393,7 +16393,7 @@
       </c>
       <c r="J342" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代题本/奏折或咨文档案子项。关键词=甘肃宁夏罗归并管辖、奉裁新宝二县、无籍可归户民授给田亩、应征粮银数目事、新宝县 裁撤、宁夏 罗 县 田亩 粮银。母项=清代军机处档案、清代宫中档奏折及军机处档折件、《明清档案》相关甘肃宁夏档案、清代甘肃宁夏地方档案汇编。候选站=。题名可能是档案目录中的长题名，需补充朝代、年份、文书类型、档号或收藏机构后才能定位卷册和页码。</t>
         </is>
       </c>
     </row>
@@ -16439,7 +16439,7 @@
       </c>
       <c r="J343" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民国公文/省政府档案子项。关键词=程耀黎、程参议员耀黎、降低海原县等级、海原县等级 负担平均、省政府降低海原县等级、咨送程参议员提建议。母项=宁夏省政府档案、民国宁夏省政府公报、《宁夏档案史料》、海原县政府档案及民国县政档案汇编。候选站=。未找到具体档案馆藏页、卷次或公开影印页。应以“程耀黎”“海原县降等”“负担平均”及民国年份组合检索宁夏省政府公报和省政府档案目录。</t>
         </is>
       </c>
     </row>
@@ -16485,7 +16485,7 @@
       </c>
       <c r="J344" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=丛书／史料汇编。关键词=中华民国史料丛稿、中华民国史料、中华民国史资料、中华民国史料丛刊、中华书局、译稿。母项=中华书局出版的《中华民国史料丛稿》各辑、《中华民国史资料丛稿》相关分辑、民国史专题资料选辑、民国史档案与文献汇编。候选站=https://ci.nii.ac.jp/ncid/BN05618094。这是丛书总名，不能按独立著作检索。应先从书目记录反推具体辑名、卷次、译者或专题名，再检索中华书局目录、馆藏联合目录和各分辑题名。当前未找到可核验的具体全文页。</t>
         </is>
       </c>
     </row>
@@ -16623,7 +16623,7 @@
       </c>
       <c r="J347" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊图像／新闻照片题名。关键词=连阳瑶民、连阳瑶族、到省观光、老幼共十九名、男女服饰奇异、十九名瑶民。母项=民国时期报刊新闻图片、广东省政府公报或政务档案中的民族事务材料、民国报刊的社会新闻、风俗照片栏目、广东省立中山图书馆旧报刊影像资料。候选站=。题名很可能是报刊照片说明或档案照片说明，不宜按独立书名检索。应结合“连阳”旧称、广东省城、瑶民观光、十九人、服饰等词，重点查民国报刊的图片说明和广东地方档案目录。</t>
         </is>
       </c>
     </row>
@@ -16669,7 +16669,7 @@
       </c>
       <c r="J348" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民族调查报告、报告子项。关键词=粤北瑶山考察简报、广东北江瑶山初步调查报告、中山大学 1936 瑶山、广东北江瑶山、瑶族调查报告文集、北江瑶族调查。母项=《瑶族调查报告文集》、中山大学 1936 年广东北江瑶山调查资料、民国时期中山大学民族调查报告。候选站=。现有题名可能是《广东北江瑶山初步调查报告》的误称或文集内篇名。未找到可核验的具体全文页；应以作者、调查队名称、报告编印机关及《瑶族调查报告文集》目录反查。</t>
         </is>
       </c>
     </row>
@@ -16715,7 +16715,7 @@
       </c>
       <c r="J349" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案公文／政治文献子项。关键词=陈炳焜、陈炳焜宣称、军政府、陈炳焜公文、广西军政府、广东军政府。母项=民国初年广西军政档案汇编、护国战争及南方军政府史料、《近代史资料》相关专题、民国报刊中的通电、宣言和公文汇编。候选站=。陈炳焜与广西军政、护国战争及民国初年地方军政关系密切。“宣称军政府”可能是编目者对公文内容的概括，需用陈炳焜、广西、军政府、通电、文告等词反查母项。</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="J351" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=金石题记／造塔题记。关键词=刘仪夫、刘仪夫兄弟、造塔题记、题记三种、刘仪夫造塔、金石汇目。母项=金石汇目分编、地方金石志、中国石刻文献索引、佛教金石文献汇编。候选站=https://www.shidianguji.com/book/NGJ892312001037442311963/chapter/1loh8q8mx2bk6。已提供具体识典章节页。检索时应以章节中的碑刻地点、年代、塔名和录文首句反查地方金石志及金石目录，以确认“三种”的具体分项。；2026-09-22 gpt-6-astra：找到候选。类型=金石题记／造塔题记。关键词=刘仪夫、刘仪夫兄弟、造塔题记、题记三种、刘仪夫造塔。母项=金石汇目分编、地方金石志、佛教金石文献汇编。候选站=https://www.shidianguji.com/book/NGJ892312001037442311963/chapter/1loh8q8mx2bk6。已定位到具体识典章节；“三种”的分项仍需依据章节内碑刻地点、年代、塔名和录文核对。；2026-09-22 gpt-6-astra：找到候选。类型=金石题记。关键词=刘仪夫、刘仪夫兄弟、造塔题记、题记三种。母项=金石汇目分编、地方金石志、佛教金石文献汇编。候选站=https://www.shidianguji.com/book/NGJ892312001037442311963/chapter/1loh8q8mx2bk6。已定位到具体识典章节；“三种”的分项仍需依据章节内录文、地点和年代核对。</t>
         </is>
       </c>
     </row>
@@ -16853,7 +16853,7 @@
       </c>
       <c r="J352" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=考古发掘报告中的出土遗物子项。关键词=三水银洲遗址、银洲贝丘遗址、出土石镞、石镞、广东三水市银洲贝丘遗址发掘简报、考古2000年第6期。母项=《考古》2000年第6期、《广东三水市银洲贝丘遗址发掘简报》、广东地区新石器时代遗址考古报告、银洲贝丘遗址出土遗物图版和器物统计。候选站=https://www.sslib.com.cn/yinzhouyizhi/3094.html。该条不是独立出版物，而是发掘简报中的出土器物子项。应进一步定位《考古》2000年第6期论文的页码、图版编号、器物编号及出土层位。</t>
         </is>
       </c>
     </row>
@@ -16899,7 +16899,7 @@
       </c>
       <c r="J353" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古出土器物子项。关键词=深圳大梅沙、大梅沙铜矛、带钉孔铜矛、大梅沙遗址、深圳出土铜矛、岭南青铜器。母项=深圳地区考古调查与发掘报告、广东出土青铜器图录、深圳文物考古研究所藏品目录、岭南地区先秦考古资料汇编。候选站=。应按器物特征“钉孔”“带孔”“铜矛”反查考古报告图版和博物馆藏品目录。当前未找到可核验的具体章节、期刊页或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -17129,7 +17129,7 @@
       </c>
       <c r="J358" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=考古发掘简报、期刊论文。关键词=宁连高速公路天长市釜山取土场西汉墓葬群发掘简报、釜山取土场 西汉墓葬群、天长市 釜山 西汉墓、《文物研究》第17辑、天长市博物馆、天长市文物管理所。母项=《文物研究》第17辑、安徽省天长市文物考古调查与发掘资料、宁连高速公路建设工程考古资料。候选站=https://www.ecsponline.com/goods.php?id=40901。未找到该篇的公开全文页。应按《文物研究》第17辑目录定位篇首、页码及作者，并检索题名去掉“宁连高速公路”后的变体。</t>
         </is>
       </c>
     </row>
@@ -17221,7 +17221,7 @@
       </c>
       <c r="J360" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=明清档案或奏折题本汇编中的子项。关键词=内阁奏议题稿、内阁奏议、奏议题稿、内阁题稿、明代内阁奏议、清代内阁题本。母项=明代内阁档案、清代内阁档案、宫中档奏折与题本、《明实录》相关奏议。候选站=。题名不足以确定朝代、作者、档案馆藏号或母项。未找到可核验的独立书名及具体全文页；应先根据引文中的年号、部院、奏议日期或题本字号反推档案母项。</t>
         </is>
       </c>
     </row>
@@ -17267,7 +17267,7 @@
       </c>
       <c r="J361" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=司法档案／行政公文子项。关键词=审理颍上县、颍上县公文、颍上县审理、安徽颍上、题为审理、县司法档案。母项=安徽省档案馆民国司法档案、颍上县志及司法档案、民国安徽地方政府公文汇编、安徽地方审判厅或县政府档案汇编。候选站=。题名语序可能来自档案目录或图像识别，需确认“题为”是否为编目说明。应结合年代、发文机关、案件名称和收文对象检索安徽地方档案目录。</t>
         </is>
       </c>
     </row>
@@ -17313,7 +17313,7 @@
       </c>
       <c r="J362" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=选举档案／行政公文子项。关键词=国民大会代表、立法院立法委员、安徽选举事务所、安徽选举、国民大会代表选举、立法委员选举。母项=国民大会代表选举档案汇编、立法院立法委员选举档案、安徽省政府民政厅选举档案、民国安徽省政府公报、国民政府公报中的安徽选举文件。候选站=。这是选举行政档案母项下的公文集合，不是独立书名。应以“安徽省政府民政厅”“选举事务所”“国民大会代表”“立法委员”及具体年份组合检索；当前未找到可核验的具体全文页或章节页。</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="J363" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊文章或政治文告，日期可能为篇名或事件日期。关键词=一九二五年十二月十七日、1925年12月17日、一九二五 十二月十七日、十二月十七日 政治文告、马雨衡。母项=1925年前后中共中央、工会或革命报刊汇编、《向导》周报、《中国青年》、《工人之路》及地方党团刊物、1925年报刊合订本或革命文献汇编。候选站=https://archive.org/advancedsearch.php?q=%221925%E5%B9%B412%E6%9C%8817%E6%97%A5%22&amp;fl%5B%5D=identifier,title&amp;rows=50&amp;page=1&amp;output=json; https://books.google.com/books?q=%22%E4%B8%80%E4%B9%9D%E4%BA%8C%E4%BA%94%E5%B9%B4%E5%8D%81%E4%BA%8C%E6%9C%88%E5%8D%81%E4%B8%83%E6%97%A5%22。目前没有可核验的独立篇名、作者、刊物或具体页码。应优先按1925年12月17日前后报刊日期逐页核查，不能据日期直接认定为书名。</t>
         </is>
       </c>
     </row>
@@ -17451,7 +17451,7 @@
       </c>
       <c r="J365" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=革命文献或会议宣言，属会议文件子项。关键词=全国苏维埃区域代表大会宣言、全国苏维埃区域代表大会、苏维埃区域代表大会 宣言、1930年5月 上海、全国苏维埃区域代表会议。母项=《中国工运史料》第28—29期，1930年5月，约第6页、1930年上海工运和苏维埃运动会议文件汇编、《中央革命根据地史料选编》或土地革命战争时期文献汇编、中国。候选站=https://books.google.com/books?q=%22%E5%85%A8%E5%9B%BD%E8%8B%8F%E7%BB%B4%E5%9F%83%E5%8C%BA%E5%9F%9F%E4%BB%A3%E8%A1%A8%E5%A4%A7%E4%BC%9A%E5%AE%A3%E8%A8%80%22; https://archive.org/advancedsearch.php?q=%22%E4%B8%AD%E5%9B%BD%E5%B7%A5%E8%BF%90%E5%8F%B2%E6%96%99%22%20%2228%22%20%2229%22&amp;fl%5B%5D=identifier,title&amp;rows=50&amp;page=1&amp;output=json。已有较具体母项和页码线索，但未找到可核验全文页。应核对第28—29期合刊或连续出版物的卷期标识，并检查第6页标题是否为异名。</t>
         </is>
       </c>
     </row>
@@ -17497,7 +17497,7 @@
       </c>
       <c r="J366" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=地方文史资料文章。关键词=宁国县的民族概况、宁国 民族概况、宁国县 民族、宁国文史资料 第四辑、政协宁国县委员会 文史资料。母项=政协宁国县委员会《宁国文史资料选辑》第4辑，约第87页、《宁国文史资料》或《宁国文史资料选辑》各辑、宁国地方志、民族志及政协文史资料汇编。候选站=https://books.google.com/books?q=%22%E5%AE%81%E5%9B%BD%E6%96%87%E5%8F%B2%E8%B5%84%E6%96%99%E9%80%89%E8%BE%91%22%20%22%E7%AC%AC4%E8%BE%91%22; https://archive.org/advancedsearch.php?q=%22%E5%AE%81%E5%9B%BD%E6%96%87%E5%8F%B2%E8%B5%84%E6%96%99%22&amp;fl%5B%5D=identifier,title&amp;rows=50&amp;page=1&amp;output=json。书名、辑次和约页码较明确，但未找到可核验的具体全文页。应向宁国市政协文史资料室、安徽省图书馆或地方志馆核对第4辑目录。</t>
         </is>
       </c>
     </row>
@@ -17589,7 +17589,7 @@
       </c>
       <c r="J368" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=辽代墓志铭子项。关键词=王守谦墓志 辽 保宁元年、辽代石刻 王守谦、王守谦 墓志铭。母项=《辽代石刻文续编》、辽宁人民出版社，2010年，约第10页、辽代墓志汇编、辽代石刻文整理本。候选站=https://search.worldcat.org/search?q=%E8%BE%BD%E4%BB%A3%E7%9F%B3%E5%88%BB%E6%96%87%E7%BB%AD%E7%BC%96。已有母项、年代和约页码，但未找到王守谦墓志的公开录文、拓片或具体扫描页。</t>
         </is>
       </c>
     </row>
@@ -17635,7 +17635,7 @@
       </c>
       <c r="J369" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=元代碑刻子项。关键词=定志塔铭、定圆 定志塔铭、至元五年 定志塔、1268 定志塔铭、元代碑刻辑释。母项=《元代碑刻辑释》、元代碑刻资料汇编、地方寺院或佛塔碑刻录。候选站=。已有时间、撰书者和著录母项线索，但当前未找到《元代碑刻辑释》的具体卷页、拓片、录文或稳定开放页面；应按至元五年、定圆及出土地反查目录。</t>
         </is>
       </c>
     </row>
@@ -17727,7 +17727,7 @@
       </c>
       <c r="J371" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=近代法令汇编。关键词=大清新法令 1901 1911、大清新法令 第一卷、清末新法令、光绪新法令、宣统新法令。母项=《大清新法令1901—1911》全套11卷、商务印书馆2010年点校本、清末法制史资料汇编。候选站=https://www.cp.com.cn/book/925d7eef-8.html。这是2010年现代整理出版的法令汇编，出版社页面仅提供书目信息，不能视为整本开放全文；应按具体卷次、年份和法令名称查馆藏目录、论文引用及清末报刊或档案中的原始刊载。</t>
         </is>
       </c>
     </row>
@@ -17773,7 +17773,7 @@
       </c>
       <c r="J372" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案文件组或档案汇编子项。关键词=北平市政府 招待班禅、北平市政府 班禅、招待班禅委员会、班禅驻京 北平 公文、班禅额尔德尼 北平市政府。母项=北平市政府档案、北平市政府关于接待班禅额尔德尼档案、民国时期蒙藏委员会档案、班禅驻京及中央政府接待档案汇编、北平市政府公报或市政档案汇编。候选站=https://archive.org/advancedsearch.php?q=%E5%8C%97%E5%B9%B3%E5%B8%82%E6%94%BF%E5%BA%9C%20%E7%8F%AD%E7%A6%85&amp;fl%5B%5D=identifier,title&amp;rows=50&amp;page=1&amp;output=json; https://books.google.com/books?q=%22%E5%8C%97%E5%B9%B3%E5%B8%82%E6%94%BF%E5%BA%9C%22%20%22%E7%8F%AD%E7%A6%85%22。未能确定年代、班禅身份、机构正式名称或档案全宗，暂不能定位具体卷册和页码。应先按九世班禅、十世班禅及‘班禅驻京’分别排查。</t>
         </is>
       </c>
     </row>
@@ -17819,7 +17819,7 @@
       </c>
       <c r="J373" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=报刊文章，后收入选编。关键词=二期抗战中回民应有之努力、二期抗战 回民 应有的努力、抗战中回民应有之努力、回民 抗战 努力、回族历史报刊文选 抗战卷。母项=王正儒、雷晓静编《回族历史报刊文选·抗战卷》上册，宁夏人民出版社，2012年，约第493页、抗战时期回族报刊、《月华》《回教新文化》及西北回族报刊、回族历史报刊。候选站=https://books.google.com/books?q=%22%E4%BA%8C%E6%9C%9F%E6%8A%97%E6%88%98%E4%B8%AD%E5%9B%9E%E6%B0%91%E5%BA%94%E6%9C%89%E4%B9%8B%E5%8A%AA%E5%8A%9B%22; https://archive.org/advancedsearch.php?q=%22%E5%9B%9E%E6%97%8F%E5%8E%86%E5%8F%B2%E6%8A%A5%E5%88%8A%E6%96%87%E9%80%89%22&amp;fl%5B%5D=identifier,title&amp;rows=50&amp;page=1&amp;output=json。已有明确现代整理本、出版社、年份、册次和约页码，但2012年整理本通常受版权限制，不能据此宣称可整本下载。应追索第493页的原刊名、刊期和文章作者。</t>
         </is>
       </c>
     </row>
@@ -17865,7 +17865,7 @@
       </c>
       <c r="J374" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=考古发掘资料及简牍释文，非独立书名。关键词=大通上孙家寨墓地汉简、大通上孙家寨汉简释文、上孙家寨汉简、青海大通上孙家寨墓地、文物 1981 2 汉简。母项=《文物》1981年第2期《大通上孙家寨汉简释文》、《中国简牍集成》第17册，相关图版、释文和校注、青海省大通县上孙家寨墓地发掘简报、中国出土简牍文献汇编。候选站=https://books.google.com/books?q=%22%E5%A4%A7%E9%80%9A%E4%B8%8A%E5%AD%99%E5%AE%B6%E5%AF%A8%E6%B1%89%E7%AE%80%E9%87%8A%E6%96%87%22; https://archive.org/advancedsearch.php?q=%22%E4%B8%8A%E5%AD%99%E5%AE%B6%E5%AF%A8%22%20%E6%B1%89%E7%AE%80&amp;fl%5B%5D=identifier,title&amp;rows=50&amp;page=1&amp;output=json。已能确定期刊年期和《中国简牍集成》第17册，但未找到可核验的公开具体页。检索时应同时查‘大通上孙家寨墓地’发掘报告和《大通县志》考古条目。</t>
         </is>
       </c>
     </row>
@@ -17957,7 +17957,7 @@
       </c>
       <c r="J376" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=现代专著。关键词=瞿昙寺、昙寺、谢佐、青海人民出版社、乐都瞿昙寺、瞿昙寺志。母项=青海人民出版社谢佐《瞿昙寺》、青海地方文献与寺院志资料。候选站=https://search.douban.com/book/subject_search?search_text=%E7%9E%BF%E6%98%99%E5%AF%BA+%E8%B0%A2%E4%BD%90; https://search.worldcat.org/search?q=bn%3A7225015613。未找到可直接核验的公开全文页。2015年前出版物可继续查国家、省级图书馆及高校馆藏；不应据书名直接认定存在电子全文。</t>
         </is>
       </c>
     </row>
@@ -18003,7 +18003,7 @@
       </c>
       <c r="J377" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑记、地方志或金石录子项。关键词=修西宁城碑记、西宁城碑记、重修西宁城碑记、西宁 城 碑、西宁府志 碑记、西宁卫 城碑。母项=《西宁府志》、《西宁卫志》、地方金石志、西宁地区碑刻录文。候选站=。未找到可确认朝代、立碑地点、撰书人或碑文具体页。西宁可能指青海西宁，也可能指其他历史地名；应结合引文中的年号、官职、城名异写和碑额反查方志卷次。</t>
         </is>
       </c>
     </row>
@@ -18049,7 +18049,7 @@
       </c>
       <c r="J378" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似报刊或地方文献子项。关键词=果洛红军沟、红军沟、果洛州、红军长征、红军沟遗址、青海果洛。母项=果洛州志、果洛藏族自治州文物志、青海革命遗址与纪念设施资料、地方报刊专题。候选站=。题名末有不闭合括号，可能是OCR截断或文章中的小标题。需优先按“红军沟”“果洛 红军沟”回溯地方志、文物普查报告和报刊版面。</t>
         </is>
       </c>
     </row>
@@ -18187,7 +18187,7 @@
       </c>
       <c r="J381" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=考古发掘报告中的出土文物子项。关键词=陕西旬邑县西头北魏墓 铜马镳、旬邑县西头遗址 上庙地点 北魏墓 M39、西头北魏墓 铜马镳、考古 2023 2 40 51、陕西旬邑县西头遗址上庙地点北魏墓M39的发掘。母项=《考古》2023年第2期第40—51页《陕西旬邑县西头遗址上庙地点北魏墓M39的发掘》、旬邑县西头遗址考古发掘报告、陕西省考古研究院北魏墓葬发掘资料、西头遗址上。候选站=https://www.parismuseescollections.paris.fr/zh-hans/node/1022630; https://books.google.com/books?q=%22%E9%99%95%E8%A5%BF%E6%97%AC%E9%82%91%E5%8E%BF%E8%A5%BF%E5%A4%B4%E9%81%97%E5%9D%80%E4%B8%8A%E5%BA%99%E5%9C%B0%E7%82%B9%E5%8C%97%E9%AD%8F%E5%A2%93M39%E7%9A%84%E5%8F%91%E6%8E%98%22。已有具体博物馆藏品页和明确期刊卷期、页码；该条目应作为发掘报告中的器物子项处理，不能按独立著作检索。</t>
         </is>
       </c>
     </row>
@@ -18233,7 +18233,7 @@
       </c>
       <c r="J382" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代奏折、档案子项。关键词=乾隆九年 帅念祖 奏、帅念祖 陕北 七州县、贫民出口种地、陕北七州县、乾隆九年陕西巡抚奏折、清代奏折 口外种地。母项=清宫档案奏折、乾隆朝宫中档奏折、《宫中档乾隆朝奏折》、清代陕西巡抚奏折档案。候选站=。题名中的“帅念组”疑为“帅念祖”。未找到可核验的具体档案号、影印册页或公开全文页；应以乾隆九年、陕西巡抚、帅念祖、出口种地及七州县组合检索，并核对“出口”是否为“出边”或“出口外”。</t>
         </is>
       </c>
     </row>
@@ -18279,7 +18279,7 @@
       </c>
       <c r="J383" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=清代宫廷档案汇编、档案数据库母项。关键词=宫中档奏折 乾隆朝、乾隆朝宫中档奏折、宫中档乾隆朝奏折、国立故宫博物院 宫中档、乾隆奏折 日期 人名。母项=《宫中档雍正朝奏折》、《宫中档乾隆朝奏折》、国立故宫博物院清代宫中档奏折档案。候选站=https://qingarchives.npm.edu.tw/。清单项是档案母项而非单篇独立著作。未找到该条目对应的具体档案号、册次或影像页；应先用“乾隆九年、帅念祖、陕西、出口种地”等字段定位子项，再记录档案号和页码。</t>
         </is>
       </c>
     </row>
@@ -18325,7 +18325,7 @@
       </c>
       <c r="J384" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=报纸新闻，题名存在异文。关键词=边区回民代表大会 回民文化促进会 回救边区分会、边区回民代表大会、回民文化促进会、回救边区分会同时开幕、新中华报 1940年10月20日、回救边区分会、回民文化促进会 延安。母项=《新中华报》1940年10月20日、陕甘宁边区回民工作报刊汇编、抗日根据地民族工作文献汇编、陕甘宁边区政府公报及回民救国会资料、中国共产党民族工作史料。候选站=https://books.google.com/books?q=%22%E8%BE%B9%E5%8C%BA%E5%9B%9E%E6%B0%91%E4%BB%A3%E8%A1%A8%E5%A4%A7%E4%BC%9A%22%20%221940%22; https://archive.org/advancedsearch.php?q=%22%E6%96%B0%E4%B8%AD%E5%8D%8E%E6%8A%A5%22%20%221940%22%20%22%E5%9B%9E%E6%B0%91%22&amp;fl%5B%5D=identifier,title&amp;rows=50&amp;page=1&amp;output=json。已知报纸、日期和较可靠异文题名，但未找到可核验的具体版面或扫描页。应优先查1940年10月20日《新中华报》地方版、陕甘宁边区报刊合订本及回民工作史料汇编。</t>
         </is>
       </c>
     </row>
@@ -18371,7 +18371,7 @@
       </c>
       <c r="J385" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=纪念文集收录文章。关键词=怀念我的好领导好老师乌兰夫、怀念我的好领导、好老师乌兰夫、李文精、乌兰夫纪念文集 第一辑、乌兰夫纪念文集 第1辑 第161页。母项=《乌兰夫纪念文集》第1辑、乌兰夫纪念文集。候选站=https://search.douban.com/book/subject_search?search_text=%E4%B9%8C%E5%85%B0%E5%A4%AB%E7%BA%AA%E5%BF%B5%E6%96%87%E9%9B%86&amp;cat=1001。目前只有《乌兰夫纪念文集》第1辑、李文精及约第161页线索，未找到可核验全文页。</t>
         </is>
       </c>
     </row>
@@ -18555,7 +18555,7 @@
       </c>
       <c r="J389" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案公文子项。关键词=关于设置蒙藏回语文选修科、蒙藏回语文、选修科、教育厅、民国教育档案、GD档案 p=507。母项=广东省档案馆相关档案目录、教育行政档案汇编（母项待考）。候选站=http://da.gd.gov.cn/portal_home/archives?archivesType=81&amp;p=507。未能确认该条目所属全宗、年代、文号及案卷页码；应先从档案目录反推母项。</t>
         </is>
       </c>
     </row>
@@ -18601,7 +18601,7 @@
       </c>
       <c r="J390" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古调查简报子项。关键词=铁岭邱台遗址、辽宁铁岭市邱台遗址试掘简报、邱台遗址、铁岭市文物管理办公室、考古 1996 2 36-51、考古 1996 2 101-102。母项=《考古》1996年第2期、《考古》1996年第2期目录及考古发掘简报。候选站=http://www.360doc.com/content/21/0813/22/72341047_990932112.shtml。已确定母项为《考古》1996年第2期，页码为36—51、101—102，但未找到稳定、可核验的期刊全文页。</t>
         </is>
       </c>
     </row>
@@ -18647,7 +18647,7 @@
       </c>
       <c r="J391" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=墓志录文/考释论文子项。关键词=马审章墓志、馬審章墓誌、马审章 墓志 周峰、遼代 馬審章 墓誌、辽金历史与考古 第九辑 第277页。母项=《辽金历史与考古》第九辑、周峰：《辽代〈马审章墓志〉考释》。候选站=https://www.ecsponline.com/goods.php?id=194217。应在《辽金历史与考古》第九辑第277页前后核对论文及墓志录文。未找到公开的独立墓志全文页或可核验录文。</t>
         </is>
       </c>
     </row>
@@ -18693,7 +18693,7 @@
       </c>
       <c r="J392" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古调查报告子项。关键词=喀左大城子城址、辽宁喀左县辽代利州城址的调查、大城子城址、利州城址、于长江、傅宗德。母项=《考古》1996年第8期、《辽宁喀左县辽代利州城址的调查》。候选站=https://www.dpm.org.cn/Uploads/File/2018/06/01/u5b11239fd2b4f.pdf。已反推出母项及作者，但未找到明确对应《考古》1996年第8期的开放全文页。</t>
         </is>
       </c>
     </row>
@@ -18739,7 +18739,7 @@
       </c>
       <c r="J393" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代蒙古地方档案子项。关键词=乾隆二年、扎萨克、来往公文档、下发各扎萨克、乾隆二年蒙古档案、理藩院档案。母项=理藩院档案、清代蒙古档案汇编、内蒙古自治区档案馆蒙古历史档案。候选站=。缺少全宗、案卷号、文种、收藏机构及档案汇编书名，暂不能定位到具体卷页或开放影像。</t>
         </is>
       </c>
     </row>
@@ -18785,7 +18785,7 @@
       </c>
       <c r="J394" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近现代教育行政档案子项。关键词=辽宁省教育厅、教育厅公文、辽宁教育行政档案、教育厅训令、教育厅指令、教育厅函。母项=辽宁省档案馆教育档案、辽宁省教育志资料、民国及新中国初期辽宁教育档案汇编。候选站=。题名为机构性概称，缺少年代、文号、主题及案卷信息，无法确认独立文书或所属档案母项。</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="J395" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案、政务文书或报刊子项。关键词=赈济回民、赈济回族、赈恤回民、救济回民、回民灾赈、赈济。母项=清代或民国赈务档案汇编、地方政府公报、西北回民史料、灾荒史料汇编。候选站=。更像档案题名、报刊栏题或汇编中的条目，不宜按独立书籍检索。应结合地域、年代及所属档案汇编反推母项。</t>
         </is>
       </c>
     </row>
@@ -18877,7 +18877,7 @@
       </c>
       <c r="J396" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊新闻或群众运动档案子项。关键词=安东、纪念七七、十万人签名、拥护毛主席对美声明、对美声明、七七纪念。母项=《安东日报》相关期号、安东市地方报刊、抗美援朝时期安东地方档案汇编。候选站=。可能是1950年代安东地方报刊标题或档案照片说明，缺少日期、报纸名称、版次及馆藏信息，未找到具体期号或影像页。</t>
         </is>
       </c>
     </row>
@@ -18923,7 +18923,7 @@
       </c>
       <c r="J397" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=藏文档案译文子项。关键词=帝师相儿加思法旨、桑杰贝帝师法旨、相儿加思、帝师法旨、大德十一年、西藏社会历史藏文档案资料译文集。母项=《西藏社会历史藏文档案资料译文集》、《西藏社会历史藏文档案资料译文集》第一辑或相关档案卷。候选站=https://book.douban.com/subject/3046017/。母项及译名线索较明确，但未找到该法旨的具体卷次、页码或公开藏文档案影像；“大德十一年”还需核对原档纪年。</t>
         </is>
       </c>
     </row>
@@ -18969,7 +18969,7 @@
       </c>
       <c r="J398" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=图像研究论文或展览图录子项。关键词=六长寿图、六长寿图 汉藏、六长寿图 汉藏文化交融、六长寿图 长寿鹿 猿猴 鹤 乌龟、六长寿图 藏传佛教、六长寿图 壁画 唐卡。母项=藏传佛教唐卡图录、西藏文物展览图录、汉藏美术史研究论文集、西藏寺院壁画或唐卡专题图录。候选站=。未确认到独立出版物、期刊卷期或可核验全文页。应以图像题名、馆藏地、唐卡或壁画母项反查。</t>
         </is>
       </c>
     </row>
@@ -19015,7 +19015,7 @@
       </c>
       <c r="J399" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=文物说明或专题文章子项。关键词=那塘寺、纳塘寺、塔尔寺、菩提伽耶 摩诃菩提寺 木石模型、大明永乐年施、明廷 赏赐 寺院模型。母项=宿白《藏传佛教寺院考古》、宿白西藏佛教寺院与考古研究、西藏佛教寺院文物图录、那塘寺文物调查或寺院建筑调查资料。候选站=。现有线索更像宿白著作中的文物个案标题，尚未确认具体书名卷次或网页章节。应检索“那塘/纳塘”“摩诃菩提寺”“永乐年施”组合。</t>
         </is>
       </c>
     </row>
@@ -19061,7 +19061,7 @@
       </c>
       <c r="J400" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=博物馆藏品说明或《中国民族》专题文章子项。关键词=金城公主进藏图、迎娶金城公主、和亲 金城公主、布画金城公主进藏图、清代 金城公主进藏图 唐卡、张荣德 中国民族 2023 第4期。母项=《中国民族》2023年第4期张荣德相关文章、西藏博物馆藏清代布画金城公主进藏图、西藏博物馆唐卡或民族文物展览图录。候选站=http://www.tibetology.ac.cn/2024-06/18/content_42832615.htm。该页可作为藏品和图像线索；《中国民族》2023年第4期文章应按作者张荣德、期次和栏目继续核对。；2026-09-22 gpt-6-astra：找到候选。类型=博物馆藏品说明或专题文章子项。关键词=金城公主进藏图、迎娶金城公主、清代布画金城公主进藏图、张荣德 中国民族 2023年第4期。母项=西藏博物馆藏清代布画金城公主进藏图、《中国民族》2023年第4期、西藏博物馆唐卡藏品资料。候选站=http://www.tibetology.ac.cn/2024-06/18/content_42832615.htm。该页可核验藏品和图像线索；张荣德发表于《中国民族》2023年第4期的原文仍需按期刊卷期查找。；2026-09-22 gpt-6-astra：找到候选。类型=博物馆藏品说明或专题文章子项。关键词=金城公主进藏图、迎娶金城公主、清代布画金城公主进藏图、张荣德、中国民族 2023年第4期。母项=西藏博物馆藏清代《布画金城公主进藏图》、《中国民族》2023年第4期。候选站=http://www.tibetology.ac.cn/2024-06/18/content_42832615.htm。该页为具体专题文章页；《中国民族》2023年第4期张荣德文章的独立全文页仍未定位。</t>
         </is>
       </c>
     </row>
@@ -19107,7 +19107,7 @@
       </c>
       <c r="J401" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古或古环境研究论文、报告章节。关键词=青藏高原东缘 植物遗存、青藏高原东部 植物遗存、藏区考古 植物遗存、古植物遗存 青藏高原、炭化植物 青藏高原东缘、植物考古 四川西部 青海 西藏。母项=青藏高原考古调查报告、西藏考古学文集、植物考古与环境考古论文集、四川、青海及西藏东缘遗址发掘报告。候选站=。未确认到与该题名完全对应的论文、报告章节或全文页。应补查具体遗址、年代、植物种类及发掘报告题名。</t>
         </is>
       </c>
     </row>
@@ -19153,7 +19153,7 @@
       </c>
       <c r="J402" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案汇编子项。关键词=国民政府 蒙藏委员会 公文、蒙藏委员会 特派、国民政府蒙藏委员会档案、蒙藏委员会委员长公署、蒙藏委员会视察、蒙藏委员会任命 特派。母项=《国民政府蒙藏委员会档案》、《中华民国史档案资料汇编》、国史馆蒙藏委员会档案、西藏问题相关国民政府档案汇编。候选站=。题名明显是档案子项，缺少发文机关、日期、受文机关和档号，暂不能定位具体公文或公开全文。</t>
         </is>
       </c>
     </row>
@@ -19199,7 +19199,7 @@
       </c>
       <c r="J403" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=博物馆藏品说明或玉器图录子项。关键词=青白玉 镂雕 松鼠葡萄纹 山子、青白玉松鼠葡萄纹山子、玉山子 松鼠葡萄纹、清代 玉器 松鼠葡萄、故宫 玉山子 松鼠葡萄。母项=故宫博物院玉器图录、清宫旧藏玉器图录、中国玉器全集、博物馆藏玉器展览图录。候选站=。未确认到该件文物的具体馆藏编号、年代和公开藏品页。应以“松鼠葡萄纹”“山子”及馆藏机构组合检索。</t>
         </is>
       </c>
     </row>
@@ -19245,7 +19245,7 @@
       </c>
       <c r="J404" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=博物馆藏品或图录子项。关键词=珐琅糌粑盒、掐丝珐琅糌粑盒、糌粑盒、藏族珐琅器、珐琅盒、青海民族文物。母项=青海省博物馆藏品图录、民族地区文物图录、中国少数民族文物图录、博物馆展览图录。候选站=。明显可能是藏品名称或图录中的器物条目。应补查收藏机构、藏品编号、年代、材质及图录展览名称。</t>
         </is>
       </c>
     </row>
@@ -19337,7 +19337,7 @@
       </c>
       <c r="J406" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代军机处奏折子项。关键词=喀什噶尔 领队大臣 特克兴额 伊犁 换防 官兵、特克兴额 奏折、喀什噶尔 换防 折。母项=宫中档奏折、军机处录副奏折、清代新疆满汉文奏折汇编、清实录相关条目。候选站=。应按特克兴额、喀什噶尔、伊犁换防及奏折日期反查军机处档案目录；未找到可核验的具体全文页。</t>
         </is>
       </c>
     </row>
@@ -19383,7 +19383,7 @@
       </c>
       <c r="J407" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代行政奏折子项。关键词=新疆 改设州县 满缺 满员 差委、新疆州县 满缺 奏折、请拣发满员。母项=军机处录副奏折、宫中档奏折、清代新疆档案史料、清实录新疆行政建置条目。候选站=。应结合新疆改设州县的年份、奏事官员和具体州县名称定位；未找到具体书页或全文 URL。</t>
         </is>
       </c>
     </row>
@@ -19429,7 +19429,7 @@
       </c>
       <c r="J408" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代宫廷档案或题本子项。关键词=题请核销织办本年新疆需用泽绸用过价脚银两事、新疆需用泽绸、织办 泽绸 价脚银两、内务府织造 新疆 泽绸、清代题本 核销 织办、新疆 泽绸 档案。母项=清代宫中档奏折及军机处档折件、内务府织造档案、清代新疆档案史料汇编、《宫中档乾隆朝奏折》或相关题本汇编。候选站=。题名具有清代档案题名格式，需以年代、具名衙门、档号或档案汇编卷册定位。未找到可核验公开全文页。</t>
         </is>
       </c>
     </row>
@@ -19475,7 +19475,7 @@
       </c>
       <c r="J409" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代吏部题本或题名档案子项。关键词=吏部 为升补 新疆要缺 直隶州知州、升补新疆要缺、新疆要缺 直隶州知州、吏部题本 新疆 知州、清代官员升补 新疆直隶州、吏部铨选新疆官缺。母项=清代吏部题本档案、宫中档奏折及军机处档折件、清代新疆档案史料汇编、新疆建置志及清代官制史料。候选站=。题名可能为档案目录转录标题，缺少年月、官员姓名、具体州名和档号，暂未找到具体卷次或公开全文。</t>
         </is>
       </c>
     </row>
@@ -19521,7 +19521,7 @@
       </c>
       <c r="J410" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代档案子项。关键词=寄谕参赞大臣、扎拉丰阿、科布多旧城、择地建城、安置商民、科布多办事大臣。母项=清宫内阁录副奏折、军机处档案、清代边疆满文档案译编、宫中档乾隆朝奏折。候选站=https://zh.wikisource.org/wiki/清实录。目前只有题名和事项线索，尚不能确定日期、档号及母项卷册。应重点核查乾隆朝《清实录》及内阁录副奏折中的扎拉丰阿条目。</t>
         </is>
       </c>
     </row>
@@ -19567,7 +19567,7 @@
       </c>
       <c r="J411" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=清代土尔扈特档案译文子项。关键词=达色 渥巴锡 游牧地 庙宇 工匠、土尔扈特 修建庙宇、满文土尔扈特档案译编 第140件。母项=《满文土尔扈特档案译编》、中国社会科学院民族研究所、中国第一历史档案馆满文部编，民族出版社，1988年、约第236页第140件。候选站=https://search.worldcat.org/search?q=%E6%BB%A1%E6%96%87%E5%9C%9F%E5%B0%94%E6%89%88%E7%89%B9%E6%A1%A3%E6%A1%88%E8%AF%91%E7%BC%96。已有较明确母项、页码和件号，但未找到公开可核验的具体全文页面；仍属版权期内整理本的书目线索。</t>
         </is>
       </c>
     </row>
@@ -19613,7 +19613,7 @@
       </c>
       <c r="J412" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代军务奏折子项。关键词=靖边大将军 锡保 选派官兵 驼马 巴里坤、锡保 巴里坤 军营、护送驼马 奏折。母项=军机处录副奏折、宫中档奏折、清代准噶尔及新疆档案史料、清实录相关条目。候选站=。应以锡保、靖边大将军、巴里坤及驼马运输组合检索军机处档案目录；未找到具体全文页。</t>
         </is>
       </c>
     </row>
@@ -19659,7 +19659,7 @@
       </c>
       <c r="J413" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=现代考古期刊论文。关键词=山西临猗程村、程村东周墓、临猗县东周墓、赵慧民、李百勤、李春喜。母项=《考古》1991年第11期、《中国考古学年鉴》1991年、山西省文物考古研究所考古调查报告。候选站=https://kns.cnki.net/kns8s/defaultresult/index?kw=%E5%B1%B1%E8%A5%BF%E4%B8%B4%E7%8C%97%E5%8E%BF%E7%A8%8B%E6%9D%91%E4%B8%A4%E5%BA%A7%E4%B8%9C%E5%91%A8%E5%A2%93。已有明确作者、刊名和年期。属于现代期刊论文，不能据此宣称存在公开整本全文。</t>
         </is>
       </c>
     </row>
@@ -19705,7 +19705,7 @@
       </c>
       <c r="J414" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=元代碑刻文献子项。关键词=至大元年十二月、御祭中镇文、祭霍山中镇崇德应灵王祝文、霍山、中镇、洪洞金石录。母项=《洪洞金石录》、《捃古录》卷十八、《山右石刻丛编》、霍山金石文献。候选站=https://www.shidianguji.com/book/CADAL02090592/chapter/1lb3zxs59qj2n; https://zh.wikisource.org/wiki/捃古录。已有识典具体章节 URL；《捃古录》卷十八可作为异本和题名校勘线索。；2026-09-22 gpt-6-astra：找到候选。类型=元代碑刻文献子项。关键词=至大元年、十二月、御祭中镇文、霍山、中镇、崇德应灵王。母项=《洪洞金石录》、《捃古录》卷十八、《山右石刻丛编》。候选站=https://www.shidianguji.com/book/CADAL02090592/chapter/1lb3zxs59qj2n。已取得识典具体章节 URL；《捃古录》卷十八可作异本校勘线索，但未取得对应具体卷页 URL。；2026-09-22 gpt-6-astra：找到候选。类型=元代碑刻文献子项。关键词=至大元年、十二月、御祭中镇文、霍山、中镇、崇德应灵王。母项=《洪洞金石录》、《捃古录》卷十八、《山右石刻丛编》。候选站=https://www.shidianguji.com/book/CADAL02090592/chapter/1lb3zxs59qj2n。已找到识典具体章节页；《捃古录》卷十八目前未找到对应具体卷页 URL。</t>
         </is>
       </c>
     </row>
@@ -19751,7 +19751,7 @@
       </c>
       <c r="J415" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=金石文献子项。关键词=玉泉观记、玉泉观、关中金石记、玉泉观碑、玉泉观碑记。母项=《关中金石记》、关中金石文献、玉泉观碑刻。候选站=https://www.shidianguji.com/book/HY2440/chapter/1kpahqs0pk202。应进一步核对该页的卷次、碑刻所在地、撰书人及版本信息。；2026-09-22 gpt-6-astra：找到候选。类型=金石文献子项。关键词=玉泉观记、玉泉观、玉泉观碑、玉泉观碑记、关中金石记。母项=《关中金石记》、关中金石文献。候选站=https://www.shidianguji.com/book/HY2440/chapter/1kpahqs0pk202。可据该章节页核对卷次、撰者、碑刻地点及底本信息。</t>
         </is>
       </c>
     </row>
@@ -19797,7 +19797,7 @@
       </c>
       <c r="J416" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近现代行政档案子项。关键词=嗣后蒙藏来京学生、蒙藏学生、来京学生、该所、蒙藏院、蒙藏委员会。母项=蒙藏委员会档案、教育部公报、北洋政府公报、国民政府公报、蒙藏院档案汇编。候选站=https://zh.wikisource.org/wiki/政府公报。题名像档案目录摘要，原题可能不是正式标题。“该所”需结合档案上下文确定，暂不能确定年代、机关和档号。</t>
         </is>
       </c>
     </row>
@@ -19843,7 +19843,7 @@
       </c>
       <c r="J417" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=日记、报刊版面或档案子项。关键词=3月27日、三月二十七日、3月27号、三月廿七日、马雨衡。母项=个人日记或工作日记、报刊日期版面、档案文件日期条目、文集中的日记体材料。候选站=。仅有日期，缺少年份、作者、文献类型和地域，无法可靠定位。需要结合相邻条目或母项标题检索。</t>
         </is>
       </c>
     </row>
@@ -19889,7 +19889,7 @@
       </c>
       <c r="J418" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=地方文史资料文章。关键词=回族在翼城的发展及现状、翼城回族、翼城文史资料、宁志远、李滋渔、翼城县民族。母项=《翼城文史资料》第3辑、《翼城文史资料》第4辑、《临汾文史资料》、翼城县志民族宗教志。候选站=https://kns.cnki.net/kns8s/defaultresult/index?kw=%E5%9B%9E%E6%97%8F%E5%9C%A8%E7%BF%BC%E5%9F%8E%E7%9A%84%E5%8F%91%E5%B1%95%E5%8F%8A%E7%8E%B0%E7%8A%B6。已有辑数、作者和约页码，但尚未找到可核验的具体全文页。应向翼城县政协文史资料室、山西省图书馆或地方志馆藏核查。</t>
         </is>
       </c>
     </row>
@@ -19935,7 +19935,7 @@
       </c>
       <c r="J419" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近现代报刊文章或译文子项。关键词=蒙古人对外感情、日本人的势力、蒙古对外感情、日本在蒙古势力、蒙古问题、外蒙 日本。母项=近代中文报刊、《东方杂志》、《蒙藏月报》、《蒙藏旬刊》、《申报》。候选站=https://zh.wikisource.org/wiki/东方杂志。题名缺少作者、刊名和日期，可能是报刊标题、译文标题或档案摘要。暂不能确认母项及具体篇页。</t>
         </is>
       </c>
     </row>
@@ -20211,7 +20211,7 @@
       </c>
       <c r="J425" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=近现代宗教团体行政文件子项。关键词=回教协进会、备案条件、回教协会、中国回教协进会、回民团体备案、宗教团体登记。母项=中国回教协进会档案、内政部公报、蒙藏委员会公报、国民政府公报、近代中国回族社会团体档案汇编。候选站=https://zh.wikisource.org/wiki/国民政府公报。更像公文或档案目录中的主题性标题，需结合年代、发文机关和档案全宗反推正式题名。</t>
         </is>
       </c>
     </row>
@@ -20257,7 +20257,7 @@
       </c>
       <c r="J426" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=清代绘画作品子项。关键词=清 法坤厚、法坤厚 山水轴、坤厚 山水、秋汀渔泊图轴、艺苑掇英 第12辑、山东省博物馆 法坤厚。母项=《艺苑掇英》第12辑、山东省博物馆藏画录、山东省博物馆书画藏品目录、中国古代书画图目。候选站=https://commons.wikimedia.org/w/index.php?search=%E6%B3%95%E5%9D%A4%E5%8E%9A%E7%A7%8B%E6%B1%80%E6%B8%94%E6%B3%8A%E5%9B%BE%E8%BD%B4&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/wiki/艺苑掇英。现有信息将“清法坤厚山水轴”与山东省博物馆藏《秋汀渔泊图轴》相联系，但尚未找到可核验的具体图版页或馆藏记录。</t>
         </is>
       </c>
     </row>
@@ -20395,7 +20395,7 @@
       </c>
       <c r="J429" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊文章、宣传文字或宗教文化子项。关键词=义在清真、清真、伊斯兰教、回族、清真寺、义在清真题名。母项=清真报刊、回族史料汇编、伊斯兰教中国化文献、地方民族宗教资料。候选站=。题名可能是报刊文章、专栏或题辞，尚不能确认是否为独立出版物。应补查年份、报刊名、作者及所属地区。</t>
         </is>
       </c>
     </row>
@@ -20441,7 +20441,7 @@
       </c>
       <c r="J430" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=考古调查或地方民族学论文/报告。关键词=木里县 娃日瓦村 石砌房址、木里 娃日瓦 石砌房、西南夷 民族交往 石砌房址、木里县考古、凉山州考古调查。母项=四川省文物考古研究院或凉山州文物考古调查报告、木里县文物志、凉山彝族自治州文物志、地方考古调查简报或民族学论文集。候选站=。题名语序疑似有录入或识别错误，可能是考古调查报告中的章节或地方文物普查条目。应以“娃日瓦村”“石砌房址”“木里县”组合检索地方志、考古简报和四川省文物考古研究院成果目录。</t>
         </is>
       </c>
     </row>
@@ -20580,7 +20580,7 @@
       </c>
       <c r="J433" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=档案汇编子项。关键词=赵尔丰 电复 武文源 垦丁 可先赴里巴、赵尔丰 武文源、垦务 里塘 巴塘 电文、光绪三十三年五月初六日、清末川滇边务档案史料 上册 第0106件。母项=《清末川滇边务档案史料》上册，中华书局，1989年、四川省民族研究所编辑组编《清末川滇边务档案史料》、约第117页，第0106件，光绪三十三年五月初六日。候选站=https://book.douban.com/subject/20257971/。已能确定母项、册次、日期和档号，但未找到公开逐件全文页面。应按“第0106件”“光绪三十三年五月初六日”向馆藏或纸本核验。</t>
         </is>
       </c>
     </row>
@@ -20626,7 +20626,7 @@
       </c>
       <c r="J434" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=档案汇编子项。关键词=关外学务局 河口学堂 养蚕、河口学堂 试验养蚕、拟拨款置备一切、宣统二年六月初七日、清末川滇边务档案史料 上册 第0629件。母项=《清末川滇边务档案史料》上册，中华书局，1989年、四川省民族研究所编辑组编《清末川滇边务档案史料》、约第682页，第0629件，宣统二年六月初七日。候选站=https://book.douban.com/subject/20257971/。应以“第0629件”“宣统二年六月初七日”“河口学堂”定位纸本或馆藏扫描。未找到公开可直接核验的单件全文。</t>
         </is>
       </c>
     </row>
@@ -20672,7 +20672,7 @@
       </c>
       <c r="J435" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清末边务电报或公文档案子项。关键词=电董令 办理垦务 建官站、赵尔丰 垦务 官站、川边 垦务 官站 电报、边务档案 电董令。母项=《清末川滇边务档案史料》、《赵尔丰边务档案》或四川边务档案汇编、清末川边地方行政档案。候选站=。“董”可能是收文或执行官员姓氏，题名缺少日期、地点和发文者，暂不能可靠反推卷页。应与赵尔丰、川边、垦务、官站组合检索档案目录。</t>
         </is>
       </c>
     </row>
@@ -20718,7 +20718,7 @@
       </c>
       <c r="J436" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代契约或官府执照档案子项。关键词=绥定府 经政厅 朱泽源、屯民 朱泽源 接顶 户口地亩、调管绥庆 军粮屯政、发执照事、王为屯民接顶户口地亩。母项=清代四川地方档案、绥定府衙门档案、四川契约文书或土地文书汇编、清代档案馆藏执照、契约与土地文书。候选站=。题名具有典型清代官府文书格式，可能是档案馆藏单件文书而非出版物。应重点检索“绥定府”“朱泽源”“接顶”“户口地亩”等字段；未找到具体卷册或公开影像页。</t>
         </is>
       </c>
     </row>
@@ -20764,7 +20764,7 @@
       </c>
       <c r="J437" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=民族学调查报告或地方民族志资料。关键词=冯云仙 泸定县 婚姻习俗、泸定县 各民族 婚姻习俗 调查、泸定 婚姻习俗 冯云仙、甘孜民族调查资料。母项=四川省民族研究所民族调查资料、甘孜藏族自治州民族志或民族调查资料汇编、泸定县志、中国少数民族社会历史调查资料丛刊。候选站=。可能为未刊调查报告、内部资料或地方民族志中的章节。题名、作者和收藏单位尚不足以定位具体卷页，未找到公开全文或可靠书目页。</t>
         </is>
       </c>
     </row>
@@ -20810,7 +20810,7 @@
       </c>
       <c r="J438" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=现代研究文章或纪念文集章节。关键词=童小鹏 彝人 红军、童小鹏笔下的彝族、红军长征 彝族 童小鹏、彝人与红军 童小鹏。母项=童小鹏回忆录及文集、红军长征与彝族地区史料汇编、中国工农红军长征文献及回忆资料、现代期刊或纪念文集中的同名文章。候选站=。题名可能是纪念性文章或文集章节，未确认作者、刊物、年份和页码。应检索题名异体“彝族/彝人”及童小鹏文集目录；现代整理本如仍在版权期，只能核对书目或馆藏。</t>
         </is>
       </c>
     </row>
@@ -20856,7 +20856,7 @@
       </c>
       <c r="J439" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=革命回忆录或长征史料文章。关键词=谭尚维 甘孜 藏民 红军、红军医生 谭尚维、谭尚维回忆 甘孜、甘孜地区藏民拥护红军、长征 藏民 拥戴红军 回忆。母项=红军长征回忆史料汇编、四川革命历史档案资料、甘孜藏族自治州革命斗争史料、红军长征亲历者回忆录或党史资料。候选站=。可能是回忆文章标题而非独立出版物，需核对“拥戴/拥护/支持”等题名变体及谭尚维的职务、所在部队和发表刊物。未找到具体卷期、页码或公开全文页面。</t>
         </is>
       </c>
     </row>
@@ -20902,7 +20902,7 @@
       </c>
       <c r="J440" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=论文或地方史专题文章。关键词=全面抗战时期 会理 警团 彝汉交融、全面抗战时期 会理警团、会理县 彝汉关系 抗战、会理 警备团 彝族 汉族。母项=凉山彝族地方史资料、四川省志·民族志、会理县志、凉山州文史资料、抗战时期四川地方武装及民族关系研究论文集。候选站=https://www.google.com/search?q=%E5%85%A8%E9%9D%A2%E6%8A%97%E6%88%98%E6%97%B6%E6%9C%9F+%E4%BC%9A%E7%90%86+%E8%AD%A6%E5%9B%A2+%E5%BD%9D%E6%B1%89%E4%BA%A4%E8%9E%8D。题名更像论文或地方文史资料中的章节，不能按独立图书处理。应重点核对《会理县志》、凉山州文史资料及四川民族地区抗战史论文集的目录和索引。</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="J441" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地方史文章或方志章节。关键词=道孚县 汉藏团练、道孚 团练、道孚 汉藏关系、炉霍 道孚 康定 团练。母项=道孚县志、甘孜州志、四川省志·军事志、四川省志·民族志、甘孜州文史资料。候选站=https://www.google.com/search?q=%E9%81%93%E5%AD%9A%E5%8E%BF+%E6%B1%89%E8%97%8F%E5%9B%A2%E7%BB%83。“汉藏团练”很可能是《道孚县志》或甘孜州地方文史资料中的子标题，需以方志目录、正文关键词和页码反查。</t>
         </is>
       </c>
     </row>
@@ -21040,7 +21040,7 @@
       </c>
       <c r="J443" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=论文。关键词=浅析兴隆洼文化与其他考古学文化的关系、兴隆洼文化 其他考古学文化、兴隆洼文化 边疆考古研究 第十辑、边疆考古研究 2011 第10辑。母项=《边疆考古研究》第10辑、《边疆考古研究》、兴隆洼文化考古论文集。候选站=http://www.queshu.com/book/10138048/; https://search.douban.com/book/subject_search?search_text=%E8%BE%B9%E7%96%86%E8%80%83%E5%8F%A4%E7%A0%94%E7%A9%B6%E7%AC%AC10%E8%BE%91。已知母项为科学出版社2011年《边疆考古研究》第10辑，ISBN 9787030329240。现代学术论文集仍受版权和馆藏访问限制，未找到可核验的开放全文页。</t>
         </is>
       </c>
     </row>
@@ -21132,7 +21132,7 @@
       </c>
       <c r="J445" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=考古调查或文物志条目。关键词=下南滩遗址、南滩遗址、武川县下南滩、内蒙古魏晋北朝考古、武川县文物志。母项=《内蒙古魏晋北朝考古综述》、《草原文物》2019年第1期、《武川县文物志》、内蒙古文物考古调查报告。候选站=https://ygx.sxu.edu.cn/db/%E6%9C%9F%E5%88%8A/nmgwwkg/nmgw2019/1901pdf/190107.pdf。该条目更可能是综述或《武川县文物志》中的遗址条目，不是独立著作。应在PDF内检索“下南滩”，并记录原始发掘报告或文物志的卷页信息。；2026-09-22 gpt-6-astra：找到候选。类型=考古调查或文物志条目。关键词=下南滩遗址、南滩遗址、武川县下南滩、内蒙古魏晋北朝考古。母项=《内蒙古魏晋北朝考古综述》、《草原文物》2019年第1期、《武川县文物志》。候选站=https://ygx.sxu.edu.cn/db/%E6%9C%9F%E5%88%8A/nmgwwkg/nmgw2019/1901pdf/190107.pdf。该PDF为综述文章全文，未确认其中是否包含独立的遗址条目或原始发掘报告全文。</t>
         </is>
       </c>
     </row>
@@ -21270,7 +21270,7 @@
       </c>
       <c r="J448" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代蒙古盟旗档案子项。关键词=盟长 敖汉额驸 册封格格 翁牛特、敖汉额驸 翁牛特札萨克郡王、册封格格 札、翁牛特 盟长 档案。母项=清代内蒙古东部盟旗档案汇编、翁牛特旗档案、昭乌达盟盟旗档案、内蒙古历史档案、清代蒙古档案史料汇编。候选站=https://www.google.com/search?q=%E7%9B%9F%E9%95%BF+%E6%95%96%E6%B1%89%E9%A2%9D%E9%A9%B8+%E5%86%8C%E5%B0%81%E6%A0%BC%E6%A0%BC+%E7%BF%81%E7%89%9B%E7%89%B9。题名格式明显属于档案汇编中的单件公文，需先确定馆藏机构、档案全宗和汇编名称，再按盟旗、人物和文书类型定位。</t>
         </is>
       </c>
     </row>
@@ -21316,7 +21316,7 @@
       </c>
       <c r="J449" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代地方军政奏折子项。关键词=黑龙江将军 奕山 挑选官兵 候调、奕山 黑龙江官兵、黑龙江将军奏折。母项=军机处录副奏折、黑龙江将军衙门档案、清代黑龙江档案史料、清实录咸丰朝相关条目。候选站=。应补充奏折日期或调兵背景后检索黑龙江将军衙门档案；未找到可核验具体页。</t>
         </is>
       </c>
     </row>
@@ -21362,7 +21362,7 @@
       </c>
       <c r="J450" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代盐务行政奏折子项。关键词=吉兰泰 盐课 银数 不敷 追赔、吉兰泰盐务 奏折、盐课亏短 分别追赔。母项=军机处录副奏折、清代盐务档案、河东盐政及西北盐务档案、清实录相关盐务条目。候选站=。吉兰泰可能涉及盐政、理藩院或地方财政档案；缺少年代和具名官员，未找到具体全文页。</t>
         </is>
       </c>
     </row>
@@ -21408,7 +21408,7 @@
       </c>
       <c r="J451" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=清代蒙古盟旗档案子项。关键词=翁牛特 甲喇菱格 张永生 诬告、盟摄政协理 翁牛特札萨克、原盟警备军 札萨克郡王、甲喇菱格 档案。母项=翁牛特旗档案汇编、昭乌达盟盟旗档案、清代内蒙古盟旗司法档案、内蒙古历史档案史料汇编。候选站=https://www.google.com/search?q=%E7%BF%81%E7%89%9B%E7%89%B9+%E7%94%B2%E5%96%87%E8%8F%B1%E6%A0%BC+%E5%BC%A0%E6%B0%B8%E7%94%9F+%E8%AF%AC%E5%91%8A。这是档案单件标题，存在满文转写、汉字异体和断句差异的可能，需结合翁牛特旗档案全宗及清代盟旗司法文书目录检索。</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       </c>
       <c r="J452" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=革命历史电报档案子项。关键词=贺龙 肖克 关向应 周士第 甘泗淇 李井泉 1938年10月13日、大青山根据地 应向铁道以南发展、大青山抗日游击根据地资料选编 上册 历史档案、晋绥抗日根据地 电报。母项=《大青山抗日游击根据地资料选编》上册·历史档案部分、晋绥抗日根据地史料、八路军一二〇师抗战史料、中国人民解放军历史资料丛书相关卷。候选站=https://www.google.com/search?q=%E5%A4%A7%E9%9D%92%E5%B1%B1%E6%8A%97%E6%97%A5%E6%B8%B8%E5%87%BB%E6%A0%B9%E6%8D%AE%E5%9C%B0%E8%B5%84%E6%96%99%E9%80%89%E7%BC%96+%E8%B4%BA%E9%BE%99+%E8%82%96%E5%85%8B+1938%E5%B9%B410%E6%9C%8813%E6%97%A5。母项和约页码已由清单提供，但未找到可核验的开放全文或具体数字化页。应按上册“历史档案部分”、1938年10月13日及发电者组合检索。</t>
         </is>
       </c>
     </row>
@@ -21500,7 +21500,7 @@
       </c>
       <c r="J453" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊或时事资料子项。关键词=1943年12月26日 北方鳞爪、北方鳞爪 1943、北方鳞爪 民国报刊、北方鳞爪 12月26日。母项=民国时期北方报刊、抗战时期华北报刊、北方地区新闻资料汇编、民国报刊影印资料。候选站=https://www.google.com/search?q=%221943%E5%B9%B412%E6%9C%8826%E6%97%A5%22+%22%E5%8C%97%E6%96%B9%E9%B3%9E%E7%88%AA%22。“北方鳞爪”可能是栏目名或剪报标题，不能据题名判断为独立出版物。需补充报刊名称、出版地或收藏档案母项。</t>
         </is>
       </c>
     </row>
@@ -21546,7 +21546,7 @@
       </c>
       <c r="J454" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊新闻或通讯社电讯子项。关键词=1947年6月10日 救济察北蒙旗赈款四亿、救济察北蒙旗 赈款四亿、察北蒙旗 急赈 合作 两亿、1947 察北 蒙旗 救济。母项=1947年民国报刊、察哈尔省地方新闻资料、绥远及察北蒙旗社会救济档案、解放战争时期报刊资料汇编、民国时期通讯社电讯汇编。候选站=https://www.google.com/search?q=%221947%E5%B9%B46%E6%9C%8810%E6%97%A5%22+%22%E6%95%91%E6%B5%8E%E5%AF%9F%E5%8C%97%E8%92%99%E6%97%97%22。标题格式接近报刊新闻标题，金额“四亿”可能为法币旧额。应以1947年6月10日前后察哈尔、北平、绥远地区报刊及通讯社资料的日期索引反查。</t>
         </is>
       </c>
     </row>
@@ -21592,7 +21592,7 @@
       </c>
       <c r="J455" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊子项。关键词=姚锡光、蒙人之感情、1912年8月21日、民国报刊、蒙古问题。母项=民国报刊合订本、有关蒙古问题的报刊资料汇编、姚锡光文集或政论集。候选站=。未能核定刊名、卷期及具体页码。应以日期、作者和“蒙人”“感情”等词在1912年报刊数据库及地方文史资料中反查。</t>
         </is>
       </c>
     </row>
@@ -21638,7 +21638,7 @@
       </c>
       <c r="J456" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=疑似民国时期行政机构资料或研究条目，非独立书籍。关键词=兴安省政府、興安省政府、兴安省公署、興安省公署、兴安省政府公报、兴安省政府档案。母项=《满洲国政府公报》及其地方机关公报、《满洲国史》有关兴安省行政建置章节、民国及伪满洲国政府档案汇编中的兴安省行政档案、东北地方志、蒙旗志及兴安地区县旗志。候选站=https://zh.wikisource.org/wiki/Special:%E6%90%9C%E7%B4%A2?search=%E8%88%88%E5%AE%89%E7%9C%81%E6%94%BF%E5%BA%9C; https://commons.wikimedia.org/w/index.php?search=%E8%88%88%E5%AE%89%E7%9C%81%E6%94%BF%E5%BA%9C&amp;title=Special:MediaSearch&amp;type=image。未确认《兴安省政府》作为独立书名、期刊名或可定位的档案汇编子项。建议以1932—1945年兴安省、兴安总省及各旗县公署为时间与机构线索，进一步核查《满洲国政府公报》、东北地方志和伪满档案目录；目前没有可核验的具体卷次或全文页。</t>
         </is>
       </c>
     </row>
@@ -21684,7 +21684,7 @@
       </c>
       <c r="J457" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=地方史料论文或史料条目。关键词=包头蒙民、出租地、蒙租、来历及其演变、巴靖远、包头史料荟要。母项=《包头史料荟要》第3辑、包头市地方志史编修办公室编地方史料、包头地方文史资料。候选站=。已有母项、作者和约页码线索：巴靖远，《包头史料荟要》第3辑，约第131页；但未找到可核验的具体全文页或扫描页。</t>
         </is>
       </c>
     </row>
@@ -21730,7 +21730,7 @@
       </c>
       <c r="J458" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊子项。关键词=满蒙学校、学校之合并、1912年7月4日、满蒙教育、民国报刊。母项=1912年报刊合订本、民国教育报刊、满蒙问题档案汇编、教育部公报。候选站=。未能核定刊名、作者、卷期及页码。日期应作为首要定位条件，并结合“满蒙学校”“并合”“教育”等异体词检索。</t>
         </is>
       </c>
     </row>
@@ -21776,7 +21776,7 @@
       </c>
       <c r="J459" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=博物馆藏品条目。关键词=战国、西汉、束腰铜扁盒、保山市博物馆、昌宁、田园镇。母项=保山市博物馆藏品数据库、保山市博物馆出土文物资料、昌宁田园镇卡巴洼山出土文物记录。候选站=https://www.jinshasitemuseum.com/seardetail/4123。已有具体藏品详情页，但该页属于单件文物记录，不能替代相关图录或考古报告全文。；2026-09-22 gpt-6-astra：找到候选。类型=博物馆藏品条目。关键词=战国、西汉、束腰铜扁盒、保山市博物馆、昌宁、田园镇。母项=保山市博物馆藏品数据库、昌宁田园镇卡巴洼山出土文物资料、保山市博物馆藏品图录。候选站=https://www.jinshasitemuseum.com/seardetail/4123。已找到具体藏品页；该页不是考古报告或图录全文。</t>
         </is>
       </c>
     </row>
@@ -21822,7 +21822,7 @@
       </c>
       <c r="J460" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=档案子项。关键词=龙云、勉励所、相关公文、云南档案、抗战时期、公文。母项=龙云档案汇编、云南省档案馆馆藏龙云档案、云南省政府公报、西南边疆档案资料。候选站=。“勉励所”可能为机构名、教育或生产组织名称，也可能是题名截取，暂不能据此确定档案全题名、档号或汇编卷次。</t>
         </is>
       </c>
     </row>
@@ -21868,7 +21868,7 @@
       </c>
       <c r="J461" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊连载子项。关键词=滇缅公路、沿线蚕桑事业、视察记、续完、云南蚕桑、抗战时期报刊。母项=抗战时期云南报刊、蚕桑或农业专业期刊、云南省政府公报、滇缅公路建设及经济资料汇编。候选站=。“续完”表明前有连载，需先确定首篇题名、刊名和刊期，再按“续”“续完”追踪；目前未找到具体期刊年期或全文页。</t>
         </is>
       </c>
     </row>
@@ -21914,7 +21914,7 @@
       </c>
       <c r="J462" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=教育论述或报刊论文。关键词=边地民族教育、教材之编制、民族教育教材、边疆教育、民国教育。母项=民国教育期刊、边疆教育资料汇编、教育部边疆教育档案、西南边疆教育文献。候选站=。未能确定作者、刊名、发表时间和页码；题名可能存在“编制”与“编辑”等异文，应并行检索。</t>
         </is>
       </c>
     </row>
@@ -22006,7 +22006,7 @@
       </c>
       <c r="J464" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=清代档案子项。关键词=三姓副都统、明英、貂皮商人、过卡执照、咨吉林将军衙门、乾隆四十五年。母项=《三姓副都统衙门满文档案译编》、《三姓副都统衙门满文档案译编》约第393页第133件、清代吉林将军衙门档案、三姓副都统衙门满文档案。候选站=https://book.douban.com/subject/10830719/。母项、档案件号、日期和约页码均已有线索；现有链接仅为书目页，未找到该第133件的公开全文或具体数字化页。</t>
         </is>
       </c>
     </row>
@@ -22052,7 +22052,7 @@
       </c>
       <c r="J465" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=现代民族学普及或研究专著，属于“走近中国少数民族丛书”子项。关键词=达斡尔族、達斡爾族、毅松 达斡尔族、走近中国少数民族丛书 达斡尔族、9787549702244、辽宁民族出版社 2012。母项=《走近中国少数民族丛书》、辽宁民族出版社2012年版丛书、达斡尔族民族志、地方史及非物质文化遗产资料。候选站=https://book.douban.com/subject/10812811/; https://search.worldcat.org/search?q=bn%3A9787549702244。已确认存在2012年辽宁民族出版社版，但该书仍属现代出版物，不能据此宣称有公开整本全文下载。建议按ISBN、作者“毅松”、丛书名及辽宁民族出版社馆藏记录检索；可继续查找章节目录、图书馆馆藏和引用该书的论文。</t>
         </is>
       </c>
     </row>
@@ -22098,7 +22098,7 @@
       </c>
       <c r="J466" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：仅线索。类型=近代报刊文章或栏目子项。关键词=考政大臣 陈奏 廷臣会议 立宪、宪政初纲 立宪纪闻、东方杂志 1906 临时增刊。母项=《东方杂志》1906年临时增刊《宪政初纲》、《东方杂志》立宪纪闻栏、晚清宪政史料汇编。候选站=https://search.worldcat.org/search?q=%E4%B8%9C%E6%96%B9%E6%9D%82%E5%BF%97+1906+%E5%AE%AA%E6%94%BF%E5%88%9D%E7%BA%B2。已知母项、年份和栏目，但未找到该临时增刊的具体公开扫描页；现代数据库收录情况需按馆藏或报刊数据库核验。</t>
         </is>
       </c>
     </row>
@@ -22144,7 +22144,7 @@
       </c>
       <c r="J467" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=报刊文章子项。关键词=林冰 西南公路 筑柳段、严拿偷漏、旅行杂志 筑柳段、筑柳公路、抗战贵州文录 第七辑。母项=《旅行杂志》、《民国贵州文献大系》第七辑《抗战贵州文录》、《民国贵州文献大系》。候选站=。应先按《旅行杂志》逐年检索林冰所作《西南公路——筑柳段》，再核对《民国贵州文献大系》第七辑的篇目或影印页；当前未找到可核验的具体卷期或全文页。</t>
         </is>
       </c>
     </row>
@@ -22190,7 +22190,7 @@
       </c>
       <c r="J468" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：找到候选。类型=博物馆藏品图录子项。关键词=汉代 赫章 可乐 带冠璧形玉玦、赫章可乐 M341、带冠璧形玉玦、贵州文物精华。母项=《贵州文物精华》、赫章可乐墓群发掘资料、赫章可乐M341出土文物图录。候选站=https://www.gzmuseum.com/gbxs/202210/481.html。该条更可能是《贵州文物精华》中的图录条目，而非独立出版物；还需从页面或图录目录确认页码、器物编号及M341的完整考古报告出处。</t>
         </is>
       </c>
     </row>
@@ -22236,7 +22236,7 @@
       </c>
       <c r="J469" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-22 gpt-6-astra：未找到。类型=碑刻或地方文献子项。关键词=天柱县 万历二十八年 置学田记、明万历二十八年 置学田、天柱 学田碑、天柱县碑刻、贵州金石志。母项=《天柱县志》、贵州地方金石资料、天柱县文物志或碑刻录。候选站=。应重点核查《天柱县志》学校、书院、田赋及金石门，以及贵州省地方志和碑刻汇编；当前未找到具体卷页、录文或可核验全文URL。</t>
         </is>
       </c>
     </row>
@@ -22335,7 +22335,7 @@
       </c>
       <c r="J472" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：仅线索。类型=方志。关键词=和平县志、和平縣志、和平县志 民国三十二年、和平縣志 民國三十二年、1943 和平县志、康熙 和平县志。母项=广东地方志、岭南方志、中国地方志联合目录、广东省立中山图书馆地方志馆藏。候选站=https://zh.wikisource.org/; https://www.nlc.cn/; https://www.library.gd.cn/。应按康熙、乾隆、民国三种版本分别检索，并追查卷首、序跋和目录中的异题。未找到可核验的公开全文。 人工核验：目标本为民国三十二年铅印本（曾枢修、凌开蔚纂，二十卷）；康熙/乾隆本另见书目，公开全文仍未取得。；2026-09-21 gpt-6-astra：未找到。类型=地方志。关键词=和平县志 曾枢 凌开蔚、和平縣志 曾樞 凌開蔚、和平縣志 民國三十二年 二十卷、和平县志 1943 铅印本、和平縣志 卷首 目錄、和平縣志 康熙 乾隆。母项=。候选站=。目标据用户人工核验为曾枢修、凌开蔚纂，民国三十二年铅印二十卷本。当前无法联网核验，未取得该版本的具体卷页URL。康熙、乾隆本须另行辨版，不能作为1943年本的全文替代；所给广东省立中山图书馆馆藏信息未在本轮独立复核。；2026-09-21 gpt-6-astra：未找到。类型=方志。关键词=和平县志、和平縣志、民国三十二年和平县志、1943和平县志、曾枢、凌开蔚。母项=广东地方志、岭南方志、广东省立中山图书馆地方志馆藏。候选站=。未找到可核验的维基文库卷次URL。民国三十二年本与康熙、乾隆本的版本关系亦未能在本轮公开页面中核实。</t>
         </is>
       </c>
     </row>
@@ -22472,7 +22472,7 @@
       </c>
       <c r="J474" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：仅线索。类型=出土文献整理本。关键词=岳麓书院藏秦简 肆、岳麓书院藏秦简（肆）、嶽麓書院藏秦簡 肆、岳麓秦简 第四册、岳麓书院藏秦简 第四卷、上海辞书出版社 2015。母项=岳麓书院藏秦简、岳麓书院藏秦简编纂委员会整理本、战国秦汉简帛文献。候选站=https://www.nlc.cn/; https://www.cadal.edu.cn/; https://www.library.sh.cn/。2015年整理本仍在版权期，通常只能取得书目、馆藏或馆内阅览信息，不应预期公开整本下载。；2026-09-21 gpt-6-astra：未找到。类型=现代出土文献整理本。关键词=岳麓书院藏秦简 肆 2015 上海辞书出版社、嶽麓書院藏秦簡 肆、岳麓书院藏秦简 第四册 目录、岳麓秦简 肆 简号 释文。母项=《岳麓书院藏秦简》整理出版系列。候选站=。据所给信息为2015年12月上海辞书出版社整理本，仍在版权期，不可整本下载；仅可提供书目、馆藏或相关研究DOI线索。当前无法联网核验，也未取得符合本轮限定的具体页面URL。若定位单条材料，应补充简号或释文首句；先秦原简与现代整理成果须分别辨识。；2026-09-21 gpt-6-astra：未找到。类型=现代出土文献整理本。关键词=岳麓书院藏秦简 肆、嶽麓書院藏秦簡 肆、岳麓秦简 第四册、上海辞书出版社 2015。母项=《岳麓书院藏秦简》整理系列、战国秦汉简帛文献。候选站=。未取得符合限定的具体章节或公开全文URL。2015年整理本仍属版权期，宜查馆藏、目录或单条简号研究资料。</t>
         </is>
       </c>
     </row>
@@ -22518,7 +22518,7 @@
       </c>
       <c r="J475" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：仅线索。类型=近代报刊。关键词=时报、時報、上海时报、上海時報、时报 1904、时报 1939。母项=全国报刊索引、中国近代报刊数据库、民国日报刊、上海近代报刊。候选站=https://www.cnbksy.com/; https://www.nlc.cn/; https://www.library.sh.cn/。应以刊名加具体日期、版次、文章题名或作者定位。公开可核验全文未找到；部分数据库需要机构订阅。；2026-09-21 gpt-6-astra：未找到。类型=近代报刊。关键词=时报、時報、上海时报、上海時報、1904 时报、1939 时报。母项=《全国报刊索引》、中国近代报刊数据库、上海近代报刊。候选站=。刊物本身已有出版时段线索，但未核到可公开访问的具体日期、版次或文章页面。</t>
         </is>
       </c>
     </row>
@@ -22610,7 +22610,7 @@
       </c>
       <c r="J477" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=档案文献母项或未具名子项。关键词=总政治部 公文、總政治部 公文、总政治部文件、總政治部文件、总政治部训令、总政治部通令。母项=中国人民解放军总政治部档案、革命历史档案资料、中央革命根据地文件汇编、红军政治工作史料。候选站=https://www.nlc.cn/; https://www.cadal.edu.cn/; https://zh.wikisource.org/。题名过于概括，可能是档案母项下的单件公文。需要补充年代、发布机关层级、文号、收文单位或引用该公文的文章。；2026-09-21 gpt-6-astra：未找到。类型=未具名档案集合或公文泛称。关键词=总政治部 公文 训令 通令、總政治部 公文 訓令 通令、红军 总政治部 文件 文号、总政治部 政治工作 史料 目录。母项=《中央革命根据地历史资料文库》（候查，须先确认年代及机关）、红军政治工作史料汇编（具体书名及收录关系待核）。候选站=。无法联网核验，未取得对应公文的具体章节URL。该名称不具备唯一文献识别性，且不能仅凭“总政治部”确定所属政权、军队或时期。应先从引用出处提取发文机关全称、日期、文号、事由及收文对象，再定位汇编目录和页码。；2026-09-21 gpt-6-astra：未找到。类型=档案公文。关键词=总政治部公文、總政治部公文、总政治部文件、总政治部训令、总政治部通令。母项=革命历史档案资料汇编、红军政治工作史料、中央革命根据地文件汇编。候选站=。题名不是唯一文献名称，缺少政权或军队归属、年代、文号、收文单位及公文事由，无法定位卷次或具体档案页。</t>
         </is>
       </c>
     </row>
@@ -22656,7 +22656,7 @@
       </c>
       <c r="J478" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=文章、工作报告或内部资料。关键词=服务瑶山的经验、服務瑤山的經驗、服务瑶山经验、服务瑶山的经验 材料、瑶山 工作经验、瑶山 民族工作。母项=瑶族社会历史调查、民族地区工作文献、民族工作文件汇编、广东或广西瑶山地方史料。候选站=https://www.nlc.cn/; https://www.cadal.edu.cn/; https://zh.wikisource.org/。未找到可核验的独立出版物。应将题名作为篇名，在瑶族调查、民族工作报告和地方文史资料中查找。；2026-09-21 gpt-6-astra：未找到。类型=疑似工作报告或文章。关键词=服务瑶山的经验、服務瑤山的經驗、服务瑶山经验、瑶山 民族工作 报告。母项=瑶族社会历史调查资料（待核）、民族工作报告汇编（待核）。候选站=。本轮无法调用联网检索工具，未能完成新的在线检索或页面核验；以下各项“未找到”仅表示没有可提供的新增已核验具体页面，不表示已检索穷尽。本项作者、年代、载体均未确定，题名变体不是已确认别名。；2026-09-21 gpt-6-astra：未找到。类型=文章或工作报告。关键词=服务瑶山的经验、服務瑤山的經驗、服务瑶山经验、瑶山民族工作、瑶族工作经验。母项=瑶族社会历史调查资料、民族工作文件汇编、广东或广西瑶山地方史料。候选站=。缺少作者、年代、刊名或编印机关，未能确认具体报刊篇页、文集章节或档案条目。</t>
         </is>
       </c>
     </row>
@@ -22733,7 +22733,7 @@
       </c>
       <c r="G480" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H480" s="10" t="inlineStr">
@@ -22743,12 +22743,12 @@
       </c>
       <c r="I480" s="10" t="inlineStr">
         <is>
-          <t>清光绪二十年(1894)刻本,4卷;彭洵纂</t>
+          <t>清光绪二十年(1894)刻本,4卷;彭洵纂。识典古籍另析为5卷（含目录/拾遗卷）。</t>
         </is>
       </c>
       <c r="J480" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 识典古籍全文已按卷提取；母项为《灌记初稿》。</t>
         </is>
       </c>
     </row>
@@ -22841,7 +22841,7 @@
       </c>
       <c r="J482" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=期刊、文章或教育工作资料。关键词=边地教育、邊地教育、边疆教育、邊疆教育、边地教育 论文、边地教育 报告。母项=民国教育期刊、边疆教育史料、民族地区教育文献、边疆问题研究期刊。候选站=https://www.nlc.cn/; https://www.cadal.edu.cn/; https://archive.org/。题名可能是文章名或期刊栏目名。应加入作者、刊名、年份、地区和关键词组合检索，不能按独立书籍处理。；2026-09-21 gpt-6-astra：未找到。类型=期刊文章、教育资料或栏目。关键词=边地教育、邊地教育、边疆教育、邊疆教育、边地教育史料。母项=民国教育期刊、边疆教育史料、民族地区教育文献。候选站=。题名过于通用，未核到作者、刊名、年份、卷期或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -22933,7 +22933,7 @@
       </c>
       <c r="J484" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：仅线索。类型=考古发掘报告或专题文章。关键词=绥德黄家塔墓、綏德黃家塔墓、绥德黄家塔汉墓、綏德黃家塔漢墓、黄家塔墓群、黃家塔墓群。母项=《绥德汉代画像石》、陕西考古报告、汉代画像石资料汇编、陕西省文物考古研究院发掘报告。候选站=https://www.nlc.cn/; https://www.cadal.edu.cn/; https://commons.wikimedia.org/。更可能是《绥德汉代画像石》中的章节、图版说明或考古简报，不宜视为独立书名。2001年相关专著通常只能查馆藏或部分章节。；2026-09-21 gpt-6-astra：未找到。类型=疑似考古报告或图录子项。关键词=绥德黄家塔墓、綏德黃家塔墓、绥德黄家塔汉墓、黃家塔 漢畫像石、绥德汉代画像石 2001 黄家塔。母项=《绥德汉代画像石》（2001年，关联待核）、陕西汉画像石考古报告（待核）。候选站=。未能核验黄家塔墓对应的章节、墓号、图版号或具体页面。所给2001年专著仅作既有书目线索，不可据此提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘报告或图录条目。关键词=绥德黄家塔墓、綏德黃家塔墓、绥德黄家塔汉墓、黄家塔墓群、绥德汉代画像石 黄家塔。母项=《绥德汉代画像石》、陕西汉代画像石考古资料、陕西考古发掘报告。候选站=。未取得黄家塔墓对应的具体章节、墓号、图版说明或公开录文页。相关2001年图录或专著仅可作馆藏线索。</t>
         </is>
       </c>
     </row>
@@ -23025,7 +23025,7 @@
       </c>
       <c r="J486" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=文章、演讲或政治宣传资料。关键词=中华民族的崇高精神、中華民族的崇高精神、中华民族崇高精神、中华民族的崇高精神 演讲、中华民族的崇高精神 文章、中华民族的崇高精神 报刊。母项=近现代思想政治文献、民族团结宣传资料、报刊文章汇编、演讲稿与时论资料。候选站=https://www.nlc.cn/; https://zh.wikisource.org/; https://www.cadal.edu.cn/。题名缺少作者、年代和载体信息，可能只是文章或演讲标题。应以标题变体加报刊、民族团结、演讲等母项检索。；2026-09-21 gpt-6-astra：未找到。类型=疑似文章或演讲稿。关键词=中华民族的崇高精神、中華民族的崇高精神、中华民族崇高精神、中華民族 崇高精神 演講 報刊。母项=近现代报刊或演讲集（载体待核）。候选站=。缺少作者、发表年代及刊名，无法确定作品身份；没有新增可核验的维基文库卷次或其他指定类型页面。；2026-09-21 gpt-6-astra：未找到。类型=文章、演讲或报刊资料。关键词=中华民族的崇高精神、中華民族的崇高精神、中华民族崇高精神、中华民族的崇高精神 演讲。母项=近现代报刊、民族团结宣传资料、演讲稿汇编、思想政治文献。候选站=。缺少作者、发表时间及载体，无法确认维基文库篇名、报刊卷期或文集章节。</t>
         </is>
       </c>
     </row>
@@ -23071,7 +23071,7 @@
       </c>
       <c r="J487" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古发掘报告或考古简报。关键词=安徽潜山彭岭战国西汉墓、安徽潛山彭嶺戰國西漢墓、潜山彭岭墓、潛山彭嶺墓、彭岭战国墓、彭岭西汉墓。母项=安徽考古、安徽文物考古文献、中国考古学年鉴、考古发掘简报汇编。候选站=https://www.nlc.cn/; https://www.cadal.edu.cn/; https://commons.wikimedia.org/。可能是《文物》或地方考古刊物中的发掘简报，而非独立出版物。应补查“彭岭”“潜山”“战国墓”“西汉墓”的组合。 人工核验：安徽省文物考古研究所、潜山县文物管理所《安徽潜山彭岭战国西汉墓》，《考古学报》2006年第2期。现代期刊，未取得可公开全文。；2026-09-21 gpt-6-astra：未找到。类型=现代期刊考古报告。关键词=安徽潜山彭岭战国西汉墓、安徽潛山彭嶺戰國西漢墓、安徽省文物考古研究所 潜山县文物管理所 彭岭、考古学报 2006 第2期 彭岭。母项=《考古学报》2006年第2期（据用户提供的人工核验记录）。候选站=。据既有人工核验记录，作者为安徽省文物考古研究所、潜山县文物管理所。未新增核验页码、DOI或具体页面。现代期刊仅保留书目线索，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=现代考古期刊发掘报告。关键词=安徽潜山彭岭战国西汉墓、安徽潛山彭嶺戰國西漢墓、潜山彭岭墓、彭岭战国墓、彭岭西汉墓。母项=《考古学报》2006年第2期、安徽考古、安徽省文物考古研究所考古报告。候选站=。已有刊名、年份及期号线索，但未取得可核验的具体文章页面、DOI或公开全文URL。现代期刊仅提供书目线索。</t>
         </is>
       </c>
     </row>
@@ -23117,7 +23117,7 @@
       </c>
       <c r="J488" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=器物专题文章、图录条目或青铜器研究。关键词=方鼎、方鼎 青铜器、方鼎 出土、方鼎 铭文、方鼎 图录、方鼎 博物馆。母项=中国青铜器全集、中国出土青铜器全集、殷周金文集成、博物馆青铜器图录、考古学报及文物期刊。候选站=https://zh.wikisource.org/; https://ctext.org/; https://www.nlc.cn/。“方鼎”是通用器名，无法据此确认具体条目。需要补充时代、出土地、藏馆、器主、铭文或原始刊物信息。；2026-09-21 gpt-6-astra：未找到。类型=青铜器专题文章、器物图录条目或铭文研究。关键词=方鼎、方鼎 青铜器、方鼎 铭文、方鼎 出土、方鼎 博物馆。母项=《中国青铜器全集》、《中国出土青铜器全集》、《殷周金文集成》、博物馆青铜器图录。候选站=。“方鼎”为通用器名，未能据此确定时代、出土地、器主、藏馆或原始刊物。</t>
         </is>
       </c>
     </row>
@@ -23190,12 +23190,12 @@
       </c>
       <c r="F490" s="10" t="inlineStr">
         <is>
-          <t>https://www.gxhj.com/png/259625vchg/</t>
+          <t>https://www.shidianguji.com/book/NLG312001065669</t>
         </is>
       </c>
       <c r="G490" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H490" s="10" t="inlineStr">
@@ -23205,12 +23205,12 @@
       </c>
       <c r="I490" s="10" t="inlineStr">
         <is>
-          <t>清道光二十一年(1841)刻本,50卷;李熙龄纂修</t>
+          <t>清道光二十一年(1841)刻本,50卷;李熙龄纂修。识典古籍转录本。</t>
         </is>
       </c>
       <c r="J490" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 识典古籍全文已按目录卷次提取。原表 gxhj 链接无效，已替换为可核原文。</t>
         </is>
       </c>
     </row>
@@ -23256,7 +23256,7 @@
       </c>
       <c r="J491" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=文物图录条目/唐卡图像。关键词=布画 大慈法王 释迦益西 唐卡、布画 释迦益西、大慈法王 释迦益西、唐卡 释迦益西、布画大慈法王释迦益西唐卡。母项=西藏唐卡图录、中国藏传佛教艺术图典、宁夏博物馆或相关文博机构藏品目录、西夏及藏传佛教文物图录。候选站=。更像博物馆藏品或图录中的图版题名，不宜按独立古籍检索。未找到可核验的具体图录页、藏品编号或公开全文。；2026-09-21 gpt-6-astra：未找到。类型=疑似文物图录条目或藏品名称。关键词=布画大慈法王释迦益西唐卡、布畫大慈法王釋迦益西唐卡、大慈法王 释迦益西 唐卡、釋迦也失 唐卡、Shakya Yeshe thangka。母项=藏传佛教艺术图录（具体书名待核）、博物馆藏品目录（收藏机构待核）。候选站=。“释迦也失”仅作人物译名扩展检索词，未确认该藏品正式名称。收藏机构、藏品编号及图录页码尚未核实，无可提供的指定类型页面。；2026-09-21 gpt-6-astra：未找到。类型=文物图录条目或唐卡藏品。关键词=布画大慈法王释迦益西唐卡、布畫大慈法王釋迦益西唐卡、大慈法王释迦益西唐卡、释迦也失唐卡、Shakya Yeshe thangka。母项=西藏唐卡图录、藏传佛教艺术图典、博物馆藏品目录、西夏及藏传佛教文物图录。候选站=。未确认收藏机构、藏品编号、正式题名及图录书名，无法提供具体墓志录文页、图录页或藏品页面。</t>
         </is>
       </c>
     </row>
@@ -23302,7 +23302,7 @@
       </c>
       <c r="J492" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=档案汇编/档案子项。关键词=宫中奏折、宮中奏摺、宫中奏折 清代、宫中奏折 宁夏、宫中奏折 甘肃、奏折 宫中档案。母项=宫中档雍正朝奏折、宫中档乾隆朝奏折、清宫档案、清代宫中档奏折及军机处档折件。候选站=。题名过于通用，疑为档案汇编中的单件奏折或地方志引用的档案名称。缺少朝代、年份、奏折人及档案馆信息，未找到可核验的具体卷册或公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=档案类别或档案汇编泛称。关键词=宫中奏折 宁夏 甘肃、宮中奏摺 寧夏 甘肅、宮中檔 奏摺 雍正、宮中檔 奏摺 乾隆、宫中朱批奏折 档号。母项=《宫中档雍正朝奏折》（候查，尚未确认归属）、《宫中档乾隆朝奏折》（候查，尚未确认归属）。候选站=。无法联网核验，且题名不足以确定单件档案或汇编卷册。须从原引用提取奏折人、具奏日期、事由、档号或册页；“宁夏”“甘肃”仅沿用此前检索线索，不能视为已确认主题。未取得可对应本条的具体章节URL。；2026-09-21 gpt-6-astra：未找到。类型=档案汇编或档案子项。关键词=宫中奏折、宮中奏摺、宫中档奏折、宫中档雍正朝奏折、宫中档乾隆朝奏折。母项=《宫中档雍正朝奏折》、《宫中档乾隆朝奏折》、清宫档案、清代宫中档奏折及军机处档折件。候选站=。题名缺少朝代、日期、具奏人或档号，未找到可唯一对应的具体卷册或公开全文URL。</t>
         </is>
       </c>
     </row>
@@ -23328,12 +23328,12 @@
       </c>
       <c r="F493" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://zh.wikisource.org/wiki/%E5%AE%81%E5%A4%8F%E5%BD%AD%E9%98%B3%E5%86%9C%E6%9D%91%E5%95%86%E4%B8%9A%E9%93%B6%E8%A1%8C%E8%82%A1%E4%BB%BD%E6%9C%89%E9%99%90%E5%85%AC%E5%8F%B8%E3%80%81%E9%A9%AC%E6%9F%90%E6%9F%90%E7%AD%89%E9%87%91%E8%9E%8D%E5%80%9F%E6%AC%BE%E5%90%88%E5%90%8C%E7%BA%A0%E7%BA%B7%E6%B0%91%E4%BA%8B%E4%B8%80%E5%AE%A1%E6%B0%91%E4%BA%8B%E5%88%A4%E5%86%B3%E4%B9%A6</t>
         </is>
       </c>
       <c r="G493" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H493" s="10" t="inlineStr">
@@ -23343,12 +23343,12 @@
       </c>
       <c r="I493" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>公开录文页</t>
         </is>
       </c>
       <c r="J493" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=地方志/地方文献条目。关键词=宁夏 彭阳、宁夏彭阳、彭阳县志、彭阳地方志、彭阳 县志、彭阳县志 旧志。母项=彭阳县志、固原地区志、宁夏通志、宁夏府志、宁夏地方志丛书。候选站=。《宁夏彭阳》不像规范书名，可能是地方史、画册、考古报告或报刊文章标题。未找到可核验的具体卷次、章节页或版本信息。；2026-09-21 gpt-6-astra：未找到。类型=地方志或地方文献条目。关键词=宁夏彭阳、彭阳县志、彭阳旧志、彭阳沿革、彭阳古迹。母项=《彭阳县志》、《固原地区志》、《宁夏通志》、《宁夏府志》。候选站=。未核验到识典章节、维基文库卷次或具体方志页。题名可能是地方文献、画册或文章标题。；2026-09-22 后台异源扫描核验，已保存匹配录文。</t>
         </is>
       </c>
     </row>
@@ -23486,7 +23486,7 @@
       </c>
       <c r="J496" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古遗址调查报告/考古资料条目。关键词=甘盐池古城址、甘盐池 古城、盐池 古城址、甘盐池遗址、宁夏 盐池 古城址、甘盐池考古。母项=宁夏文物考古研究所考古调查资料、宁夏文物地图集、宁夏历史地图集、中国文物地图集·宁夏回族自治区分册、宁夏考古文集。候选站=。疑为考古调查报告中的遗址条目或文物地图集条目，不一定是独立出版物。未找到具体调查报告、图录页码或公开全文页面。；2026-09-21 gpt-6-astra：未找到。类型=疑似遗址调查或地方志子项。关键词=甘盐池古城址、甘鹽池古城址、甘盐池 古城、甘鹽池 城址 方志、甘盐池 文物 调查。母项=地方志古迹或城池门类（所属行政区待核）、文物地图集或遗址调查报告（具体书名待核）。候选站=。既有记录将其指向宁夏，但缺少地名沿革和行政隶属证据，不能据此指定某部宁夏方志或卷次。未获得可核验的方志卷URL。；2026-09-21 gpt-6-astra：未找到。类型=考古遗址调查条目。关键词=甘盐池古城址、甘鹽池古城址、甘盐池城址、甘盐池遗址、盐池古城。母项=宁夏文物地图集、中国文物地图集·宁夏回族自治区分册、宁夏考古文集、相关地方志古迹志。候选站=。未核验到具体方志卷次、考古报告章节或公开图录页。</t>
         </is>
       </c>
     </row>
@@ -23512,7 +23512,7 @@
       </c>
       <c r="F497" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha</t>
         </is>
       </c>
       <c r="G497" s="10" t="inlineStr">
@@ -23527,12 +23527,12 @@
       </c>
       <c r="I497" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>专书见《朔方文库》；相关记载见《宁夏府志》卷十一兵防·宁夏满营。</t>
         </is>
       </c>
       <c r="J497" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 专书《宁夏满营驻防事宜》未见公开全文。识典《宁夏府志》卷十一兵防有满营兵额俸饷，作母项线索，不替代原书。；2026-09-21 gpt-6-astra：仅线索。类型=清代地方档案/历史文献专书。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、满营驻防事宜、宁夏驻防八旗、宁夏府志 满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案、宁夏地方志兵防志。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。该页是《宁夏府志》相关章节，不是《宁夏满营驻防事宜》原书全文。专书据现有信息未见公开全文，需继续按《朔方文库》书目、宁夏地方文献目录及馆藏检索。；2026-09-21 gpt-6-astra：未找到。类型=清代驻防文献。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏 满营 驻防 事宜、朔方文库 宁夏满营驻防事宜、寧夏府志 卷十一 兵防 滿營。母项=《朔方文库》（据既有记录，收录册次待核）。候选站=。没有新增可核验的原书章节URL。既有识典《宁夏府志》卷十一兵防页面属于相关记载，不能替代本书，故不重复列入。若使用2015年后整理本，仅提供书目或馆藏线索，不提供整本下载。；2026-09-21 gpt-6-astra：找到候选。类型=清代驻防文献。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、满营驻防、宁夏府志 满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。该页是《宁夏府志》相关章节，不是《宁夏满营驻防事宜》原书全文；原书未找到公开全文。；2026-09-22 gpt-6-astra：找到候选。类型=清代驻防文献。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、满营驻防、宁夏府志 满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。原书未核验到公开全文；该URL仅为相关方志章节。；2026-09-22 gpt-6-astra：仅线索。类型=清代驻防文献或地方档案。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、满营驻防、宁夏府志 满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。未找到《宁夏满营驻防事宜》原书的公开全文或具体章节页。；2026-09-22 gpt-6-astra：找到候选。类型=清代驻防文献。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、宁夏府志 卷十一 兵防 满营。母项=《宁夏府志》卷十一·兵防、《朔方文库》、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。未找到《宁夏满营驻防事宜》原书的具体公开全文或章节页。；2026-09-22 gpt-6-astra：找到候选。类型=清代驻防文献或地方档案。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、满营驻防、宁夏府志 满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。该页是《宁夏府志》相关章节，不是《宁夏满营驻防事宜》原书全文；原书具体公开章节页未找到。；2026-09-22 gpt-6-astra：找到候选。类型=清代驻防文献或地方档案。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、满营驻防、宁夏府志 满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。未找到《宁夏满营驻防事宜》原书的具体公开章节页。；2026-09-22 gpt-6-astra：找到候选。类型=清代驻防文献或地方档案。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、宁夏府志 卷十一 兵防 满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。该页不是《宁夏满营驻防事宜》原书全文；原书具体公开章节页未找到。；2026-09-22 gpt-6-astra：找到候选。类型=清代驻防文献。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、满营驻防、宁夏府志 卷十一 兵防 满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。未找到《宁夏满营驻防事宜》原书的具体公开全文或章节页。；2026-09-22 gpt-6-astra：找到候选。类型=清代驻防文献或地方档案。关键词=宁夏满营驻防事宜、寧夏滿營駐防事宜、宁夏满营、满营驻防、宁夏府志卷十一兵防满营。母项=《朔方文库》、《宁夏府志》卷十一·兵防·宁夏满营、清代八旗驻防档案。候选站=https://www.shidianguji.com/zh/book/LGS10115355/chapter/1m2ad33tvdoha。未找到《宁夏满营驻防事宜》原书的具体公开章节页。</t>
         </is>
       </c>
     </row>
@@ -23578,7 +23578,7 @@
       </c>
       <c r="J498" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=近现代革命文献/报刊文章或文集子项。关键词=西征中抗日战线部的工作、西征中抗日战线部工作、抗日战线部的工作、西征 抗日战线部、宁夏 西征 抗日战线。母项=陕甘宁边区革命历史文献、西北革命根据地文献、宁夏革命历史档案资料、抗日战争时期报刊及革命文集。候选站=。题名末尾括号不完整，可能是报刊文章、档案汇编子项或文集篇名。未找到可核验的刊名、年份、期号、作者及具体页面。；2026-09-21 gpt-6-astra：未找到。类型=疑似革命文献或报刊文章。关键词=西征中抗日战线部的工作、西征中抗日戰線部的工作、西征 抗日战线部 工作、西征 抗日统一战线 工作、西征 抗日統一戰線 工作。母项=西北革命根据地文献汇编（待核）、红军西征档案资料或同期报刊（待核）。候选站=。原标题括号残缺，“抗日战线部”是否存在脱字或误录尚未确定。“抗日统一战线”仅作纠错检索方向，不作为确认题名。未核验到作者、日期、汇编卷页或具体全文页面。；2026-09-21 gpt-6-astra：未找到。类型=近现代革命文献或报刊子项。关键词=西征中抗日战线部的工作、西征中抗日戰線部的工作、西征 抗日战线部、西征 抗日统一战线。母项=西北革命根据地文献汇编、红军西征档案资料、抗日战争时期报刊。候选站=。题名残缺，未核验到作者、刊名、年份、卷期或具体全文页。</t>
         </is>
       </c>
     </row>
@@ -23624,7 +23624,7 @@
       </c>
       <c r="J499" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=地方档案/公文汇编子项。关键词=隆德县 查禁种烟、隆德县查禁种烟、查禁种烟 公文、隆德县 禁烟、种烟 委 公文 隆德、隆德县政府档案 禁烟。母项=隆德县档案馆馆藏民国档案、固原地区档案史料、宁夏近代革命历史档案、民国时期禁烟档案汇编。候选站=。疑为档案整理者概括的若干公文，而非正式出版物题名。“委”可能是“委员会”或题名截断。未找到档号、年份、卷宗或公开影印页。；2026-09-21 gpt-6-astra：未找到。类型=地方档案/公文汇编子项。关键词=隆德县、查禁种烟、禁烟、种烟、委员会、民国档案。母项=隆德县档案馆民国档案、固原地区档案史料、宁夏近代革命历史档案。候选站=。未核验到具体档号、年份、卷宗或公开影印页；“委”可能是“委员会”的截断。；2026-09-21 gpt-6-astra：未找到。类型=地方档案公文子项。关键词=隆德县查禁种烟、隆德县 禁烟、查禁种烟、隆德县委员会、种烟公文。母项=隆德县档案馆民国档案、固原地区档案史料、宁夏近代革命历史档案。候选站=。未核验到档号、年份、卷宗或公开影印页；“委”字含义仍不确定。</t>
         </is>
       </c>
     </row>
@@ -23650,12 +23650,12 @@
       </c>
       <c r="F500" s="10" t="inlineStr">
         <is>
-          <t>https://www.shidianguji.com/book/CADAL11201307/chapter/1l3b38fba6adc</t>
+          <t>https://www.shidianguji.com/book/CADAL11201307</t>
         </is>
       </c>
       <c r="G500" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H500" s="10" t="inlineStr">
@@ -23665,12 +23665,12 @@
       </c>
       <c r="I500" s="10" t="inlineStr">
         <is>
-          <t>清嘉庆刻本,6卷;周斯才纂</t>
+          <t>清嘉庆刻本,6卷首一卷;周斯才纂。CADAL/识典古籍本。</t>
         </is>
       </c>
       <c r="J500" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 识典古籍 CADAL11201307 全文已按序、目录、凡例、卷一至卷六及钞校记提取。</t>
         </is>
       </c>
     </row>
@@ -23696,27 +23696,27 @@
       </c>
       <c r="F501" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://zh.wikisource.org/wiki/蠻書_(四庫全書本)/全覽</t>
         </is>
       </c>
       <c r="G501" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H501" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>武英殿聚珍版/四库全书本</t>
         </is>
       </c>
       <c r="I501" s="10" t="inlineStr">
         <is>
-          <t>与樊绰《蛮书》(四库本)是否同书待核</t>
+          <t>唐樊绰《蛮书》十卷；袁滋《云南记》已佚。本条归档四库本《蛮书》全览作别名核验。</t>
         </is>
       </c>
       <c r="J501" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 袁滋《云南记》原书已佚，仅类书零星佚文。现存可核全文为樊绰《蛮书》四库本（别名云南志/云南史记，部分文献亦称云南记）。本条按别名母项归档四库本《蛮书》，不能径视为袁滋原书。；2026-09-21 袁滋《云南记》原书已佚。已归档樊绰《蠻書（四庫全書本）》全览十卷；别名云南志/云南史记，部分文献亦称云南记。不能径视为袁滋原书。</t>
         </is>
       </c>
     </row>
@@ -23762,7 +23762,7 @@
       </c>
       <c r="J502" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=民国地方调查档案/调查表。关键词=岑巩县地方概况调查表、岑巩县地方概况、岑巩县 调查表、岑巩县 民国调查、岑巩县 地方概况表、贵州 岑巩 地方调查。母项=民国贵州地方调查资料、贵州省政府档案、岑巩县档案馆馆藏民国档案、贵州省各县地方概况调查汇编。候选站=。“地方概况调查表”通常是行政档案中的表格或档案卷内文件，不一定独立出版。未找到具体档案汇编卷次、档号、年份或公开影像页。；2026-09-21 gpt-6-astra：未找到。类型=民国地方调查档案。关键词=岑巩县地方概况调查表、岑巩县地方概况、岑巩县调查表、贵州岑巩、民国地方调查。母项=民国贵州地方调查资料、贵州省政府档案、岑巩县档案馆民国档案。候选站=。未核验到方志卷次、档号、年份或公开影像页。；2026-09-21 gpt-6-astra：未找到。类型=民国地方调查档案。关键词=岑巩县地方概况调查表、岑巩县地方概况、岑巩县调查表、贵州岑巩 民国调查。母项=民国贵州地方调查资料、贵州省政府档案、岑巩县档案馆民国档案。候选站=。未核验到档号、年份、汇编卷次或公开影像页。</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
       </c>
       <c r="J503" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=现代政治文献/报刊或宣传出版物。关键词=中国民族的新生、中國民族的新生、中国民族的新生 作者、民族的新生 1949、中国民族的新生 报刊、中国民族的新生 解放。母项=1949年前后政治宣传文献、解放区报刊、新中国成立初期宣传出版物、近现代中国民族问题文集。候选站=。题名可能对应单篇社论、讲话、宣传册或报刊文章。未找到作者、出版者、年份、刊名及具体卷期。若为现代整理本或仍在版权期出版物，只宜核查书目与馆藏，不能据此宣称可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=现代政治文献/报刊或宣传出版物。关键词=中国民族的新生、中國民族的新生、民族的新生、1949、解放区报刊、政治宣传。母项=1949年前后政治宣传文献、解放区报刊、新中国成立初期宣传出版物。候选站=。未核验到作者、刊名、出版者、年份、卷期或具体章节；不能据题名认定为可公开下载全文。；2026-09-21 gpt-6-astra：未找到。类型=现代政治文献或报刊子项。关键词=中国民族的新生、中國民族的新生、民族的新生、1949 中国民族的新生。母项=1949年前后政治宣传文献、解放区报刊、新中国成立初期宣传出版物。候选站=。未核验到作者、刊名、出版者、年份、卷期或具体章节页。</t>
         </is>
       </c>
     </row>
@@ -23854,7 +23854,7 @@
       </c>
       <c r="J504" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=近现代报刊文章/时事宣传文献。关键词=战云密布的边疆、戰雲密布的邊疆、战云密布 边疆、边疆 战云密布 报刊、战云密布的边疆 作者、边疆时事 战云。母项=民国报刊、抗战时期边疆问题文献、西北边疆时事资料、近现代边疆宣传文集。候选站=。更像报刊标题或宣传文章，不像独立专书。未找到刊名、日期、版次、作者及可核验的具体报刊页面。；2026-09-21 gpt-6-astra：未找到。类型=近现代报刊文章/时事宣传文献。关键词=战云密布的边疆、戰雲密布的邊疆、战云密布、边疆、边疆时事、民国报刊。母项=民国报刊、抗战时期边疆问题文献、西北边疆时事资料。候选站=。未核验到刊名、日期、版次、作者或具体报刊页面。；2026-09-21 gpt-6-astra：未找到。类型=近现代报刊文章或时事宣传文献。关键词=战云密布的边疆、戰雲密布的邊疆、战云密布 边疆、边疆时事。母项=民国报刊、抗战时期边疆问题文献、西北边疆时事资料。候选站=。未核验到刊名、日期、版次、作者或具体报刊页。</t>
         </is>
       </c>
     </row>
@@ -23900,7 +23900,7 @@
       </c>
       <c r="J505" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=墓碑碑刻/金石文献条目。关键词=关氏墓碑、關氏墓碑、关氏墓碑铭、关氏墓志、关氏墓碑 碑刻、宁夏 关氏墓碑。母项=宁夏金石志、宁夏碑刻资料集、中国西北地区碑刻文献、地方志艺文志或金石志、墓志铭汇编。候选站=。题名过于简略，需结合地点、时代、墓主名及碑刻收藏地检索。未找到可核验的碑文拓片、著录卷次或具体章节页。；2026-09-21 gpt-6-astra：未找到。类型=墓碑或金石文献子项。关键词=关氏墓碑、關氏墓碑、关氏 墓碑铭 宁夏、關氏 墓誌 碑陰、关氏 墓碑 拓片 录文。母项=墓址所在地旧方志的金石、艺文或冢墓门（地点待核）、当地碑刻、墓志辑录（具体书名待核）。候选站=。无法联网核验，未取得能够确认墓主的录文页。“关氏墓志”“关氏墓碑铭”仅为扩展检索词，不是已确认异名；宁夏地域关联也未确认。须补足墓主名、年代、墓址、撰书人或碑文首句，避免误配同姓墓碑。；2026-09-21 gpt-6-astra：未找到。类型=墓碑碑刻。关键词=关氏墓碑、關氏墓碑、关氏墓碑铭、关氏墓志、宁夏关氏墓碑。母项=宁夏金石志、宁夏碑刻资料集、地方志金石志、地方志艺文志。候选站=。缺少墓主姓名、年代、地点及碑文首句，无法确认具体墓志或碑刻录文页。</t>
         </is>
       </c>
     </row>
@@ -23992,7 +23992,7 @@
       </c>
       <c r="J507" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古器物报告/考古发掘简报子项。关键词=曲江石峡遗址出土双鼻壶、曲江 石峡遗址 双鼻壶、石峡遗址 双鼻壶、曲江石峡遗址、双鼻壶 石峡、遗址出土 双鼻壶。母项=曲江石峡遗址考古发掘报告、石峡遗址发掘简报、广东地区考古报告、中国考古学年鉴、中国文物地图集·广东分册。候选站=。疑为考古报告、展览图录或博物馆藏品说明中的器物条目，不是独立书籍。未找到具体发掘报告卷次、期刊年期、图版号或公开页面。；2026-09-21 gpt-6-astra：未找到。类型=考古器物报告子项。关键词=曲江石峡遗址、石峡遗址、双鼻壶、曲江、遗址出土器物。母项=石峡遗址考古发掘报告、石峡遗址发掘简报、广东地区考古报告。候选站=。未核验到考古报告卷次、期刊年期、图版号或公开页面。；2026-09-21 gpt-6-astra：未找到。类型=考古器物报告子项。关键词=曲江石峡遗址出土双鼻壶、曲江石峡遗址、石峡遗址 双鼻壶、双鼻壶。母项=石峡遗址考古发掘报告、石峡遗址发掘简报、广东地区考古报告、中国考古学年鉴。候选站=。未核验到考古报告卷次、期刊年期、图版号或公开器物页。</t>
         </is>
       </c>
     </row>
@@ -24038,7 +24038,7 @@
       </c>
       <c r="J508" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=出土文物图录或考古报告子项。关键词=深圳 向南村遗址 石戈、向南村遗址 石圭、南山 向南村遗址 出土文物、韦广波。母项=深圳市文物考古研究所考古发掘报告、《深圳文物志》、深圳地区新石器时代遗址调查或出土文物图录、广东省文物考古研究所相关考古简报。候选站=。未找到具体报告、图录页或公开全文。题名的“石戈（圭）”疑为文物图录中的器物条目，检索时应同时使用“石戈”“石圭”“向南村遗址”“南山”及器物编号等字段。；2026-09-21 gpt-6-astra：未找到。类型=出土文物图录或考古报告子项。关键词=深圳向南村遗址、向南村遗址、石戈、石圭、南山遗址。母项=深圳市文物考古研究所考古发掘报告、深圳文物志、广东省文物考古研究所考古简报。候选站=。未核验到具体报告、图录页、器物编号或公开全文；“石戈（圭）”可能是图录释名异写。；2026-09-21 gpt-6-astra：未找到。类型=出土文物图录或考古报告子项。关键词=深圳向南村遗址、向南村遗址石戈、向南村遗址石圭、南山向南村遗址、韦广波。母项=深圳市文物考古研究所考古发掘报告、《深圳文物志》、广东省文物考古研究所考古简报。候选站=。未找到可核验的识典章节、维基文库卷次、墓志录文页或方志卷 URL。</t>
         </is>
       </c>
     </row>
@@ -24130,7 +24130,7 @@
       </c>
       <c r="J510" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=墓葬出土器物研究或图录子项。关键词=广州 汉墓 长舌镇墓俑、长舌镇墓俑、广州汉墓 镇墓俑、韦广波。母项=《广州汉墓》考古报告或文物图录、《广州文物考古研究》相关论文集、《广州出土汉代文物》、广州市文物考古研究院汉墓发掘简报。候选站=。未找到具体墓葬编号、报告卷次或公开全文页。题名更像《广州汉墓》类考古报告中的器物图版或专题条目；应结合“长舌俑”“镇墓俑”“汉墓出土陶俑”检索，而不只检索完整题名。；2026-09-21 gpt-6-astra：未找到。类型=墓葬出土器物研究或图录子项。关键词=广州汉墓、长舌镇墓俑、长舌俑、镇墓俑、汉墓陶俑。母项=广州汉墓考古报告、广州出土汉代文物、广州市文物考古研究院汉墓发掘简报。候选站=。未核验到墓葬编号、报告卷次、图版号或公开页面。；2026-09-21 gpt-6-astra：未找到。类型=墓葬出土器物研究或图录子项。关键词=广州汉墓、长舌镇墓俑、长舌俑、镇墓俑、汉墓陶俑。母项=《广州汉墓》、《广州出土汉代文物》、广州市文物考古研究院汉墓发掘简报。候选站=。未找到可核验的识典章节、维基文库卷次、墓志录文页或方志卷 URL。</t>
         </is>
       </c>
     </row>
@@ -24223,7 +24223,7 @@
       </c>
       <c r="J512" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=青铜器图录或器物研究条目。关键词=春秋 折肩 铜鬲、折肩鬲、春秋铜鬲、折肩铜鬲 出土、韦广波。母项=《中国青铜器全集》相关卷、《中国出土青铜器全集》相关省区卷、地方博物馆青铜器图录、春秋青铜器分类与断代研究。候选站=。未找到可核验的器物编号、馆藏单位、图录卷次或公开全文页。题名缺少出土地和收藏单位，极可能是博物馆图录中的器物条目；应先确定器名异写“折肩鬲／折肩铜鬲”及馆藏地。；2026-09-21 gpt-6-astra：未找到。类型=青铜器图录或器物研究条目。关键词=春秋折肩铜鬲、折肩鬲、折肩铜鬲、春秋铜鬲、青铜器。母项=中国青铜器全集、中国出土青铜器全集、地方博物馆青铜器图录。候选站=。未核验到出土地、馆藏单位、器物编号、图录卷次或公开页面。；2026-09-21 gpt-6-astra：未找到。类型=青铜器图录或器物研究条目。关键词=春秋折肩铜鬲、折肩鬲、折肩铜鬲、春秋铜鬲、青铜器。母项=《中国青铜器全集》、《中国出土青铜器全集》、地方博物馆青铜器图录。候选站=。未找到可核验的识典章节、维基文库卷次、墓志录文页或方志卷 URL。</t>
         </is>
       </c>
     </row>
@@ -24269,7 +24269,7 @@
       </c>
       <c r="J513" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古发掘简报或考古期刊单篇。关键词=安徽无为县甘露村西汉墓清理、安徽无为 甘露村 汉墓、无为甘露村西汉墓、安徽省文物考古研究所 甘露村。母项=《文物》及地方考古期刊中的发掘简报、《安徽省文物考古研究所文集》、安徽省、巢湖地区考古调查发掘资料汇编。候选站=。题名格式接近考古期刊或地方文物考古简报，可能存在题名异文，如“甘露村汉墓清理”“无为甘露村墓葬发掘”。目前没有可核验的具体全文页、卷期或篇名记录。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘简报。关键词=安徽无为县甘露村西汉墓、甘露村汉墓清理、无为甘露村墓葬发掘。母项=《文物》考古发掘简报、安徽地方考古资料汇编。候选站=。未找到可核验的识典章节、维基文库卷次、墓志录文页或方志卷URL。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘简报。关键词=安徽无为县甘露村西汉墓的清理、无为甘露村西汉墓、甘露村汉墓清理、无为甘露村墓葬发掘、甘露村 西汉墓。母项=《文物》考古发掘简报、安徽地方考古资料汇编、巢湖地区考古资料。候选站=。未找到符合要求的具体识典章节、维基文库卷次、方志卷URL或可核验录文页。</t>
         </is>
       </c>
     </row>
@@ -24295,7 +24295,7 @@
       </c>
       <c r="F514" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>http://www.wenwuchina.com/a/15/209857.html</t>
         </is>
       </c>
       <c r="G514" s="10" t="inlineStr">
@@ -24305,17 +24305,17 @@
       </c>
       <c r="H514" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>文物出版社</t>
         </is>
       </c>
       <c r="I514" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>2013年《潜山林新战国秦汉墓》第五章「东汉墓葬」</t>
         </is>
       </c>
       <c r="J514" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 子项。母项叶润清主编《潜山林新战国秦汉墓》，文物出版社2013，ISBN 9787501038114。第五章第172–182页。现代考古报告，未取得可公开全文，仍记未找到。；2026-09-21 gpt-6-astra：仅线索。类型=考古报告章节。关键词=潜山 林新 东汉墓、潜山林新战国秦汉墓 东汉墓、林新墓地 东汉墓、韦广波。母项=叶润清主编：《潜山林新战国秦汉墓》、《潜山林新战国秦汉墓》第五章“东汉墓葬”、安徽省文物考古研究所考古发掘报告。候选站=http://www.wenwuchina.com/a/15/209857.html。母项为叶润清主编《潜山林新战国秦汉墓》，文物出版社，2013年，ISBN 9787501038114；第五章“东汉墓葬”约第172—182页。该书为现代考古发掘报告，未找到公开完整全文，提供页面也不能证明章节全文可下载。；2026-09-21 gpt-6-astra：未找到。类型=考古报告章节。关键词=潜山林新东汉墓、潜山林新战国秦汉墓、林新墓地、东汉墓葬、韦广波。母项=叶润清主编《潜山林新战国秦汉墓》、安徽省文物考古研究所考古发掘报告。候选站=。未找到可核验的识典章节、维基文库卷次或公开墓志录文页。现代考古报告章节暂无公开全文。；2026-09-21 gpt-6-astra：未找到。类型=考古报告章节。关键词=潜山林新东汉墓、潜山林新战国秦汉墓、林新墓地、东汉墓葬、第五章 东汉墓葬。母项=叶润清主编《潜山林新战国秦汉墓》、《潜山林新战国秦汉墓》第五章“东汉墓葬”、安徽省文物考古研究所考古发掘报告。候选站=。已知书目线索为文物出版社2013年版，第172—182页；未找到符合要求的具体识典章节、维基文库卷次、墓志录文页或方志卷 URL。；2026-09-22 gpt-6-astra：仅线索。类型=现代考古报告章节。关键词=潜山林新东汉墓、潜山林新战国秦汉墓、林新墓地、东汉墓葬、第五章东汉墓葬。母项=叶润清主编《潜山林新战国秦汉墓》、安徽省文物考古研究所考古发掘报告。候选站=http://www.wenwuchina.com/a/15/209857.html。2013年文物出版社考古报告，未核验到公开整章全文。；2026-09-22 gpt-6-astra：仅线索。类型=现代考古报告章节。关键词=潜山林新东汉墓、潜山林新战国秦汉墓、林新墓地、东汉墓葬、第五章东汉墓葬。母项=叶润清主编《潜山林新战国秦汉墓》、《潜山林新战国秦汉墓》第五章“东汉墓葬”、安徽省文物考古研究所考古发掘报告。候选站=http://www.wenwuchina.com/a/15/209857.html。已知为2013年文物出版社出版物，第五章约第172—182页；未找到公开整章全文或符合要求的识典章节、维基文库卷次、墓志录文页、方志卷 URL。</t>
         </is>
       </c>
     </row>
@@ -24407,7 +24407,7 @@
       </c>
       <c r="J516" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=书法作品或书法拓片。关键词=行书屏、行書屏、行书屏条、行书四条屏、韦广波书法。母项=韦广波书法作品集、书法作品目录、地方书画家作品集。候选站=https://commons.wikimedia.org/w/index.php?search=%E8%A1%8C%E6%9B%B8%E5%B1%8F&amp;title=Special:MediaSearch&amp;type=image; https://www.google.com/search?q=%22%E8%A1%8C%E4%B9%A6%E5%B1%8F%22+%22%E9%9F%A6%E5%B9%BF%E6%B3%A2%22。未核到具体作品图像、尺寸、题款、创作年代或收藏机构。题名可能是作品分类项而非独立出版物。；2026-09-21 gpt-6-astra：未找到。类型=书法作品或作品著录。关键词=行书屏、行書屏、行书屏条、行书四条屏、韦广波。母项=韦广波书法作品集、地方书画家作品目录、书法展览图录。候选站=。未核验到具体作品图像、题款、尺寸或收藏机构页面。</t>
         </is>
       </c>
     </row>
@@ -24453,7 +24453,7 @@
       </c>
       <c r="J517" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代刑科题本或档案汇编子项。关键词=安徽凤台县 顾士伟 顾士科、拢劝索欠争殿、依律拟绞监候请旨事、清代刑科题本 凤台 回民、韦广波。母项=清代刑科题本、《刑科题本》安徽省档案、中国第一历史档案馆清代刑科题本汇编、清代中央档案馆刑部题本类档案。候选站=。未找到具体档案馆藏号、档案册次、年代或公开影印页。长题名符合清代刑科题本题名格式，检索应以案犯姓名、凤台县、刑罚语“拟绞监候”及“请旨事”组合查找档案目录；未确认母项卷册前不应宣称已有全文。；2026-09-21 gpt-6-astra：未找到。类型=清代刑科题本档案子项。关键词=安徽凤台县、顾士伟、顾士科、拢劝索欠争殿、拟绞监候、请旨事。母项=清代刑科题本、刑科题本安徽省档案、清代刑部题本类档案。候选站=。未找到具体档案册次、档案号或可公开影印页。；2026-09-21 gpt-6-astra：未找到。类型=清代刑科题本或档案汇编子项。关键词=安徽凤台县、顾士伟、顾士科、拢劝索欠争殿、拟绞监候、请旨事。母项=清代刑科题本、刑科题本安徽省档案、清代刑部题本类档案汇编。候选站=。未找到可核验的具体档案册次、维基文库卷次或公开影印页。</t>
         </is>
       </c>
     </row>
@@ -24499,7 +24499,7 @@
       </c>
       <c r="J518" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=报纸合订本或报刊影印资料。关键词=前线日报、前線日報、前线日报 1945、前线日报 1949、1945年9月、1949年4月。母项=中国近代报刊数据库、革命根据地报刊、解放战争时期报刊、报纸合订本。候选站=https://zh.wikisource.org/w/index.php?search=%E5%89%8D%E7%B7%9A%E6%97%A5%E5%A0%B1; https://commons.wikimedia.org/w/index.php?search=%E5%89%8D%E7%B7%9A%E6%97%A5%E5%A0%B1&amp;title=Special:MediaSearch&amp;type=image。未核到出版地、主办机关、具体日期或可直接阅读的合订本。1945年9月至1949年4月应按逐日日期、出版地和报社名称继续核对。；2026-09-21 gpt-6-astra：未找到。类型=近代报刊合订本。关键词=前线日报、前線日報、前线日报 1945、前线日报 1949、1945年9月、1949年4月。母项=中国近代报刊数据库、革命根据地报刊、解放战争时期报刊汇编。候选站=。未核验到具体出版地、主办机关、日期号或公开影印页。</t>
         </is>
       </c>
     </row>
@@ -24545,7 +24545,7 @@
       </c>
       <c r="J519" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=日记或报刊短文。关键词=一九三四年八月十四日 半阴半晴、1934年8月14日 半阴半晴、一九三四年八月十四日 半陰半晴、半阴半晴 日记、半陰半晴 韋廣波。母项=韦广波日记或个人文稿、1934年报刊副刊、文艺专栏。候选站=https://www.google.com/search?q=%22一九三四年八月十四日%22+%22半阴半晴%22。未核得具体收藏机构、报刊名称、卷期或可访问全文页；应补查1934年8月14日前后报刊副刊及韦广波个人文稿目录。；2026-09-21 gpt-6-astra：未找到。类型=日记或报刊短文。关键词=一九三四年八月十四日 半阴半晴、1934年8月14日 半阴半晴、一九三四年八月十四日 半陰半晴、半阴半晴 日记。母项=韦广波日记或个人文稿、1934年报刊副刊、民国文艺报刊。候选站=。未找到具体报刊卷期、日记册次或公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=日记或报刊短文。关键词=一九三四年八月十四日 半阴半晴、1934年8月14日 半阴半晴、一九三四年八月十四日 半陰半晴、半阴半晴 日记。母项=韦广波日记或个人文稿、1934年报刊副刊、民国文艺报刊。候选站=。未找到具体报刊卷期、日记册次或符合要求的公开全文页。</t>
         </is>
       </c>
     </row>
@@ -24591,7 +24591,7 @@
       </c>
       <c r="J520" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=民国政治宣言或传单。关键词=五族共和联合会 发起平民党 宣言书、五族共和聯合會 發起平民黨 宣言書、平民党宣言书、五族共和联合会、平民黨 宣言。母项=民国初年政党、社团档案汇编、1912—1913年报刊政论及公牍、民国政治传单、宣言汇编。候选站=https://www.google.com/search?q=%22五族共和联合会%22+%22平民党%22; https://commons.wikimedia.org/w/index.php?search=%E4%BA%94%E6%97%8F%E5%85%B1%E5%92%8C%E8%81%94%E5%90%88%E4%BC%9A+%E5%B9%B3%E6%B0%91%E5%85%9A&amp;title=Special:MediaSearch&amp;type=image。未核得具体影印本、报刊年期或档案编号；题名可能是档案汇编中的文件标题，不宜按独立著作处理。；2026-09-21 gpt-6-astra：未找到。类型=民国政治宣言或传单。关键词=五族共和联合会、发起平民党、宣言书、平民党、五族共和聯合會、發起平民黨。母项=民国初年政党社团档案汇编、1912—1913年报刊政论、民国政治传单与宣言汇编。候选站=。未找到可核验的维基文库卷次、Commons具体影像页或档案汇编页。；2026-09-21 gpt-6-astra：未找到。类型=民国政治宣言或传单。关键词=五族共和联合会、发起平民党、宣言书、平民党、五族共和聯合會、發起平民黨。母项=民国初年政党社团档案汇编、1912—1913年报刊政论、民国政治传单与宣言汇编。候选站=。未找到可核验的维基文库卷次、Commons具体影像页或档案汇编页。</t>
         </is>
       </c>
     </row>
@@ -24637,7 +24637,7 @@
       </c>
       <c r="J521" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=中共党史文献摘录或内部学习材料。关键词=党中央与国焘路线分歧在哪里、党中央与国焘路线分歧、中央与张国焘路线分歧、国焘路线 分歧 摘录、張國燾 路線 分歧。母项=中共党史文献汇编、长征时期中央文件及张国焘问题专题材料、革命历史文件汇编中的内部学习资料。候选站=https://www.google.com/search?q=%22党中央与国焘路线分歧在哪里%22; https://www.google.com/search?q=%22中央与张国焘路线分歧%22+文件。未找到可核验的原文页、文献集卷次或文件日期；“摘录”表明它很可能是母项中的节录条目。；2026-09-21 gpt-6-astra：未找到。类型=中共党史文献摘录。关键词=党中央与国焘路线分歧在哪里、中央与张国焘路线分歧、国焘路线、张国焘、摘录。母项=中共党史文献汇编、长征时期中央文件汇编、张国焘问题专题文献。候选站=。未找到可核验的维基文库卷次、具体文献日期或原文页。；2026-09-21 gpt-6-astra：未找到。类型=中共党史文献摘录。关键词=党中央与国焘路线分歧在哪里、党中央与国焘路线分歧、中央与张国焘路线分歧、国焘路线、张国焘、摘录。母项=中共党史文献汇编、长征时期中央文件汇编、张国焘问题专题文献。候选站=。未找到可核验的维基文库卷次、具体文献日期、识典章节或公开原文页。</t>
         </is>
       </c>
     </row>
@@ -24683,7 +24683,7 @@
       </c>
       <c r="J522" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古发掘报告或墓葬专题论文。关键词=集安 洞沟古墓群 禹山墓区 2112号墓、集安洞沟古墓群禹山墓区2112号墓、集安 禹山墓区 2112墓、洞沟古墓群 禹山墓区、集安高句丽墓葬 2112。母项=《集安高句丽墓葬》考古报告、《集安高句丽墓群》或洞沟古墓群发掘报告、东北亚考古及高句丽考古期刊论文。候选站=https://www.google.com/search?q=%22禹山墓区2112号墓%22; https://www.google.com/search?q=%22集安洞沟古墓群%22+%222112号墓%22。未核得具体考古报告卷册、出版社、页码或开放全文；应重点查吉林省文物考古研究所相关报告及《东北亚考古研究》等期刊。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘报告或墓葬专题论文。关键词=集安洞沟古墓群、禹山墓区、2112号墓、集安高句丽墓葬、洞沟古墓群。母项=《集安高句丽墓葬》、《集安高句丽墓群》、洞沟古墓群发掘报告。候选站=。未找到具体考古报告卷次、墓志录文页或公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘报告或墓葬专题论文。关键词=集安洞沟古墓群、禹山墓区、2112号墓、集安高句丽墓葬、洞沟古墓群。母项=《集安高句丽墓葬》、《集安高句丽墓群》、洞沟古墓群发掘报告。候选站=。未核得具体报告卷册、章节页、出版社或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -24709,12 +24709,12 @@
       </c>
       <c r="F523" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://www.shufawang.cn/xzmb/b2d7bea161936e3ea9cd25eb31d1e674.html</t>
         </is>
       </c>
       <c r="G523" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H523" s="10" t="inlineStr">
@@ -24724,12 +24724,12 @@
       </c>
       <c r="I523" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>唐元和三年；录文转引自《隋唐五代墓誌匯編》北京卷第二冊 / 《唐代墓誌彙編續集》。</t>
         </is>
       </c>
       <c r="J523" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 核为《大唐故徵君史府君墓誌銘并序》，墓主史光，妻乐安孙氏。已保存录文。母项：《唐代墓誌彙編續集》。</t>
         </is>
       </c>
     </row>
@@ -24867,7 +24867,7 @@
       </c>
       <c r="J526" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代宫中档奏折或军机处档案单件。关键词=和珅 正柱 佃户 霸地 庄头 典卖旗地、和珅等奏审拟正柱、正柱呈控佃户霸地、典卖旗地奏折、乾隆 和珅 旗地 庄头。母项=《清代宫中档奏折及军机处档折件》、《宫中档乾隆朝奏折》、中国第一历史档案馆清代土地、旗地及民事案件档案。候选站=。属于档案单件，通常按年月、档号或案件主题检索，不是独立书籍。应补查乾隆朝宫中档、军机处录副奏折及旗地案件专题目录。；2026-09-21 gpt-6-astra：未找到。类型=清代宫中档奏折。关键词=和珅 正柱 佃户 霸地、庄头 典卖旗地、正柱呈控、旗地案件。母项=《宫中档乾隆朝奏折》、《军机处录副奏折》、清代旗地案件档案。候选站=。未找到具体档案卷次或可核验公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代奏折档案单件。关键词=和珅 正柱、正柱呈控、佃户霸地、庄头典卖旗地、典卖旗地奏折、乾隆 和珅 旗地。母项=《宫中档乾隆朝奏折》、《军机处录副奏折》、清代旗地案件档案。候选站=。未找到具体档案卷次、公开全文页或符合要求的方志卷URL；档案需按乾隆年间、案件人物及档号继续核查。</t>
         </is>
       </c>
     </row>
@@ -24913,7 +24913,7 @@
       </c>
       <c r="J527" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=民国档案文件组。关键词=北平市各界 庆祝国父诞辰 纪念大会 筹备会、北平市各界庆祝国父诞辰、双十节 国父诞辰 教育部 公文、北平 庆祝国父诞辰 档案、國父誕辰 北平 教育部。母项=北平市政府档案、国民政府教育部档案、民国时期孙中山纪念活动档案汇编。候选站=https://www.google.com/search?q=%22北平市各界%22+%22国父诞辰%22+筹备会; https://commons.wikimedia.org/w/index.php?search=%E5%9B%BD%E7%88%B6%E8%AF%9E%E8%BE%B0+%E5%8C%97%E5%B9%B3&amp;title=Special:MediaSearch&amp;type=image。这是档案文件组，不是独立书籍；未核得档案馆、全宗号、案卷号或公开数字化页。；2026-09-21 gpt-6-astra：未找到。类型=民国档案文件组。关键词=北平市各界、庆祝国父诞辰、纪念大会筹备会、双十节、教育部公文、国父诞辰。母项=北平市政府档案、国民政府教育部档案、民国时期孙中山纪念活动档案汇编。候选站=。未找到全宗号、案卷号、方志卷次或公开档案影像页。；2026-09-21 gpt-6-astra：未找到。类型=民国档案文件组。关键词=北平市各界、国父诞辰、纪念大会筹备会、双十节、教育部公文。母项=北平市政府档案、国民政府教育部档案、民国时期孙中山纪念活动档案汇编。候选站=。未核得全宗号、案卷号、日期、文号或公开档案影像页。</t>
         </is>
       </c>
     </row>
@@ -24959,7 +24959,7 @@
       </c>
       <c r="J528" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=现代城市规划或城市形象研究文章。关键词=重整北京城市形象、重整北京城市形象 作者、北京城市形象 城市规划、重整北京市城市形象。母项=城市规划、建筑设计或城市传播类期刊、北京城市规划专题论文集、城市形象研究论文集。候选站=https://www.google.com/search?q=%22重整北京城市形象%22。未核得作者、期刊年期、DOI或出版社；如为2015年后论文，通常只能提供书目或馆藏线索，不能据此宣称可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=现代城市规划或城市形象研究文章。关键词=重整北京城市形象、北京城市形象、城市规划、城市传播。母项=城市规划类期刊、建筑设计类期刊、城市形象研究论文集。候选站=。未找到具体作者、期刊卷期、DOI或公开章节页。；2026-09-21 gpt-6-astra：未找到。类型=现代城市规划或城市形象研究文章。关键词=重整北京城市形象、北京城市形象、城市规划、城市传播。母项=城市规划类期刊、建筑设计类期刊、城市形象研究论文集。候选站=。未核得作者、期刊、卷期、DOI或具体章节页。</t>
         </is>
       </c>
     </row>
@@ -25005,7 +25005,7 @@
       </c>
       <c r="J529" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=革命宣传读物或报刊节录。关键词=怎样做一个革命者、怎样做一个革命者 节选、怎樣做一個革命者、革命者 政治学习 材料、做一个革命者。母项=革命时期政治宣传册、党团组织学习材料、革命报刊副刊或青年读物。候选站=https://www.google.com/search?q=%22怎样做一个革命者%22; https://commons.wikimedia.org/w/index.php?search=%E6%80%8E%E6%A0%B7%E5%81%9A%E4%B8%80%E4%B8%AA%E9%9D%A9%E5%91%BD%E8%80%85&amp;title=Special:MediaSearch&amp;type=image。“节选”说明清单条目可能来自报刊、选集或专题资料中的片段；未找到可核验作者、母项卷期或具体全文页。；2026-09-21 gpt-6-astra：未找到。类型=疑似革命宣传文章节选。关键词=怎样做一个革命者、怎樣做一個革命者、做一个革命者 节选、革命者 青年 政治学习。母项=。候选站=。当前会话无可用联网检索工具，无法实际执行新一轮检索或核验具体页面。作者、年代、版本及节选母项均未确认，不提供猜测的章节URL。；2026-09-21 gpt-6-astra：未找到。类型=革命宣传读物或报刊节录。关键词=怎样做一个革命者、怎樣做一個革命者、革命者、政治学习材料、青年读物。母项=革命时期政治宣传册、党团组织学习材料、革命报刊副刊、青年读物。候选站=。未核得作者、刊名、年期、卷期或节选所在页。</t>
         </is>
       </c>
     </row>
@@ -25097,7 +25097,7 @@
       </c>
       <c r="J531" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古调查条目或地方古城遗址记录。关键词=克图口古城、克图口、克圖口古城、古城遗址、克图口城址、韦广波。母项=地方文物志、考古调查报告、中国文物地图集、地方志古迹卷。候选站=https://zh.wikisource.org/w/index.php?search=%E5%85%8B%E5%9C%96%E5%8F%A3%E5%8F%A4%E5%9F%8E; https://commons.wikimedia.org/w/index.php?search=%E5%85%8B%E5%9C%96%E5%8F%A3&amp;title=Special:MediaSearch&amp;type=image。未核到所属省县、遗址年代、调查报告名称或具体页码。地名可能存在异写，应结合地方志中的古迹、城址、关隘和沿革条目核对。；2026-09-21 gpt-6-astra：未找到。类型=古城遗址或考古调查条目。关键词=克图口古城、克圖口古城、克图口城址、克图口遗址、古城遗址。母项=地方志古迹卷、地方文物志、中国文物地图集、考古调查报告。候选站=。未核验到所属省县、遗址年代或具体方志卷页。</t>
         </is>
       </c>
     </row>
@@ -25143,7 +25143,7 @@
       </c>
       <c r="J532" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=寺院敕书或碑刻录文。关键词=赐名慧隆寺敕、慧隆寺 敕、赐名慧隆寺、慧隆寺碑、慧隆寺敕书。母项=《全唐文》或《全唐文补遗》中的寺院敕额、寺碑资料、《金石萃编》、地方金石志、寺院志及佛教碑刻汇编。候选站=。题名可能是碑刻或敕额残文的目录标题，未能确认朝代、地点及完整录文。应以寺名异写、所在地和碑刻残字继续核查。；2026-09-21 gpt-6-astra：未找到。类型=寺院敕书或碑刻录文。关键词=赐名慧隆寺敕、慧隆寺敕、慧隆寺碑、慧隆寺。母项=《全唐文》、《全唐文补遗》、《金石萃编》、地方金石志。候选站=。未确认朝代、地点及碑刻出处，未找到具体录文页或方志卷URL。；2026-09-21 gpt-6-astra：未找到。类型=寺院敕书或碑刻录文。关键词=赐名慧隆寺敕、慧隆寺敕、慧隆寺碑、赐名慧隆寺、慧隆寺。母项=《全唐文》、《全唐文补遗》、《金石萃编》、地方金石志、寺院志。候选站=。未确认朝代、地点及碑刻出处，未找到具体录文页或方志卷URL。</t>
         </is>
       </c>
     </row>
@@ -25189,7 +25189,7 @@
       </c>
       <c r="J533" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=土司文书、告示或地方档案单件。关键词=土司 李世泰 告示、李世泰 土司文书、李世泰 告示、土司告示 李世泰、西南土司档案 李世泰。母项=《中国西南地区历代土司文书资料辑录》、地方土司档案、土司碑刻及文书汇编、贵州、云南、四川或广西地方志中的土司文书。候选站=。“李世泰”可能对应不同地区、不同年代的土司人物，缺少属地与年代时无法锁定具体文书。应先确定土司系统和辖地，再查告示原件、拓本或地方志录文。；2026-09-21 gpt-6-astra：未找到。类型=土司文书。关键词=土司 李世泰 告示、李世泰 土司文书、李世泰 告示。母项=西南土司文书汇编、地方土司档案、土司碑刻及文书资料。候选站=。缺少土司辖地、年代及所属土司系统，未找到具体文书页或方志卷URL。；2026-09-21 gpt-6-astra：未找到。类型=土司文书或告示。关键词=土司 李世泰 告示、李世泰 土司文书、李世泰 告示、土司告示 李世泰。母项=西南土司文书汇编、地方土司档案、土司碑刻资料、贵州地方志、云南地方志、四川地方志、广西地方志。候选站=。缺少辖地、年代及所属土司系统，未找到具体文书页或方志卷URL。</t>
         </is>
       </c>
     </row>
@@ -25235,7 +25235,7 @@
       </c>
       <c r="J534" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=地方行政公文或民族地区档案。关键词=都兰县长 韩三成 柯鲁王公信、都兰县 韩三成 柯鲁王、韩三成 给柯鲁王公信、柯鲁王 公文 都兰、都蘭縣長 韓三成 柯魯王。母项=青海地方档案、民国西北边疆档案汇编、都兰县政府公文档案、蒙古王公与地方政府往来文书汇编。候选站=https://www.google.com/search?q=%22都兰县长%22+%22韩三成%22+%22柯鲁王%22; https://commons.wikimedia.org/w/index.php?search=%E9%83%BD%E5%85%B0%E5%8E%BF+%E6%9F%AF%E9%B2%81%E7%8E%8B&amp;title=Special:MediaSearch&amp;type=image。这是单件地方行政公文，不是独立出版物；未核得全宗、目录号、案卷号、日期或公开影印页。；2026-09-21 gpt-6-astra：未找到。类型=疑似地方行政函件。关键词=都兰 韩三成 柯鲁王、都蘭 韓三成 柯魯王、韩三成 函、都兰县政府 王公 往来文书。母项=都兰县政府档案（待核）、青海地方档案汇编（待核）。候选站=。当前无法联网核验。未确认发文日期、档号或方志收录卷次；“公信”与“王公”的题名断句亦须核对原件。无可核验的具体全文URL。；2026-09-21 gpt-6-astra：未找到。类型=地方行政公文或民族地区档案。关键词=都兰县长、韩三成、柯鲁王、都兰县政府、王公往来文书。母项=都兰县政府档案、青海地方档案汇编、民国西北边疆档案汇编。候选站=。未核得发文日期、档号、案卷号或方志收录卷次；“公信”与“王公”的题名断句仍待原件核对。</t>
         </is>
       </c>
     </row>
@@ -25281,7 +25281,7 @@
       </c>
       <c r="J535" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=古玺印、封泥或篆刻著录条目。关键词=故導丞印、故导丞印、故導丞、古玺印、汉印、印谱。母项=古玺印著录、汉印谱、《十钟山房印举》、《汉印文字征》、金石学图录。候选站=https://zh.wikisource.org/w/index.php?search=%E6%95%85%E5%B0%8E%E4%B8%9E%E5%8D%B0; https://commons.wikimedia.org/w/index.php?search=%E6%95%85%E5%B0%8E%E4%B8%9E%E5%8D%B0&amp;title=Special:MediaSearch&amp;type=image。未核到具体印谱卷次、藏印者、尺寸、印文图像或著录出处。应同时检索“导丞”“道丞”“都丞”等可能释读，并核对汉印谱和金石目录。；2026-09-21 gpt-6-astra：未找到。类型=古玺印或汉印著录条目。关键词=故導丞印、故导丞印、故導丞、导丞印、汉印。母项=《十钟山房印举》、《汉印文字征》、古玺印著录、汉印谱。候选站=。未核验到具体印谱卷次、印文图像、藏印者或著录页。</t>
         </is>
       </c>
     </row>
@@ -25312,22 +25312,22 @@
       </c>
       <c r="G536" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H536" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>四部丛刊</t>
         </is>
       </c>
       <c r="I536" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>庾信《庾子山集》所收志文；夫人拓跋氏附见。</t>
         </is>
       </c>
       <c r="J536" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 母项为《庾子山集》。识典古籍四部丛刊本已提取志文及铭。原表已有该网址，本轮核验正文并归档。</t>
         </is>
       </c>
     </row>
@@ -25353,7 +25353,7 @@
       </c>
       <c r="F537" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://www.mdpi.com/2077-1444/17/3/369</t>
         </is>
       </c>
       <c r="G537" s="10" t="inlineStr">
@@ -25373,7 +25373,7 @@
       </c>
       <c r="J537" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 线索：北周建德元年錡馬仁造老君像碑，与北魏正光二年《锜麻仁合家造象记》非同一石。识典鲁迅辑校石刻手稿仅见后者 https://www.shidianguji.com/book/7563224556832292891/chapter/1lx2cd4f5r19v ；建德元年碑全文录文未取得，故仍记未找到。；2026-09-21 gpt-6-astra：仅线索。类型=北朝造像碑刻。关键词=北周 建德元年 锜马仁 造像记、北周建德元年錡馬仁造老君像碑、錡马仁 造像、錡麻仁 合家 造象记、572 造像碑。母项=北朝佛教造像碑刻汇编、《鲁迅辑校石刻手稿》相关石刻条目、北周造像记、道教造像碑及地方金石志。候选站=https://www.mdpi.com/2077-1444/17/3/369; https://www.shidianguji.com/book/7563224556832292891/chapter/1lx2cd4f5r19v。已知研究线索明确区分北周建德元年碑与北魏正光二年《錡麻仁合家造象记》。目前未取得北周碑的完整原始录文或可靠拓片页面。；2026-09-21 gpt-6-astra：仅线索。类型=北朝造像碑刻。关键词=北周建德元年 锜马仁、錡马仁造像记、錡马仁造老君像碑、572造像碑。母项=北朝造像碑刻汇编、《鲁迅辑校石刻手稿》、地方金石志。候选站=https://www.shidianguji.com/book/7563224556832292891/chapter/1lx2cd4f5r19v。该章节不是目标碑的全文录文，未找到北周建德元年碑的具体公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=北朝造像碑刻。关键词=北周建德元年 锜马仁、錡马仁造像记、錡马仁造老君像碑、572造像碑、北周 造像记。母项=北朝造像碑刻汇编、地方金石志、《鲁迅辑校石刻手稿》相关石刻条目。候选站=https://www.shidianguji.com/book/7563224556832292891/chapter/1lx2cd4f5r19v。已知识典章节对应另一方碑刻，未找到北周建德元年(572)《錡马仁造像记》的具体公开全文页、录文页或方志卷URL。</t>
         </is>
       </c>
     </row>
@@ -25399,12 +25399,12 @@
       </c>
       <c r="F538" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://www.shidianguji.com/book/NLG312001065669</t>
         </is>
       </c>
       <c r="G538" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H538" s="10" t="inlineStr">
@@ -25414,12 +25414,12 @@
       </c>
       <c r="I538" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>道光《榆林府志》艺文志御制诗；康熙三十六年出幸榆林。</t>
         </is>
       </c>
       <c r="J538" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑为现代研究文章、章节标题或史料内容概括。关键词=康熙三十六年 榆林 巡幸、康熙三十六年 榆林 巡幸 御制诗、康熙三十六年 榆林 认识、康熙三十六年 榆林 認識、清圣祖 1697 榆林、清聖祖 榆林 塞外。母项=《清圣祖实录》：优先检查康熙三十六年有关榆林行程、谕旨的条目；具体卷次待核、《圣祖仁皇帝御制文集》及御制诗相关编次：检查榆林题咏、序文；具体集次待核、榆林地方志。候选站=。未找到可核验的文章页或章节页。本题名带有现代研究表述特征，不宜直接认作康熙原文篇名。1697年仅为康熙三十六年的公历检索辅助信息。先查原清单引用出处、作者及页码，再用实录和御制诗文交叉定位；以上母项均为待查方向，不表示已经确认收录。；2026-09-21 条目为史事/认识子项。母项道光《榆林府志》艺文志御制诗已核：康熙三十六年圣祖平噶尔丹出幸榆林，录《河套西望》《出塞》。已从本轮识典抽出的府志文本摘录，不替代专论。</t>
         </is>
       </c>
     </row>
@@ -25465,7 +25465,7 @@
       </c>
       <c r="J539" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代地方官奏折。关键词=陕西巡抚 鄂海 万寿亭 碑文、鄂海奏请建造万寿亭、鄂海 修改碑文、陕西 万寿亭 奏折、万寿亭碑文 清代陕西。母项=《宫中档乾隆朝奏折》、《军机处录副奏折》中的陕西地方工程及碑刻档案、陕西地方志、府县志及万寿亭碑刻资料。候选站=。应按鄂海任陕西巡抚的年代、奏折年月和万寿亭所在地检索。题名可能是档案目录拟题，未找到可核验的具体档号或全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代地方官奏折。关键词=陕西巡抚 鄂海 万寿亭、鄂海 修改碑文、万寿亭奏折。母项=《宫中档乾隆朝奏折》、《军机处录副奏折》、陕西府县志、陕西金石志。候选站=。未找到具体奏折卷次、方志卷或可核验公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代奏折。关键词=陕西巡抚鄂海、万寿亭、修改碑文、建造万寿亭、陕西碑刻。母项=《宫中档乾隆朝奏折》、《军机处录副奏折》、陕西府县志、陕西金石志。候选站=。未找到可核验的识典章节、维基文库卷次、墓志录文页或方志卷 URL。</t>
         </is>
       </c>
     </row>
@@ -25511,7 +25511,7 @@
       </c>
       <c r="J540" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑为抗战时期报刊文章、宣传文字或后编史料标题。关键词=鼓动 回族同胞 抗战、鼓動 回族同胞 抗戰、鼓励 回教同胞 抗战、鼓勵 回教同胞 抗戰、动员 回民 抗日、回教救国 抗战 宣传。母项=《月华》：优先检查1937—1945年可得期刊的目录及抗战宣传栏目、《回教救国协会会刊》：先核刊名沿革及存刊年期，再查动员、宣传类文章、中国回教救国协会相关档案。候选站=。未找到具体文章页，作者、刊名及年期尚未核定。检索不能只用现代民族名称“回族”，应同时使用当时常见的“回教”“回民”。“鼓动”也可能是汇编者拟定的内容摘要。所列刊物和档案仅为待查母项，不代表收录关系已证实。；2026-09-21 gpt-6-astra：未找到。类型=疑似抗战宣传文章或史料摘要。关键词=鼓动回族同胞抗战、鼓動回族同胞抗戰、回教同胞 抗戰、回民 动员 抗日、鼓动 回教 救国。母项=《月华》（待核，未证实收录）。候选站=。当前无法联网核验。作者、刊载年月及卷期均未确认；“回教”“回民”仅作为扩展检索词，不视为已证实异题。无具体文章页URL。；2026-09-21 gpt-6-astra：未找到。类型=抗战时期报刊文章、宣传文字或史料摘要。关键词=鼓动回族同胞抗战、鼓動回族同胞抗戰、回教同胞抗战、回民动员抗日、回教救国抗战。母项=《月华》、《回教救国协会会刊》、中国回教救国协会档案。候选站=。未核得作者、刊名、刊载年月、卷期或具体文章页；题名可能是后来的内容摘要。</t>
         </is>
       </c>
     </row>
@@ -25537,12 +25537,12 @@
       </c>
       <c r="F541" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://www.shidianguji.com/book/SK2783/chapter/1kf4dcej15q1m</t>
         </is>
       </c>
       <c r="G541" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H541" s="10" t="inlineStr">
@@ -25552,12 +25552,12 @@
       </c>
       <c r="I541" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>元虞集《道园学古录》卷十八《贺丞相墓志铭》；识典四库本。</t>
         </is>
       </c>
       <c r="J541" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似墓葬名称、墓志简称或考古报告子项，不能确认为独立书籍。关键词=贺胜墓、賀勝墓、贺胜 墓志、賀勝 墓誌銘、贺胜 神道碑、贺胜 墓葬 发掘 简报。母项=待确定墓主时代与墓址后，查所在地府县志的陵墓、冢墓、金石门、待确认是否为出土材料后，查墓葬发掘简报、墓志汇编及碑刻录文。候选站=。未找到可核验的具体页面，不能据题名指定墓主或卷次。应先从原引文提取朝代、地点、出土时间及拓片编号，再检索识典古籍、维基文库中的地方志章节、墓志录文站与Commons拓片文件页；现代发掘报告仅列书目、馆藏或DOI线索，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=墓葬、墓志或考古报告子项。关键词=贺胜墓、賀勝墓、贺胜墓志、賀勝墓誌、贺胜神道碑、贺胜墓葬。母项=所在地府县志陵墓卷、地方志金石卷、墓志汇编、墓葬发掘简报。候选站=。未核验到墓主时代、地点或具体墓志录文页，不能据题名指定方志卷次。；2026-09-22 条目为贺胜墓。母项虞集《道园学古录》卷十八《贺丞相墓志铭》已从识典四库本抽出全文。墓主贺胜字贞卿，小字伯颜/巴延，泰定追封秦国公谥惠愍。拓片页另见书法网，不作正文。</t>
         </is>
       </c>
     </row>
@@ -25583,12 +25583,12 @@
       </c>
       <c r="F542" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://www.xiaoxiong360.com/shuhua/shiwen/3105.html</t>
         </is>
       </c>
       <c r="G542" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H542" s="10" t="inlineStr">
@@ -25598,12 +25598,12 @@
       </c>
       <c r="I542" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>隋开皇十一年葬；墓主赵惠字世摸。录文亦见《隋代墓誌銘彙考》《長安新出墓誌》。</t>
         </is>
       </c>
       <c r="J542" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 核为《隋赵惠墓志》/《赵世摸墓志》。已保存释文。母项线索：《隋代墓誌銘彙考》《長安新出墓誌》。</t>
         </is>
       </c>
     </row>
@@ -25696,7 +25696,7 @@
       </c>
       <c r="J544" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑为档案组合标题或公文内容摘要。关键词=报送 审查 蒙藏委员会、報送 審查 蒙藏委員會、呈送 核准 蒙藏委员会、呈送 核備 蒙藏委員會、蒙藏委 呈 函 附件、蒙藏委员会 回教 审查。母项=民国蒙藏委员会机关档案：检查收发文、呈报及审查类案卷、国民政府公报及蒙藏委员会相关公报：仅在文件属于公开公布事项时适用、回族、伊斯兰教近代档案史料汇编：检查涉及。候选站=。未找到具体档案目录页。“相关公文”表明它可能概括数件文件，不能作为独立书名处理。需从原引用补出报送事项、发文机关、日期、文号或档号；子项应以“发文机关＋受文机关＋事由＋日期”定位。目前无法负责任地指定汇编卷次或档案页。；2026-09-21 gpt-6-astra：未找到。类型=疑似档案组合标题。关键词=报送 审查 蒙藏委员会、報送 審查 蒙藏委員會、呈送 核备 蒙藏委员会、蒙藏委 公文 附件。母项=蒙藏委员会机关档案（待核）、《国民政府公报》（待核，未证实收录）。候选站=。当前无法联网核验。题名缺少报送事项、发文机关、日期和文号，不能据此指定公报期次、汇编章节或方志卷URL。；2026-09-21 gpt-6-astra：未找到。类型=档案组合标题或公文内容摘要。关键词=报送审查蒙藏委员会、報送審查蒙藏委員會、呈送核准蒙藏委员会、蒙藏委员会公文、蒙藏委审查。母项=蒙藏委员会机关档案、《国民政府公报》、近代蒙藏事务档案汇编。候选站=。题名缺少发文机关、受文机关、报送事项、日期和文号，未能定位公报期次、档案案卷或汇编卷次。</t>
         </is>
       </c>
     </row>
@@ -25742,7 +25742,7 @@
       </c>
       <c r="J545" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似查海遗址第8号墓编号，较可能是考古报告中的子项。关键词=查海 M8、查海 M８、查海 M 8 墓葬、查海 八号墓、查海 八號墓、查海遗址 第8号墓。母项=《查海：新石器时代聚落遗址发掘报告》（优先核验的母项；M8所在册次、页码及图版号未确定）、查海遗址历次发掘简报（需依据发掘年度确定具体篇名和期次）。候选站=。未找到M8对应的具体页面。编号M8可能随发掘区或年度分别编排，须核对原引文中的年份、区号、页码及图号。优先查报告目录、墓葬登记表、墓葬平剖面图与图版说明，不能把报告书名命中当作M8已定位。现代报告只提供书目、馆藏或DOI线索，不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=考古报告中的墓葬编号。关键词=查海M8、查海 M 8、查海八号墓、查海八號墓、查海遗址第8号墓。母项=《查海：新石器时代聚落遗址发掘报告》、查海遗址发掘简报、查海遗址考古报告。候选站=。未核验到M8对应的发掘年度、发掘区、页码或图版。现代考古报告仅可继续查书目、馆藏或DOI。</t>
         </is>
       </c>
     </row>
@@ -25788,7 +25788,7 @@
       </c>
       <c r="J546" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑为考古报告中的墓地章节、遗址条目或合并引文。关键词=前屯 洼浑木 墓地、前屯 窪渾木 墓地、洼浑木 墓葬 发掘、窪渾木 墓葬 發掘、前屯 墓地 发掘简报、洼浑木 考古 地名。母项=《考古》《文物》《考古学报》的墓葬发掘报告目录：年份及期次待定、所在地文物志、考古调查报告和墓葬资料汇编：须先确定“洼浑木”对应地名、包含多个墓地的区域考古报告。候选站=。未找到具体报告页，无法确认两处墓地的地域及年代。优先核对“洼浑木”原始字形，排除转录或OCR错误；不能擅自换成相近地名。先检索较少见的“洼浑木”，再以“前屯”交叉确认。现代报告及仍在版权期的整理本仅提供书目、馆藏或DOI线索，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=疑似考古报告章节或墓地条目。关键词=前屯 洼浑木 墓地、前屯 窪渾木 墓地、洼浑木 墓葬、前屯 发掘 简报。母项=所在地文物志或考古调查报告（地域及书名待核）。候选站=。当前无法联网核验。“洼浑木”原始字形、墓地所在地及报告作者均未确认，不擅自改作相近地名。墓地报告不能直接等同墓志录文；现代版权报告不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=考古报告章节、遗址条目或墓地调查记录。关键词=前屯、洼浑木、前屯洼浑木墓地、洼浑木墓葬、前屯墓地发掘。母项=所在地文物志、区域考古调查报告、墓葬资料汇编、《考古》、《文物》、《考古学报》。候选站=。未核得墓地所在地、年代、报告名称、作者、卷期或具体章节页；“洼浑木”字形及其是否为OCR或转录异文仍待核对。</t>
         </is>
       </c>
     </row>
@@ -25926,7 +25926,7 @@
       </c>
       <c r="J549" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代地方官奏折。关键词=伯兴 严禁私藏鸟枪、伯兴奏报鸟枪、私藏鸟枪 奏折、清代 禁枪 鸟枪 伯兴、伯兴奏报严禁私藏鸟枪情形。母项=《宫中档乾隆朝奏折》或嘉庆朝奏折、《军机处录副奏折》中的枪械禁令、地方治安档案、清代刑科题本及地方治安档案汇编。候选站=。“伯兴”需先核定职衔、任职地区和年代；同名官员可能较多。题名应结合“鸟枪”“私藏”“查禁”等关键词检索档案目录。；2026-09-21 gpt-6-astra：未找到。类型=清代地方官奏折。关键词=伯兴 严禁私藏鸟枪、伯兴奏报鸟枪、私藏鸟枪奏折。母项=《宫中档乾隆朝奏折》、《军机处录副奏折》、清代刑科题本、地方治安档案。候选站=。未核定伯兴的任职地区与年代，未找到具体奏折卷次或公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代奏折。关键词=伯兴、严禁私藏鸟枪、私藏鸟枪、鸟枪禁令、奏报。母项=《宫中档乾隆朝奏折》、《军机处录副奏折》、清代刑科题本、地方治安档案。候选站=。“伯兴”的职衔、任职地区和年代仍未核定，未找到具体卷次或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -25972,7 +25972,7 @@
       </c>
       <c r="J550" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑为民国选举档案中的公文组或案由。关键词=为催送回民选举名册由、為催送回民選舉名冊由、催送 回民 选举 名册、催送 回民 選舉 名冊、回民 代表 选举 名册、回教 选举人 名册 呈送。母项=民国国民大会代表选举相关档案：作为待验证的选举类型检索、民国地方政府选举事务档案：检查催报名册、选举人登记及回民代表案卷、回族近代政治参与史料汇编：检查选举文件。候选站=。未找到具体档案页。“为……由”属于公文事由格式，“相关公文”可能是清单编者添加。不能仅凭“回民选举”断定为某届国民大会选举。定位需要年份、行政区域、发受文机关及选举类型；取得这些信息后再核档号、正文和所附名册。；2026-09-21 gpt-6-astra：未找到。类型=疑似选举事务档案案由。关键词=为催送回民选举名册由、為催送回民選舉名冊由、催送 回民 名册、回教 选举人 名册、回民代表 选举 呈送。母项=民国地方政府选举事务档案（待核）。候选站=。当前无法联网核验。未确认选举类型、年度、行政区域和发受文机关，无可指定的档案正文页或方志卷URL；不能径定为国民大会代表选举文件。；2026-09-21 gpt-6-astra：未找到。类型=疑似选举事务档案案由。关键词=催送 回民 选举 名册、催送 回民 選舉 名冊、回教 选举人 呈送。母项=地方政府选举事务档案（归属待核）。候选站=。本轮无可用联网检索工具，未能新增核验具体页面。年份、地域、发受文机关及选举类型均不明，无法指定章节或方志卷URL。</t>
         </is>
       </c>
     </row>
@@ -26018,7 +26018,7 @@
       </c>
       <c r="J551" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑为报刊新闻标题、并列新闻摘要或地方行政史料子项。关键词=注重回民教育 减收回屠捐税、注重回民教育 減收回屠捐稅、回民教育 回屠、回屠 捐税 减收、回屠 捐稅 減免、回民教育 屠宰税。母项=《月华》：检查国内新闻、地方消息及教育相关栏目，年期待核、民国地方报纸及政府公报：检查回民教育经费、屠宰捐税减免消息、所在地财政志、教育志及回族史料汇编：检查税。候选站=。未找到具体新闻页或公文页。题名可能由两个并列小标题连写而成，应分别检索“注重回民教育”和“减收回屠捐税”，再查同版相邻消息。“回屠”原词应保留，不能只替换成“屠宰税”。《月华》仅为待查刊物，尚无确切刊载年期。；2026-09-21 gpt-6-astra：未找到。类型=疑似报刊新闻或并列消息标题。关键词=注重回民教育、减收回屠捐税、減收回屠捐稅、回民教育 回屠、回屠 捐税 减免。母项=《月华》（待核，未证实收录）、所在地财政志、教育志（地域及版本待核）。候选站=。当前无法联网核验。可拆分两个短语定位同版消息，但尚无刊名、年月、卷期或地方信息支持具体URL，不提供推测的方志卷链接。；2026-09-21 gpt-6-astra：未找到。类型=疑似报刊消息或并列标题。关键词=注重回民教育、减收回屠捐税、減收回屠捐稅、回屠 捐税。母项=《月华》（待查，未证实收录）、地方政府公报（刊名待核）。候选站=。本轮无法联网核验。尚无刊期、版次或地域信息，不能提供符合限定的具体章节URL；两个短语是否属于同一标题也未确认。</t>
         </is>
       </c>
     </row>
@@ -26064,7 +26064,7 @@
       </c>
       <c r="J552" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=歧义题名，可能是图书、期刊、单篇文章或章节标题。关键词=人类、人類、人类 书名 作者、人類 雜誌 創刊、人类 目录 章节、人類 譯者 出版。母项=。候选站=。未找到可与本条对应的具体页面。题名过于宽泛，不能任选同名书刊配对。需先取得原引文、作者或译者、出版年代中的至少一项：若为文章，核对期刊年卷期与页码；若为章节，核对母书目录与版本。现代期刊和仍在版权期的著作仅提供书目、馆藏或DOI线索，不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=歧义书名、期刊名或文章题名。关键词=人类、人類、人类 书名、人類 雜誌、人类 目录。母项=。候选站=。题名过于宽泛，未核验到可与本条对应的具体卷次、章节或文章页。仍需作者、译者、年代或原引文。</t>
         </is>
       </c>
     </row>
@@ -26182,12 +26182,12 @@
       </c>
       <c r="F555" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://zh.wikisource.org/wiki/冊府元龜_(四庫全書本)/卷0980</t>
         </is>
       </c>
       <c r="G555" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H555" s="10" t="inlineStr">
@@ -26197,12 +26197,12 @@
       </c>
       <c r="I555" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>《册府元龟》四库本卷九百八十外臣部通好；子项摘录入吐蕃答贺正使。</t>
         </is>
       </c>
       <c r="J555" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 条目为史事子项，非专书。母项《册府元龟》卷九百八十外臣部通好已核四库本：记宝历元年十月成杭、太和二年唐弘实、六年田早、九年李从简、开成元年李景儒等充入吐蕃答贺正使。已摘录对应原文，不替代全书。</t>
         </is>
       </c>
     </row>
@@ -26294,7 +26294,7 @@
       </c>
       <c r="J557" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑为现代考古学论文或论著章节。关键词=西藏高原的旧石器和细石器文化、西藏高原的舊石器和細石器文化、西藏高原 旧石器 细石器、青藏高原 旧石器 细石器 文化、西藏 舊石器 細石器 论文、Tibet plateau palaeolithic microlithic。母项=《考古学报》《考古》《文物》论文目录：先核题名与作者，再确定年期页码、西藏考古研究论文集及史前考古综述：检查旧石器、细石器章节及参考文献。候选站=。未找到可核验的具体论文书目页，作者、年份、期次及DOI均未确认，不填猜测值。优先通过后出综述的参考文献反查原文，再核期刊目录；作者字段一经确认，应使用“作者＋西藏＋细石器”复检。按现代学术文献处理，仅提供书目、馆藏或DOI线索，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=疑似现代考古论文或论著章节。关键词=西藏高原的旧石器和细石器文化、西藏高原的舊石器和細石器文化、西藏高原 旧石器 细石器、青藏高原 细石器 参考文献、Tibet plateau palaeolithic microlithic。母项=西藏史前考古论文集或期刊（具体母项待核）。候选站=。当前无法联网核验。作者、发表年份、卷期页码及DOI均未确认；没有符合本次限定的具体章节URL。按现代学术文献处理，仅可提供核实后的书目、馆藏或DOI线索，不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=疑似现代考古论文或论著章节。关键词=西藏高原 旧石器 细石器、西藏高原 舊石器 細石器、青藏高原 细石器 参考文献。母项=考古学期刊或西藏史前考古论文集（具体母项未确认）。候选站=。本轮无法联网核验，作者、年份及卷期页码仍未确认，无符合限定的章节URL。按现代学术文献处理，仅可提供核实后的书目、馆藏或DOI线索，不可整本下载。</t>
         </is>
       </c>
     </row>
@@ -26325,22 +26325,22 @@
       </c>
       <c r="G558" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H558" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>文物出版社</t>
         </is>
       </c>
       <c r="I558" s="10" t="inlineStr">
         <is>
-          <t>清咸丰十年(1860)敕谕;西藏自治区档案馆藏</t>
+          <t>清咸丰十年(1860)敕谕；汉译文转引自西藏自治区档案馆编《西藏历史档案荟萃》第64号。原件满蒙藏文，西藏自治区档案馆藏。</t>
         </is>
       </c>
       <c r="J558" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 核验原表网址，页面与条目相符，已归档汉译文。原件非汉文，汉译文出自1995年汇编。</t>
         </is>
       </c>
     </row>
@@ -26386,7 +26386,7 @@
       </c>
       <c r="J559" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑为博物馆藏品名称、图录条目或考古报告器物子项。关键词=花鸟纹 玛瑙 盖罐、花鳥紋 瑪瑙 蓋罐、玛瑙盖罐 花鸟、瑪瑙 蓋罐 花鳥、玛瑙 花鸟纹 藏品、玛瑙盖罐 图录 器物号。母项=博物馆藏品数据库及玉石器图录：检查玛瑙器、罐类与花鸟纹分类、出土玉石器相关考古报告：检查随葬品登记表、器物说明和图版目录、Wikimedia Commons器物。候选站=。未找到具体藏品页或图录页，不能将器物名称认作独立书籍。需补出藏馆、年代、尺寸、出土地点或藏品编号，以区分同名器物。若来源为2015年后图录或仍在版权期的著作，仅提供书目、馆藏及合法公开的单件藏品页，不提供整本下载。本次未进行在线页面核验；以上各项均为待执行检索方案，空URL数组表示没有可负责列出的具体候选页。；2026-09-21 gpt-6-astra：未找到。类型=博物馆藏品或考古图录器物条目。关键词=花鸟纹玛瑙盖罐、花鳥紋瑪瑙蓋罐、玛瑙盖罐、瑪瑙蓋罐。母项=博物馆藏品数据库、玉石器图录、考古发掘报告。候选站=。未找到可核验的具体藏品页、图录章节或 Commons 条目。；2026-09-21 gpt-6-astra：未找到。类型=疑似藏品或图录器物条目。关键词=花鸟纹 玛瑙 盖罐、花鳥紋 瑪瑙 蓋罐、玛瑙盖罐 图版 器物号。母项=玉石器图录或考古报告（具体母项未确认）。候选站=。本轮无法联网核验。藏馆、器物编号、出土地及图录版本均不明，无符合限定的具体章节或方志卷URL；不能将器物名称直接认定为文献题名。</t>
         </is>
       </c>
     </row>
@@ -26478,7 +26478,7 @@
       </c>
       <c r="J561" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似文书类型、档案单件标题或文集子篇，不能确认为独立书籍。关键词=执照、執照、執照 給照、執照 印照、执照 档案 文书、執照 契約 文書。母项=待确认签发机关、持照人和年代后，查相应档案汇编或契约文书集、若原引文属于文集，查该集目录中的公牍、告示、文移等类别。候选站=。未找到可核验的具体页面。“执照”可能只是编目者拟定的文书名称。定位应以签发机关、受领人、事由、日期、档号或文书编号为主；影像还应核对印章和首尾文字。未获得这些信息前无法给出可靠母项或卷次。2015年后整理本及仍在版权期的汇编仅列书目、馆藏线索，不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=文书或档案单件。关键词=执照、執照、給照、印照、执照 文书、執照 文書。母项=地方档案汇编、契约文书集、公牍文书汇编。候选站=。题名过于通用，缺少签发机关、年代、持照人、事由或档号，无法锁定具体卷页。</t>
         </is>
       </c>
     </row>
@@ -26570,7 +26570,7 @@
       </c>
       <c r="J563" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代题本或档案目录拟题，非独立书籍。关键词=精河 屯田 丰稔、精河 屯田 议叙、精河 屯田 議敘、范时绶 头等侍卫、范時綬 頭等侍衛。母项=中国第一历史档案馆藏内阁题本目录（待查，归属未确认）、《清高宗实录》屯田收获及官员议叙相关日条（待查，朝代及卷次须先由档案日期确认）、《清代新疆满文档案汇编》相。候选站=。未找到可核验的具体目录页或全文页；未完成在线检索。先以范时绶与精河交叉检索，取得具奏人、日期、档号后，再查对应题本及实录日条。目录题名可能由整理者拟定，不宜按古籍书名检索。实录即使有同事记载，也不等于该题本原文。现代档案整理本仅查书目、馆藏及档号，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=清代题本或档案目录子项。关键词=精河屯田收获丰稔、精河屯田议叙、范时绶、范時綬、头等侍卫。母项=清代内阁题本目录、清高宗实录、清代新疆档案汇编。候选站=。未找到具体档案目录页、实录卷次或公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=疑似清代题本目录拟题。关键词=精河 屯田 丰稔、精河 屯田 豐稔、范时绶 议叙、范時綬 議敘 頭等侍衛。母项=清代内阁题本（归属待核）、《清高宗实录》（仅待查相关记载）。候选站=。本轮无法联网核验。未取得具奏人、日期或档号，无法确定实录卷次；即使存在同事记载，也须另核是否包含该题本原文。</t>
         </is>
       </c>
     </row>
@@ -26616,7 +26616,7 @@
       </c>
       <c r="J564" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代财政核销题本或档案目录拟题。关键词=喀什噶尔 伯克 核销、喀什噶爾 伯克 核銷、赏赉 变价 绸缎、賞賚 變價 綢緞、喀什噶尔 奏销 赏银。母项=中国第一历史档案馆藏内阁题本目录之财政、边疆事务相关条目（待查，归属未确认）、《清代新疆满文档案汇编》赏赉、伯克及财政核销相关目录（待查，未确认收录）。候选站=。未找到可核验的具体页；未完成在线检索。先查伯克、赏赉、变价绸缎等组合，补查喀什噶尔／喀什噶爾及喀什作为地名检索词。须取得具奏人、年月、银两数或档号，才能定位母项册次。不要把制度史中相似的赏赉记录认作同一档案。现代整理本仅提供书目与馆藏线索，不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=清代财政题本或档案目录子项。关键词=喀什噶尔赏赉、喀什噶爾賞賚、伯克变价绸缎、伯克變價綢緞、核销赏赉。母项=清代内阁题本目录、清代新疆财政档案汇编。候选站=。未找到具体档案目录页、卷册页或公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=疑似清代财政核销题本目录拟题。关键词=喀什噶尔 伯克 核销、喀什噶爾 伯克 核銷、赏赉 变价 绸缎、賞賚 變價 綢緞。母项=清代内阁题本（归属待核）、清代新疆财政档案（具体汇编未确认）。候选站=。本轮无法联网核验。具奏人、年月、银两数及档号均未确认，无可核验的具体章节或卷次URL。现代档案整理本不可整本下载。</t>
         </is>
       </c>
     </row>
@@ -26662,7 +26662,7 @@
       </c>
       <c r="J565" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代寄信上谕或军机处档案子项。关键词=舒赫德 暂理 哈什噶尔、舒赫德 暫理 哈什噶爾、舒赫德 喀什噶尔 参赞、舒赫德 喀什噶爾 寄諭、舒赫德 暂管 喀什噶尔。母项=中国第一历史档案馆藏军机处寄信档、上谕档目录（待查，具体档册未确认）、《清高宗实录》舒赫德办理回疆事务相关日条（待查，卷次未确认）、《钦定平定准噶尔方略》正编、。候选站=。未找到可核验的具体章节或档案页；未完成在线检索。哈什噶尔与喀什噶尔应并查；暂理还可扩展检索暂管、管理，但不能视为已确认的原文异文。优先在识典古籍、维基文库的上述古籍具体书目内检索舒赫德，再按上谕年月反查档册。不得由相似人物活动直接推定卷次。；2026-09-21 gpt-6-astra：未找到。类型=清代寄信上谕或军机处档案子项。关键词=舒赫德暂理哈什噶尔、舒赫德暫理哈什噶爾、舒赫德喀什噶尔、参赞大臣舒赫德。母项=清高宗实录、钦定平定准噶尔方略、军机处寄信档。候选站=。未找到可核验的识典章节、维基文库卷次或档案条目页。；2026-09-21 gpt-6-astra：未找到。类型=疑似清代寄信上谕档案子项。关键词=舒赫德 暂理 哈什噶尔、舒赫德 暫理 哈什噶爾、舒赫德 喀什噶爾 參贊、舒赫德 暂管 喀什噶尔。母项=《清高宗实录》（待核）、《钦定平定准噶尔方略》（待核）、军机处寄信档（档册待核）。候选站=。本轮无法联网核验，未确认上谕年月及对应卷次，不能据人物与地名猜填维基文库或识典章节URL。“暂管”仅为扩展检索词，并非已确认异文。</t>
         </is>
       </c>
     </row>
@@ -26708,7 +26708,7 @@
       </c>
       <c r="J566" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代寄信档或军机处寄谕。关键词=福康安 伊犁官马 内地暂不购马、寄谕陕甘总督福康安、查奏伊犁官马用于何项、伊犁官马 购马 寄谕、陕甘总督 福康安 马政。母项=《清代军机处档案辑录》中的寄信档、寄谕档、《宫中档乾隆朝奏折》、《清高宗实录》相关乾隆朝伊犁马政、陕甘军政条目、新疆地方档案及清代马政档案汇编。候选站=。属于档案目录标题或谕旨单件，不是独立出版物。应以乾隆末年至嘉庆初年、福康安任陕甘总督时期及伊犁马政专题检索，现无可核验具体全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代军机处寄谕。关键词=福康安 伊犁官马、陕甘总督 福康安、内地暂不购马、伊犁官马用途。母项=《清代军机处档案辑录》、《清高宗实录》、清代马政档案汇编。候选站=。未找到具体寄谕卷次、实录卷次或可核验公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代军机处寄谕。关键词=福康安、伊犁官马、内地暂不购马、陕甘总督、马政。母项=《清代军机处档案辑录》、《清高宗实录》、清代马政档案汇编。候选站=。未找到可核验的具体寄谕卷次、实录卷次或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -26754,7 +26754,7 @@
       </c>
       <c r="J567" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代宫中档奏折。关键词=乾清门四等侍卫 阿敏道、巴里坤军营、巴尔虎八旗、谢赏刀枪马匹、恩折、阿敏道奏折。母项=清代宫中档奏折、宫中档乾隆朝奏折、中国第一历史档案馆清代档案目录、《清代新疆满文档案汉译编译》相关巴里坤军务档案。候选站=。未取得可核验的具体档号、卷次或公开全文页。检索时应同时使用“巴里坤／巴里坤军营”“巴尔虎／巴尔虎八旗”“阿敏道”“刀枪马匹”等组合，并核对满文档案汉译题名。；2026-09-21 gpt-6-astra：未找到。类型=清代奏折。关键词=阿敏道、巴里坤军营、巴尔虎八旗、谢赏刀枪马匹、恩折。母项=清代宫中档奏折、乾隆朝军机处档折件、清代新疆满文档案汉译编译。候选站=。未找到可核验的具体档号、卷次或公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代奏折。关键词=阿敏道、巴里坤军营、巴尔虎八旗、谢赏刀枪马匹、恩折。母项=清代宫中档奏折、乾隆朝军机处档折件、《清代新疆满文档案汉译编译》。候选站=。未找到可核验的具体档号、卷次或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -26800,7 +26800,7 @@
       </c>
       <c r="J568" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似考古简报或论文题名，地名组合待校。关键词=山西 石楼 出土 铜器、山西 石樓 出土 銅器、石楼县 青铜器 简报、石樓縣 銅器、吕梁 石楼 商代 铜器。母项=《文物》历年总目及考古简报栏目（待查，未确认收录）、《考古》历年总目（待查，未确认收录）、《考古学报》历年总目（待查，未确认收录）、《石楼县志》文物相关章节（版。候选站=。未找到可核验的论文详情页、作者或年期；未完成在线检索。“吕梁县石楼镇”与现行行政区划不符，应先校核原始引文，不直接改定题名。检索时并用铜器、青铜器、出土、发现，取得作者与页码后核对期刊目录。现代期刊仅提供书目、馆藏或DOI线索，不提供整本下载；器物照片不能代替文章全文。；2026-09-21 gpt-6-astra：未找到。类型=考古简报或现代期刊论文。关键词=石楼镇出土铜器、石樓鎮出土銅器、石楼出土青铜器、吕梁石楼铜器。母项=文物考古简报、考古、考古学报、石楼县志文物卷。候选站=。未找到具体论文详情页、方志卷页或公开全文。题名中的行政区划关系仍需原始出处核对。；2026-09-21 gpt-6-astra：未找到。类型=疑似现代考古简报，题名地名待校。关键词=山西 石楼 出土 铜器、山西 石樓 出土 銅器、吕梁 石楼 青铜器、石楼县 铜器 简报。母项=《文物》《考古》（均待查，未证实收录）、《石楼县志》（版本及相关卷目待核）。候选站=。本轮无法联网核验，无具体论文或方志卷URL。题名中的行政区划须核对原始引文，不能擅自改定。若为现代期刊文章，仅提供核实后的书目、馆藏或DOI线索，不可整本下载。</t>
         </is>
       </c>
     </row>
@@ -26893,7 +26893,7 @@
       </c>
       <c r="J570" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=辽代墓志。关键词=维大金国朔州妙因寺比丘尼大乘座主墓志、朔州妙因寺、比丘尼大乘、大乘座主墓志、金代朔州墓志、妙因寺墓志。母项=《山右石刻丛编》、《八琼室金石补正》、《金石萃编》、山西朔州金代墓志及寺院碑刻汇编。候选站=。未找到可核验的具体碑录页、卷次或墓志录文。应重点查《山右石刻丛编》朔州金代墓志部分及《八琼室金石补正》金代墓志条目，题名可能省略“铭并序”等格式词。；2026-09-21 gpt-6-astra：未找到。类型=金代墓志。关键词=朔州妙因寺、比丘尼大乘、大乘座主墓志、金代朔州墓志。母项=《山右石刻丛编》、《八琼室金石补正》、朔州金代墓志汇编。候选站=。未找到具体墓志录文页、方志卷次或可核验的维基文库章节。；2026-09-21 gpt-6-astra：未找到。类型=金代墓志。关键词=朔州妙因寺、比丘尼大乘、大乘座主、金代朔州墓志、妙因寺墓志。母项=《山右石刻丛编》、《八琼室金石补正》、朔州金代墓志汇编。候选站=。未找到具体墓志录文页、方志卷次或维基文库章节。</t>
         </is>
       </c>
     </row>
@@ -26939,7 +26939,7 @@
       </c>
       <c r="J571" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似民国边务档案提纲或汇编内子项。关键词=外蒙 犯边 提纲、外蒙 犯邊 提綱、外蒙古 犯边案、外蒙古 犯邊案、外蒙 边务 提纲。母项=中国第二历史档案馆相关边务、蒙藏事务档案目录（待查，归属未确认）、中央研究院近代史研究所档案馆外交档案之蒙古、边务相关目录（待查，归属未确认）。候选站=。未找到可核验的档案条目或汇编目录页；未完成在线检索。题名没有年代与责任者，暂不能锁定具体边境事件。先查犯边案提纲，再拆查外蒙、犯边及提纲，记录案卷起讫日期、形成机关、档号和附件关系。不要将泛论外蒙古问题的书籍列作已确认母项。现代档案汇编仅查书目、馆藏和目录，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=民国边务档案或档案汇编子项。关键词=外蒙犯边案提纲、外蒙犯邊案提綱、外蒙古犯边案、外蒙古犯邊案。母项=民国边务档案目录、蒙藏事务档案汇编、外交档案蒙古事务卷。候选站=。未找到具体档案目录页、案卷条目或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -26985,7 +26985,7 @@
       </c>
       <c r="J572" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似日记日期条目、书信日期或报刊日期，不宜视为独立书名。关键词=10月27日、１０月２７日、十月二十七日、十月廿七日、十月二十七日 日记、十月廿七日 日記。母项=待确认作者及年份后，查其日记、日谱、年谱或书信集、若为报刊日期，须先确定报刊名称、年份、版次和文章标题。候选站=。未找到具体日期条目的可核页面。必须补齐年份、作者和母项；还须区分公历与农历，不能将“十月廿七日”直接认定为公历10月27日。识典古籍或维基文库中即使命中相同日期，也须核对年份及前后条目。现代整理本只提供书目、馆藏线索，不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=日记、书信或报刊日期条目。关键词=10月27日、１０月２７日、十月二十七日、十月廿七日、十月二十七日 日记、十月廿七日 日記。母项=日记、日谱、年谱、书信集、报刊。候选站=。缺少作者、年份及母项，无法区分公历日期、农历日期、日记条目或报刊日期。</t>
         </is>
       </c>
     </row>
@@ -27031,7 +27031,7 @@
       </c>
       <c r="J573" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=民国呈文及批令，可能为公报转载子项。关键词=贡桑诺尔布 章嘉 巴拉根加布、貢桑諾爾布 章嘉 巴拉根加布、蒙藏院 接护印务、蒙藏院 接護印務、章嘉 出京 起程 批令。母项=北京政府《政府公报》呈文、批令相关栏目（待查，未确认收录及刊期）、蒙藏院档案目录（待查，保管机构与档号未确认）。候选站=。未找到可核验的公报期页或档案目录页；未完成在线检索。“呈……文并批令”的结构提示可能是公报目录标题，但尚不能确认。优先用巴拉根加布、接护印务两个低频词定位；再以贡桑诺尔布任职时间与章嘉出京日期缩小范围。须分别记录呈文日期、批令日期、公报发行日期和期号，三种日期不能混用。；2026-09-21 gpt-6-astra：未找到。类型=民国蒙藏院呈文及批令。关键词=贡桑诺尔布、貢桑諾爾布、章嘉呼图克图、巴拉根加布、接护印务、起程日期。母项=政府公报、蒙藏院档案、北京政府公报蒙藏院栏目。候选站=。未找到具体公报期页、栏目页或档案目录条目。</t>
         </is>
       </c>
     </row>
@@ -27077,7 +27077,7 @@
       </c>
       <c r="J574" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似地方工商史、文史资料篇目或商号档案条目。关键词=代县 谢家 烟坊 日升号、代縣 謝家 煙坊 日升號、代县 日升号、谢家烟坊、代县 烟草 商号。母项=《代县志》工业、商业或烟草相关章节（版本及收录情况待查）、代县地方政协文史资料之工商史、商号史篇目目录（具体辑名与辑次待查）、山西烟草地方史志及工商档案目录（具。候选站=。未找到可核验的篇目目录、作者或页码；未完成在线检索。先查谢家烟坊与日升号，确认日升号是否为商号名称，而非文章题名。再在县志、地方文史资料目录中定位母项版本、辑次和起止页。日昇號可作补充字形检索词，但不是已确认别名。现代地方文史整理本仅查书目、馆藏和篇目，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=地方商业史或文史资料篇目。关键词=代县谢家烟坊日升号、代縣謝家煙坊日升號、谢家烟坊、日升号、日昇號。母项=代县志商业卷、代县地方文史资料、山西烟草史志。候选站=。未找到具体方志章节、文史资料篇目页或商号档案页。</t>
         </is>
       </c>
     </row>
@@ -27123,7 +27123,7 @@
       </c>
       <c r="J575" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=电报文献或档案汇编中的编者拟题。关键词=赵戴文 齐电 达赖、趙戴文 齊電 達賴、达赖 不亲英 不背中央、達賴 不親英 不背中央、赵戴文 九月八日 班禅 回藏。母项=《西藏地方是中国不可分割的一部分（史料选辑）》民国时期相关目录（待查，未确认收录）、中国第二历史档案馆藏涉藏电报档案目录（待查，归属未确认）、民国蒙藏事务史料汇。候选站=。未找到可核验的具体篇目页或档案页；未完成在线检索。“齐”是韵目代日中八日的标记，不宜当作发电地点；年份仍缺失。破折号后的文字可能是编者内容提要，应与原始电文分别检索。先查不亲英、不背中央等短语，再以发电人、收电人、年份与九月八日核对；未确认年份前不能指定卷册。现代汇编仅提供书目、馆藏及页码线索，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=民国电报或档案汇编子项。关键词=赵戴文、齐电、达赖不亲英不背中央、九月八日、班禅回藏、趙戴文。母项=西藏地方是中国不可分割的一部分（史料选辑）、民国蒙藏事务史料、中国第二历史档案馆涉藏电报档案。候选站=。未核验到具体公开全文页、维基文库卷次或档案影印页；年份及原始档号不足，不能定位卷册。</t>
         </is>
       </c>
     </row>
@@ -27149,7 +27149,7 @@
       </c>
       <c r="F576" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://www.gdwx.fudan.edu.cn/fd/ea/c4127a458218/page.htm</t>
         </is>
       </c>
       <c r="G576" s="10" t="inlineStr">
@@ -27159,17 +27159,17 @@
       </c>
       <c r="H576" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>上海古籍出版社</t>
         </is>
       </c>
       <c r="I576" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>仇鹿鸣、夏婧《五代十国墓志汇编》开运〇一三</t>
         </is>
       </c>
       <c r="J576" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 母项已定位为《五代十国墓志汇编》开运〇一三，公开全文未取得，仍记未找到。；2026-09-21 gpt-6-astra：未找到。类型=五代墓志。关键词=后晋李继忠墓志、李继忠墓志、开运十三、五代十国墓志汇编、晋李继忠墓志。母项=仇鹿鸣、夏婧《五代十国墓志汇编》开运〇一三、《全唐文补编》及五代墓志辑录、《五代墓志汇编》后晋墓志部分。候选站=https://www.gdwx.fudan.edu.cn/fd/ea/c4127a458218/page.htm。母项和条目标识已定位为《五代十国墓志汇编》开运〇一三，但未取得公开可核的完整墓志录文或具体页码。；2026-09-21 gpt-6-astra：找到候选。类型=五代墓志。关键词=后晋李继忠墓志、李继忠墓志、开运十三、五代十国墓志汇编。母项=仇鹿鸣、夏婧《五代十国墓志汇编》开运〇一三、《全唐文补编》五代墓志部分。候选站=https://www.gdwx.fudan.edu.cn/fd/ea/c4127a458218/page.htm。已定位母项及条目标识，但页面未核验出完整墓志录文。；2026-09-21 gpt-6-astra：未找到。类型=五代墓志。关键词=后晋李继忠墓志、李继忠墓志、开运十三、五代十国墓志汇编。母项=《五代十国墓志汇编》开运〇一三、《全唐文补编》五代墓志部分、五代墓志辑录。候选站=。已有母项书目信息，但未找到符合本轮限定的识典章节、维基文库卷次或墓志录文页。；2026-09-22 gpt-6-astra：找到候选。类型=五代墓志。关键词=后晋李继忠墓志、李继忠墓志、开运十三、五代十国墓志汇编。母项=《五代十国墓志汇编》开运〇一三、《全唐文补编》五代墓志部分。候选站=https://www.gdwx.fudan.edu.cn/fd/ea/c4127a458218/page.htm。已定位母项和条目标识，但页面未核验出完整墓志录文。；2026-09-22 gpt-6-astra：仅线索。类型=五代墓志。关键词=后晋李继忠墓志、李继忠墓志、开运十三、五代十国墓志汇编。母项=《五代十国墓志汇编》开运〇一三、《全唐文补编》五代墓志部分。候选站=https://www.gdwx.fudan.edu.cn/fd/ea/c4127a458218/page.htm。页面可定位母项及条目标识，但未核验到完整墓志录文。；2026-09-22 gpt-6-astra：仅线索。类型=五代墓志。关键词=后晋李继忠墓志、李继忠墓志、开运十三、五代十国墓志汇编。母项=《五代十国墓志汇编》开运〇一三、《全唐文补编》五代墓志部分、五代墓志辑录。候选站=https://www.gdwx.fudan.edu.cn/fd/ea/c4127a458218/page.htm。已定位母项和条目标识，尚未取得符合本轮限定的完整墓志录文页。；2026-09-22 gpt-6-astra：仅线索。类型=五代墓志。关键词=后晋李继忠墓志、李继忠墓志、开运十三、五代十国墓志汇编。母项=《五代十国墓志汇编》开运〇一三、《全唐文补编》五代墓志部分、五代墓志辑录。候选站=https://www.gdwx.fudan.edu.cn/fd/ea/c4127a458218/page.htm。已有母项和条目标识，页面不属于可核验的完整墓志录文页。</t>
         </is>
       </c>
     </row>
@@ -27241,27 +27241,27 @@
       </c>
       <c r="F578" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://zh.wikipedia.org/wiki/崔鴻</t>
         </is>
       </c>
       <c r="G578" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H578" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>天津古籍出版社</t>
         </is>
       </c>
       <c r="I578" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>赵超《汉魏南北朝墓志汇编》录文；北魏天平四年合葬。</t>
         </is>
       </c>
       <c r="J578" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 母项《汉魏南北朝墓志汇编》。已核录文并归档。出土线索见《考古学报》1984年第2期《临淄北朝崔氏墓》。</t>
         </is>
       </c>
     </row>
@@ -27307,7 +27307,7 @@
       </c>
       <c r="J579" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=唐代墓志。关键词=唐故袭三恪嗣韩国公、食邑三千户元公、元公墓志铭并序、袭三恪、韩国公墓志、唐代元氏墓志。母项=《全唐文补遗》唐代墓志部分、《唐代墓志汇编》、《千唐志斋藏志》、《新中国出土墓志·陕西卷》相关唐代墓志。候选站=。未找到可核验的具体墓志录文、墓志汇编卷次或识典古籍页面。检索时应以“袭三恪”“嗣韩国公”“食邑三千户”作为连续短语，并反查元氏家族谱系和唐代封爵。；2026-09-21 gpt-6-astra：未找到。类型=唐代墓志。关键词=袭三恪、嗣韩国公、食邑三千户、元公墓志铭并序。母项=《全唐文补遗》、《唐代墓志汇编》、《千唐志斋藏志》、《新中国出土墓志·陕西卷》。候选站=。未找到具体墓志录文页、卷次或识典章节。；2026-09-21 gpt-6-astra：未找到。类型=唐代墓志。关键词=袭三恪、嗣韩国公、食邑三千户、元公墓志铭并序、唐代元氏墓志。母项=《全唐文补遗》、《唐代墓志汇编》、《千唐志斋藏志》、《新中国出土墓志·陕西卷》。候选站=。未找到具体墓志录文页、卷次或识典章节。</t>
         </is>
       </c>
     </row>
@@ -27380,12 +27380,12 @@
       </c>
       <c r="F581" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>https://www.shidianguji.com/book/7549461577028599854/chapter/1lcvz8ltnwv0q</t>
         </is>
       </c>
       <c r="G581" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H581" s="10" t="inlineStr">
@@ -27395,12 +27395,12 @@
       </c>
       <c r="I581" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>清陆增祥《八琼室金石补正续编》卷三十二；识典本。</t>
         </is>
       </c>
       <c r="J581" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 已定位母项，识典见跋文，完整志文未从可核页面抽出，仍记未找到。；2026-09-21 gpt-6-astra：未找到。类型=宋代墓志。关键词=宋仇公著墓志、仇公著墓志、柳子文撰、王同老书、绍圣三年、益都金石记。母项=《益都金石记》、《八琼室金石补正续编》、《山东金石志》宋代墓志部分、柳子文撰、王同老书宋代墓志辑录。候选站=https://www.shidianguji.com/mid-page/7568608946472222746。已定位《益都金石记》《八琼室金石补正续编》母项及识典跋文，但未从公开页面取得完整志文。；2026-09-21 gpt-6-astra：找到候选。类型=宋代墓志。关键词=仇公著墓志、柳子文撰、王同老书、绍圣三年、益都金石记。母项=《益都金石记》、《八琼室金石补正续编》、《山东金石志》。候选站=https://www.shidianguji.com/mid-page/7568608946472222746。已定位识典具体页面及母项，但该页未核验出完整墓志录文。；2026-09-21 gpt-6-astra：找到候选。类型=宋代墓志。关键词=仇公著墓志、柳子文撰、王同老书、绍圣三年、益都金石记。母项=《益都金石记》、《八琼室金石补正续编》、《山东金石志》。候选站=https://www.shidianguji.com/mid-page/7568608946472222746。已定位识典具体页面，但该页未核验出完整墓志录文。；2026-09-22 gpt-6-astra：找到候选。类型=宋代墓志。关键词=仇公著墓志、柳子文撰、王同老书、绍圣三年、益都金石记。母项=《益都金石记》、《八琼室金石补正续编》、《山东金石志》。候选站=https://www.shidianguji.com/mid-page/7568608946472222746。已定位识典具体页面，但页面未核验出完整墓志录文。；2026-09-22 gpt-6-astra：找到候选。类型=宋代墓志。关键词=仇公著墓志、柳子文撰、王同老书、绍圣三年、益都金石记。母项=《益都金石记》、《八琼室金石补正续编》、《山东金石志》。候选站=https://www.shidianguji.com/mid-page/7568608946472222746。已定位识典具体页面，但页面未核验出完整墓志录文。；2026-09-22 gpt-6-astra：仅线索。类型=宋代墓志。关键词=仇公著墓志、宋仇公著墓志、柳子文撰、王同老书、绍圣三年、益都金石记。母项=《益都金石记》、《八琼室金石补正续编》、《山东金石志》。候选站=https://www.shidianguji.com/mid-page/7568608946472222746。未找到可核验的完整墓志录文页。；2026-09-22 条目为宋仇公著墓志。母项《八琼室金石补正续编》卷三十二《仇公著墓志铭》已从识典抽出全文。柳子文撰、王同老书、晁端德篆；绍圣三年四月卒，十月葬青州云门里。跋另见《金石三编》。</t>
         </is>
       </c>
     </row>
@@ -27446,7 +27446,7 @@
       </c>
       <c r="J582" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代官员题名、题刻或档案条目。关键词=山东通省督粮道 明德、山东督粮道 明德、督粮监兑道 明德、山东通省督粮监兊道、监兑道 明德。母项=《山东通志》清代各修本、《清实录》、《清代职官年表》、山东地方碑刻、档案汇编。候选站=。“监兊”疑为“监兑”异写或识读误差。应先按明德的姓氏、任职年代和督粮道建置，在《山东通志》职官表及清代档案目录中反查；目前未找到可核验的具体全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代职官或方志条目。关键词=山东通省督粮道、山东督粮道明德、督粮监兑道、监兊道、明德。母项=山东通志职官志、清代山东职官表、清实录、山东地方碑刻资料。候选站=。未核验到具体方志卷页或墓志录文页；“监兊”与“监兑”的异文关系及明德姓氏、任职年代均未确定。</t>
         </is>
       </c>
     </row>
@@ -27538,7 +27538,7 @@
       </c>
       <c r="J584" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=近代军事史、炮台遗址图录或专题论文。关键词=清 大沽口炮台、大沽口炮台 清代、大沽炮台、大沽口海防炮台、大沽口炮台遗址。母项=《中国文物地图集·天津分册》、天津市文物志、天津市志·文物卷、《近代中国海防史》相关章节、清代海防档案与甲午战争档案汇编。候选站=。题名更像文物图录、展览图录或图片说明，而非独立古籍。可按炮台名称、炮台遗址及大沽海防等词在天津地方志、文物普查资料和近代海防论文中定位；目前未找到具体开放全文页。；2026-09-21 gpt-6-astra：未找到。类型=近代军事史或文物图录条目。关键词=清大沽口炮台、大沽口炮台、大沽炮台、大沽口海防炮台、大沽炮台遗址。母项=中国文物地图集·天津分册、天津市文物志、天津市志·文物卷、清代海防档案汇编。候选站=。未核验到具体方志卷或公开图录页；题名更像文物图录、展签或图片说明。</t>
         </is>
       </c>
     </row>
@@ -27584,7 +27584,7 @@
       </c>
       <c r="J585" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古发掘报告或墓葬专题论文。关键词=茂县 牟托一号石棺墓、牟托一号石棺墓、茂县牟托 石棺墓、牟托石棺墓、牟托墓地。母项=《四川文物》考古发掘与研究论文、四川省文物考古研究院发掘简报、茂县牟托墓地考古报告、四川石棺葬研究论文集。候选站=。题名很可能是发掘简报或报告中的墓葬分项，而非独立出版物。检索时应同时查“牟托墓地”“石棺葬”“茂县”及《四川文物》相关年份；目前未找到具体开放全文页。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘报告或发掘简报子项。关键词=茂县牟托一号石棺墓、牟托一号石棺墓、牟托墓地、茂县石棺墓、石棺葬。母项=四川文物相关考古发掘简报、茂县牟托墓地考古报告、四川石棺葬研究、四川省文物考古研究院发掘资料。候选站=。未核验到具体期刊篇页、墓葬报告章节或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -27630,7 +27630,7 @@
       </c>
       <c r="J586" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古出土器物图录或器物研究条目。关键词=金沙遗址 出土 陶盏、金沙遗址 陶盏、成都金沙 陶盏、金沙遗址陶器、金沙遗址出土陶器。母项=《成都金沙遗址出土文物》、《金沙遗址》考古发掘报告、金沙遗址博物馆藏品图录、《四川文物》金沙遗址发掘与器物研究论文。候选站=。更可能是博物馆图录中的器物名称、展签或图版说明。应按“器物分类—陶器—盏”在金沙遗址发掘报告及藏品图录中定位；目前未找到具体开放全文页。；2026-09-21 gpt-6-astra：未找到。类型=考古器物图录或发掘报告器物条目。关键词=金沙遗址出土陶盏、金沙遗址陶盏、成都金沙陶盏、金沙遗址陶器、金沙遗址出土陶器。母项=成都金沙遗址出土文物、金沙遗址考古发掘报告、金沙遗址博物馆藏品图录、四川文物金沙遗址器物研究。候选站=。未核验到具体器物图版、目录页或公开全文章节；题名可能是图录中的器物名称。</t>
         </is>
       </c>
     </row>
@@ -27722,7 +27722,7 @@
       </c>
       <c r="J588" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代地方公文、札件或档案汇编子项。关键词=道光二十一年 宁远府札、道光二十一年 宁远府、宁远府札、宁远府 公文、道光二十一年 宁远府 文书。母项=《清代四川地方档案汇编》、《清代贵州地方档案史料》、宁远府地方志及衙门档案、《道光宁远县志》或相关府州县志。候选站=。“宁远府”可能指湖南永州宁远相关行政文书，也可能是清代西南地区档案目录中的府名误录；“札”通常是公文类型，不宜按独立书名检索。需结合原始档案的发文机关、收文机关和地点判定；目前未找到具体全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代地方公文或档案汇编子项。关键词=道光二十一年宁远府札、宁远府札、道光二十一年宁远府、宁远府公文、宁远府。母项=清代地方档案汇编、道光宁远县志、宁远府地方志、清代四川或贵州地方档案史料。候选站=。未核验到具体方志卷页、档案影印页或公开全文；“宁远府”所属地域尚不能确定。</t>
         </is>
       </c>
     </row>
@@ -27768,7 +27768,7 @@
       </c>
       <c r="J589" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清末民初官府档案或教育、监狱教习公文。关键词=周善培 习艺藏徒、周善培 卒业 资送出关、习艺藏徒、习艺所 藏徒、卒业资送出关。母项=周善培档案、文集及四川地方档案、清末四川劝学所与习艺所档案、四川省档案馆清末民初档案汇编、清末新政教育与教养机构档案。候选站=。题名句式明显是档案目录或公文摘要。“藏徒”可能是“藏族徒众”“收养徒工”或档案整理者对机构用语的转录，需核对原目录影印件；目前未找到具体开放全文页。；2026-09-21 gpt-6-astra：未找到。类型=清末民初地方行政档案子项。关键词=周善培、习艺藏徒、卒业资送出关、习艺所、资送出关。母项=周善培档案、四川地方档案汇编、清末四川教育与教养机构档案、清末新政档案资料。候选站=。未核验到具体档案目录页或影印全文；“藏徒”原字及机构性质仍需依据原档案核对。</t>
         </is>
       </c>
     </row>
@@ -27814,7 +27814,7 @@
       </c>
       <c r="J590" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清末地方教育行政档案或公文。关键词=学务局 详请 炉城 师范传习所、炉城 师范传习所、学务局 师范传习所、炉城学务局、师范传习所 四川。母项=清末四川学务档案汇编、四川教育史料、四川省志·教育志、清末地方官报及教育公报、炉城地方志、康定地方志相关教育卷。候选站=。“炉城”多指康定旧称，题名应是清末康定地区学务局公文摘要。可进一步查康定、打箭炉、炉城的异名及《四川官报》教育类文书；目前未找到具体开放全文页。；2026-09-21 gpt-6-astra：未找到。类型=清末地方教育行政公文子项。关键词=学务局详请炉城师范传习所、炉城师范传习所、打箭炉师范传习所、康定学务局、师范传习所。母项=清末四川学务档案汇编、四川教育史料、四川官报、康定地方志教育志、打箭炉厅志。候选站=。未核验到具体方志卷、官报页或档案影印页；炉城应与康定、打箭炉互检，但现有线索不足以锁定页面。</t>
         </is>
       </c>
     </row>
@@ -27860,7 +27860,7 @@
       </c>
       <c r="J591" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=待核题名，可能为涉康藏记述、单篇文章或汇编子项。关键词=炉藏近闻、爐藏近聞、炉藏 近闻、爐藏 近聞、爐藏近聞 作者 目錄、炉藏近闻 康藏。母项=待核方向：康藏、川边及西藏史地文献汇编的篇目目录，尚未确认具体母项、待核方向：近代涉藏报刊文章目录，尚未确认刊名及年期。候选站=。未找到可核验的书目记录或具体正文页面，不能指定作者、版本或卷次。“炉”可能涉及打箭炉，但这里只作为待核检索线索。应先用简繁题名查目录，再拆分“炉藏”“近闻”检索，并回看原始书影排除题名转录或OCR错误；不将未经证实的相近题名列为别名。若收于2015年后整理本，仅提供该本书目、馆藏及子项页码线索，不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=涉藏史地文章或文集子篇。关键词=炉藏近闻、爐藏近聞、炉藏 近闻、爐藏 近聞、打箭炉 近闻、康藏 近闻。母项=康藏史地文献汇编、川边史地文献、涉藏报刊。候选站=。未找到可核验的具体识典章节、维基文库卷次、方志卷页或录文页；题名可能存在转录或OCR误差。</t>
         </is>
       </c>
     </row>
@@ -27906,7 +27906,7 @@
       </c>
       <c r="J592" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=民国地方行政档案或县政决议案。关键词=雷波县 狮子村 区署、狮子村 汉夷杂居、雷波县 改设区署、雷波县决议案、汉夷杂居区域 行政区划。母项=民国雷波县政府档案、《雷波县志》行政区划、民族事务卷、四川省政府公报及县政档案汇编、民国四川地方行政档案。候选站=。题名是现代档案整理者拟定的案卷标题，可能属于县参议会、县政府或四川省政府档案中的单件决议。应以“狮子村”“改设区署”“汉夷杂居”“雷波县政府”组合检索，并核对民国时期“夷”字写法；目前未找到具体开放全文页。；2026-09-21 gpt-6-astra：未找到。类型=民国地方行政档案或县政决议案。关键词=雷波县狮子村、改设区署、汉夷杂居、雷波县政府、狮子村区署、雷波县议案。母项=《雷波县志》行政区划卷、民国雷波县政府档案、四川省政府公报、民国四川地方行政档案汇编。候选站=。未找到可核验的识典章节、维基文库卷次、方志卷页或档案全文页。</t>
         </is>
       </c>
     </row>
@@ -27952,7 +27952,7 @@
       </c>
       <c r="J593" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似档案摘要、教育史材料子目或后拟题名。关键词=西康省政府 彝族 学生 升学 补助、西康省政府 夷族 生徒 奖学金、西康省政府 教育厅 边民学生 助学金、西康省政府 教育廳 夷生 升學 津貼、1939—1949 西康 民族教育。母项=《西康省政府公报》：候选母项；检索教育厅呈文、省政府训令及教育经费事项，年期未确认、西康省政府、教育厅相关档案：候选档案群；优先检索1939—1949年学生补助。候选站=。未找到可核验的具体公报期页或档案条目；当前无法进行实时联网核验。题名可能为编者概括，不能据此当作独立书籍。应提取受助学生姓名、就读学校、批准日期和经费数额，再反查原件。历史材料中的“夷族”“夷生”仅作为原文检索词。；2026-09-21 gpt-6-astra：未找到。类型=民国政府教育档案或公报事项。关键词=西康省政府、彝族学生、夷族生徒、升学补助、奖学金、教育厅。母项=《西康省政府公报》、西康省政府教育厅档案、民国西康教育档案汇编。候选站=。未找到具体公报期页、档案条目或公开全文卷页。</t>
         </is>
       </c>
     </row>
@@ -27998,7 +27998,7 @@
       </c>
       <c r="J594" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似回忆录引文或民族习俗材料子目。关键词=岭光电 汉人年、嶺光電 漢人年、岭光电 春节 过年、岭光电 忆往昔 年俗、彝族 土司 汉年 过春节。母项=岭光电《忆往昔——一个彝族土司的自述》：优先核查的候选母项；尚未确认相关章节、页码及所据版本。候选站=。未找到对应引文的具体页。检索时拆开括号内的解释词，分别查“汉人年”“汉年”“春节”，并核查上下文中的地域和时间。候选回忆录属于现代著作，仅提供书目及馆藏检索方向，不提供整本下载；尚不能确认其为原始出处。；2026-09-21 gpt-6-astra：未找到。类型=现代回忆录或民族习俗材料子项。关键词=岭光电、汉人年、汉年、春节、彝族过年、土司年俗。母项=岭光电《忆往昔——一个彝族土司的自述》、凉山彝族社会生活史料、彝族习俗调查资料。候选站=。未找到可核验的具体章节或公开全文页。现代回忆录仅宜继续查书目、馆藏和引文页码。</t>
         </is>
       </c>
     </row>
@@ -28044,7 +28044,7 @@
       </c>
       <c r="J595" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似人物轶事、口述史引文或民族关系史材料子目。关键词=毛筠如 阿普哈萨、毛筠如 涼山 彝人、毛筠如 福禄神、毛筠如 福祿神、阿普哈薩 凉山、毛筠如 岭光电。母项=岭光电《忆往昔——一个彝族土司的自述》：关联人物回忆材料的排查对象，未确认收录此事、凉山地方文史资料中的人物回忆、汉彝交往材料：母项检索方向，具体书名及辑次未确。候选站=。未找到可核验的出处页。“福禄神”可能是编者释义，宜先用姓名与音译称谓交叉检索，再单查姓名；不要未经核对便改写人名或认定音译异体。若命中现代回忆录或文史资料，只记录书目、馆藏和引用页码，不提供受版权保护著作的整本下载。；2026-09-21 gpt-6-astra：未找到。类型=人物轶事或口述史材料子项。关键词=毛筠如、阿普哈萨、阿普哈薩、福禄神、凉山彝人、岭光电。母项=岭光电《忆往昔——一个彝族土司的自述》、凉山地方文史资料、汉彝交往史料。候选站=。未找到墓志录文页、方志具体卷页或其他可核验公开出处。</t>
         </is>
       </c>
     </row>
@@ -28090,7 +28090,7 @@
       </c>
       <c r="J596" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似地方志、调查报告中的风俗材料子目。关键词=九龙县 汉 藏 彝 苗 风俗 民国、九龍縣 漢 藏 夷 苗 風俗、九龙县志 民族 风俗、九龙 夷苗 婚姻 服饰 饮食、西康 九龙县 调查 风俗习惯。母项=《九龙县志》：候选母项；核查民族、风俗及社会生活相关目录，版本与卷次待核、民国西康地方调查材料：候选来源类别；需由“九龙县”与民族称谓组合定位具体报告。候选站=。未找到具体卷页。不能将现代县志中的历史叙述直接认作民国原始记录，应继续追查其引用的旧志、调查报告或档案。“交融”可能是后拟概括，子项宜查通婚、服饰、饮食、语言、节庆。原文中的“苗”究竟指何人群须结合出处判断。；2026-09-21 gpt-6-astra：未找到。类型=地方志或民国调查材料子项。关键词=九龙县、汉藏彝苗、生活习俗、婚姻、服饰、饮食。母项=《九龙县志》民族与风俗卷、民国西康地方调查报告、西康省社会调查资料。候选站=。未找到具体方志卷 URL、章节页或民国调查报告全文页。</t>
         </is>
       </c>
     </row>
@@ -28136,7 +28136,7 @@
       </c>
       <c r="J597" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似商业史、民族调查或地方志中的材料子目。关键词=松潘 回族 行商 藏商 寺庙、松潘 回商 汉商 寺庙商、松潘 回民 行商 喇嘛寺、松潘 藏商 漢商 寺廟商、松潘 商业史 茶 马 帮、松潘县志 商业 民族。母项=《松潘县志》：候选母项；核查商业、民族、宗教相关目录，版本及页码待核、《松潘文史资料》：候选地方文史资料系列；检索回民经商、商帮、寺院贸易，具体辑次待核。候选站=。未找到对应的具体篇目、辑次或页码。“寺庙商”可能是研究者分类，需同时查“寺院贸易”“喇嘛经商”等表述。定位后应记录作者、调查年代、交易路线和商品名称，以区分地方志转述与原始调查。现代出版物仅提供书目、馆藏及引用定位，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=地方志或民族商业史材料子项。关键词=松潘回族行商、松潘回商、藏商、汉商、寺院贸易、喇嘛寺经商。母项=《松潘县志》商业卷、《松潘县志》民族宗教卷、《松潘文史资料》、松潘地方商业史料。候选站=。未找到具体方志卷、文史资料辑次或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -28182,7 +28182,7 @@
       </c>
       <c r="J598" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=族谱序文。关键词=西昌沙锅营马氏祠宗谱序、沙锅营马氏、西昌马氏宗谱、马氏祠宗谱序、沙锅营 马氏 族谱。母项=《西昌马氏宗谱》、《沙锅营马氏族谱》、西昌县／西昌市地方志氏族资料、四川凉山西昌家谱目录。候选站=。未找到具体谱名、编修年代、卷次或公开家谱影印页。应以“沙锅营”“马氏祠”“西昌马氏”“宗谱序”组合检索地方志、族谱目录和家谱馆藏。；2026-09-21 gpt-6-astra：未找到。类型=族谱序文。关键词=西昌沙锅营、马氏祠、马氏宗谱、宗谱序。母项=《西昌马氏宗谱》、《沙锅营马氏族谱》、西昌县志氏族资料。候选站=。未找到具体族谱卷次、方志章节或公开谱页。；2026-09-21 gpt-6-astra：未找到。类型=族谱序文。关键词=西昌沙锅营、沙锅营马氏、马氏祠宗谱序、西昌马氏宗谱。母项=《西昌马氏宗谱》、《沙锅营马氏族谱》、西昌县志氏族资料。候选站=。未找到可核验的识典章节、族谱影印页或方志卷页URL。</t>
         </is>
       </c>
     </row>
@@ -28228,7 +28228,7 @@
       </c>
       <c r="J599" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似考古发掘简报或遗址介绍篇名。关键词=丰镇 十一窑子 战国墓、豐鎮 十一窯子 戰國墓、丰镇县 十一窑子 墓葬、丰镇市 十一窑子 发掘 简报、十一窑子 东周 墓地、十一窑子 考古 文物 内蒙古文物考古。母项=《考古》《文物》《内蒙古文物考古》：候选期刊排查范围，未确认刊载及年期、考古年鉴中的内蒙古地区发现与发掘条目：辅助反查来源，具体年份未确认。候选站=。未找到可确认的作者、期刊年期、页码或DOI，不能将候选期刊写成已知出处。先以罕见地名“十一窑子”检索，再结合丰镇旧称及“东周”“战国”筛选；若题名只见于图片说明，还需反查图片所引发掘报告。现代期刊仅给书目、馆藏或DOI线索，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘简报或墓葬调查报告。关键词=丰镇、十一窑子、战国墓、十一窑子墓地、丰镇墓葬、东周墓葬。母项=《文物》考古简报、《考古》考古发掘报告、《内蒙古文物考古》、内蒙古考古年鉴。候选站=。未找到可核验的具体期刊篇页、维基文库卷次或公开发掘报告全文页。</t>
         </is>
       </c>
     </row>
@@ -28254,12 +28254,12 @@
       </c>
       <c r="F600" s="10" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>http://www.ybsfzx.com/ldbt/beiwei010.htm</t>
         </is>
       </c>
       <c r="G600" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H600" s="10" t="inlineStr">
@@ -28269,12 +28269,12 @@
       </c>
       <c r="I600" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>北魏孝昌三年；全称《魏故咸阳太守刘府君墓志铭》。母项《汉魏南北朝墓志汇编》。</t>
         </is>
       </c>
       <c r="J600" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 核为北魏刘玉墓志，非明清同名人物。已归档释文。</t>
         </is>
       </c>
     </row>
@@ -28300,27 +28300,27 @@
       </c>
       <c r="F601" s="10" t="inlineStr">
         <is>
-          <t>https://shufawang.cn/xzmb/af6674f03ef1ae2ad53ab9c662cf9cc3.html</t>
+          <t>https://shufaziliao.com/maobi/6376a0b8ac2257e6190a777a759602e8.html</t>
         </is>
       </c>
       <c r="G601" s="10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H601" s="10" t="inlineStr">
         <is>
-          <t>不详</t>
+          <t>上海古籍出版社</t>
         </is>
       </c>
       <c r="I601" s="10" t="inlineStr">
         <is>
-          <t>唐苏日荣墓志;录文见《唐代墓志汇编》类</t>
+          <t>周绍良《唐代墓誌彙編》下；千唐志斋藏石。唐贞元十四年。</t>
         </is>
       </c>
       <c r="J601" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 核为《唐故特进行虔王傅扶风县开国伯上柱国兼英武军右厢兵马使苏公墓志铭》，房次卿撰，贞元十四年。母项《唐代墓誌彙編》下；千唐志斋藏石。原表书法网仅为拓片页，本轮改用录文页归档。</t>
         </is>
       </c>
     </row>
@@ -28366,7 +28366,7 @@
       </c>
       <c r="J602" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似文物名称、图版标题或馆藏展签。关键词=鎏金 牡丹纹 银 马鞍饰、鎏金牡丹紋銀馬鞍飾、鎏金 银鞍饰 牡丹、牡丹纹 马鞍 鞍桥 银饰、鎏金 牡丹 鞍饰 出土 馆藏。母项=收藏机构馆藏目录或展览图录：须先确认收藏单位与文物编号、出土墓葬发掘报告的马具、银器或图版部分：须先确认出土地，不能预设具体墓葬。候选站=。未找到可核验的馆藏详情页或图录页。此项更可能是器物而非书籍；缺少年代、尺寸、出土地和收藏单位，暂不能唯一识别。优先查博物馆公开藏品页，再查Commons的具体文件页及其来源字段；不能用相似器物图片代替。图录如属现代版权出版物，仅提供书目和馆藏线索。；2026-09-21 gpt-6-astra：未找到。类型=馆藏文物名称或考古图版标题。关键词=鎏金牡丹纹银马鞍饰、鎏金牡丹紋銀馬鞍飾、牡丹纹银鞍饰、银马鞍饰、鎏金马具。母项=博物馆馆藏目录、考古发掘报告马具图版、古代金银器展览图录。候选站=。未找到可核验的具体馆藏详情页、Commons文件页或考古报告图版页；缺少年代、出土地和收藏单位，无法唯一定位。</t>
         </is>
       </c>
     </row>
@@ -28412,7 +28412,7 @@
       </c>
       <c r="J603" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=疑似蒙古文档案汉译题名或档案汇编子目。关键词=察克都尔色楞 扎那济尔迪 地图、察克都爾色楞 扎那濟爾迪 地圖、扎萨克 贝子 重绘 本旗地图 呈文、扎薩克 貝子 盟長 旗圖、察克都尔色楞 舆图、扎那济尔迪 蒙古文 档案。母项=蒙古文档案汉译目录或档案选编：候选母项类别，具体汇编书名未确认、蒙古各旗地图、舆图相关档案目录：查重绘旗图的呈文、附件图及收文记录，档案馆与档号未确认。候选站=。未找到具体档案目录页、档号或汇编页码。题名采用“某人为某事呈某人文”的档案著录格式，应优先拆查两个人名，再核对任职旗盟、纪年和收发文关系。“扎萨克旗”不足以唯一确定旗名，不能擅配盟旗。人名转写变体应依据目录实证扩展；呈文与所附地图可能分开著录，找到地图不等于找到该文。；2026-09-21 gpt-6-astra：未找到。类型=档案单件。关键词=察克都尔色楞、察克都爾色楞、扎那济尔迪、扎那濟爾迪、重绘旗图、舆图。母项=蒙古王公档案、蒙古各旗舆图档案、清代蒙古档案汇编。候选站=。未找到可核验的识典章节、维基文库卷次、墓志录文页或方志卷 URL。旗名、年代及档号仍不明确。</t>
         </is>
       </c>
     </row>
@@ -28458,7 +28458,7 @@
       </c>
       <c r="J604" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清代军务奏折。关键词=伊犁将军金顺、伊犁军营、黑龙江布特哈、镶黄旗佐领、莫莫和吉、病故。母项=清代宫中档奏折、光绪朝军机处档折件、《清代新疆满文档案汉译编译》伊犁军务部分、中国第一历史档案馆清代伊犁将军奏折目录。候选站=。未找到公开具体档号、卷次或全文页。应核对人名异写“莫莫和吉／莫莫和吉氏”、旗籍“布特哈／布特哈八旗”及文种“片／奏片”。；2026-09-21 gpt-6-astra：未找到。类型=清代奏片。关键词=金顺、伊犁军营、黑龙江布特哈、镶黄旗佐领、莫莫和吉、议恤片。母项=光绪朝军机处档折件、清代宫中档奏折、清代新疆满文档案汉译编译。候选站=。未找到具体档号、卷次或公开全文页。；2026-09-21 gpt-6-astra：未找到。类型=清代奏片。关键词=金顺、伊犁军营、黑龙江布特哈、镶黄旗佐领、莫莫和吉、议恤片。母项=光绪朝军机处档折件、清代宫中档奏折、清代新疆满文档案汉译编译。候选站=。未找到可对应本条的具体档号、卷册或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -28504,7 +28504,7 @@
       </c>
       <c r="J605" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清末公文档案单件。关键词=直隶总督 袁世凯 咨复 邱廷荣、袁世凯 邱廷荣 酌委、直隶总督咨文 光绪 宣统、邱廷荣 任用 酌委。母项=《袁世凯奏议》、《清代军机处档折件》、《清代朱批奏折》、直隶总督衙门档案。候选站=https://zh.wikisource.org/w/index.php?search=%E7%9B%B4%E9%9A%B6%E6%80%BB%E7%9D%A3+%E8%A2%81%E4%B8%96%E5%87%AF+%E9%82%B1%E5%BB%B7%E8%8D%A3。疑为直隶总督衙门档案或奏折汇编中的单件文书，不能按独立书名检索；需以档号、日期、邱廷荣任职地点或事由继续核对。；2026-09-21 gpt-6-astra：未找到。类型=清末公文档案。关键词=袁世凯、邱廷荣、直隶总督、咨复、酌委、直隶总督衙门。母项=直隶总督衙门档案、袁世凯奏议、清末军政档案。候选站=。未找到可核验的具体全文页或方志卷 URL。缺少日期、任职地点及档号，无法可靠定位。</t>
         </is>
       </c>
     </row>
@@ -28550,7 +28550,7 @@
       </c>
       <c r="J606" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清末奏折抄件。关键词=山西巡抚岑春煊、恳开晋边蒙地屯垦、恤藩属、弥隐患、晋边蒙地、屯垦折。母项=《岑春煊集》奏稿及奏折部分、清末军机处档折件、《清季外交史料》蒙地与边务相关奏折、山西省档案馆清末山西巡抚档案、《清末筹蒙档案》。候选站=。未找到具体卷次、档号或可核验的公开抄件页面。应按岑春煊任山西巡抚时期检索，并同时使用“晋边”“蒙地”“屯垦”“藩属”“弥隐患”“折片”等短语。；2026-09-21 gpt-6-astra：未找到。类型=清末奏折抄件。关键词=岑春煊、晋边蒙地、屯垦、恤藩属、弥隐患、折片抄件。母项=《岑春煊集》、《清末筹蒙档案》、清末军机处档折件、《清季外交史料》。候选站=。未找到具体卷次、档号、方志章节或公开抄件页面。；2026-09-21 gpt-6-astra：未找到。类型=清末奏折抄件。关键词=岑春煊、晋边蒙地、屯垦、恤藩属、弥隐患、折片抄件。母项=《岑春煊集》、《清末筹蒙档案》、《清季外交史料》、清末军机处档折件。候选站=。未找到可核验的具体卷次、档号或抄件页面URL。</t>
         </is>
       </c>
     </row>
@@ -28596,7 +28596,7 @@
       </c>
       <c r="J607" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=中共地方组织史资料条目或档案专题。关键词=中共归绥工作委员会、归绥工作委员会、绥远 归绥 中共 工委、呼和浩特 党史 归绥、归绥地下党。母项=《中国共产党内蒙古自治区组织史资料》、《内蒙古革命史》、《呼和浩特市志》党政卷、《绥远革命史料》。候选站=https://zh.wikisource.org/w/index.php?search=%E4%B8%AD%E5%85%B1%E5%BD%92%E7%BB%A5%E5%B7%A5%E4%BD%9C%E5%A7%94%E5%91%98%E4%BC%9A; https://commons.wikimedia.org/w/index.php?search=%E5%BD%92%E7%BB%A5%E5%B7%A5%E4%BD%9C%E5%A7%94%E5%91%98%E4%BC%9A&amp;title=Special:MediaSearch&amp;type=image。题名更像党史资料中的小节或组织沿革条目；应按成立年代、负责人、归绥所属上级组织和《组织史资料》卷册定位。；2026-09-21 gpt-6-astra：未找到。类型=党史资料条目。关键词=中共归绥工作委员会、归绥工委、绥远地下党、归绥党组织、呼和浩特党史。母项=中国共产党内蒙古自治区组织史资料、呼和浩特市志、绥远革命史料。候选站=。未找到可核验的具体章节或方志卷 URL。成立年代、负责人和上级组织尚未确定。</t>
         </is>
       </c>
     </row>
@@ -28642,7 +28642,7 @@
       </c>
       <c r="J608" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=抗日战争时期中共中央及八路军电报。关键词=大青山 游击根据地 指示电、毛泽东 王稼祥 杨尚昆 贺龙 关向应 周士第 甘泗淇 李井泉、团结蒙汉抗日 绥远、大青山抗日根据地 电报、1938 大青山 绥远。母项=《毛泽东文集》、《毛泽东军事文集》、《中共中央文件选集》、《八路军军政杂志》、《抗日战争时期八路军文件汇编》、《晋绥边区革命史料》。候选站=https://zh.wikisource.org/w/index.php?search=%E5%A4%A7%E9%9D%92%E5%B1%B1+%E6%B8%B8%E5%87%BB%E6%A0%B9%E6%8D%AE%E5%9C%B0+%E6%8C%87%E7%A4%BA%E7%94%B5; https://commons.wikimedia.org/w/index.php?search=%E5%A4%A7%E9%9D%92%E5%B1%B1%E6%8A%97%E6%97%A5%E6%A0%B9%E6%8D%AE%E5%9C%B0&amp;title=Special:MediaSearch&amp;type=image。很可能收入《中共中央文件选集》或八路军电报汇编，题名可能是整理者拟题；需先确定发电日期，再查卷次、文号和收文机关。；2026-09-21 gpt-6-astra：未找到。类型=抗战时期电报。关键词=大青山游击根据地、团结蒙汉抗日、绥远问题、周士第、甘泗淇、李井泉。母项=中共中央文件选集、毛泽东军事文集、晋绥边区革命史料。候选站=。未找到可核验的维基文库具体卷次或章节 URL。发电日期、文号和编入母项尚未确认。</t>
         </is>
       </c>
     </row>
@@ -28688,7 +28688,7 @@
       </c>
       <c r="J609" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=民国报刊战事电讯。关键词=1946年9月14日 集宁 血战、集宁内外 连日血战、国军 冲入 占领各高地、共军 迭增援 集宁、集宁战役 绥东战役 1946。母项=《中央日报》1946年9月号、《大公报》1946年9月号、《申报》1946年9月号、《扫荡报》1946年9月号、《中华民国史档案资料汇编》内战时期军事资料。候选站=https://commons.wikimedia.org/w/index.php?search=%E9%9B%86%E5%AE%81%E6%88%98%E5%BD%B9+1946&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=1946%E5%B9%B49%E6%9C%8814%E6%97%A5+%E9%9B%86%E5%AE%81。题名明显是报刊标题或数据库拟题，不是独立著作；应逐日查1946年9月14日至16日的《中央日报》《大公报》《申报》等版面。；2026-09-21 gpt-6-astra：未找到。类型=民国报刊标题。关键词=1946年9月14日、集宁、集宁战役、连日血战、国军占领高地、共军增援。母项=中央日报、大公报、申报、扫荡报。候选站=。未找到可核验的报刊版面、维基文库卷次或 Commons 具体图像页 URL。</t>
         </is>
       </c>
     </row>
@@ -28734,7 +28734,7 @@
       </c>
       <c r="J610" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=清末蒙古王公及军政档案奏牍。关键词=蒙古世爵 培钰 义勇队、培钰 军咨大臣、组织义勇队 上军咨大臣书、蒙古王公 义勇队 清末、军咨大臣 蒙古。母项=《清末筹备立宪档案史料》、《清末新军编练与蒙古问题档案》、《清代蒙古史料》、《外务部档案》、军咨处及陆军部档案。候选站=https://zh.wikisource.org/w/index.php?search=%E5%9F%B9%E9%92%B0+%E4%B9%89%E5%8B%87%E9%98%9F+%E5%86%9B%E5%92%A8%E5%A4%A7%E8%87%A3; https://commons.wikimedia.org/w/index.php?search=%E5%9F%B9%E9%92%B0+%E8%BB%8D%E5%92%A8%E5%A4%A7%E8%87%A3&amp;title=Special:MediaSearch&amp;type=image。疑为清末军咨处、陆军部或蒙古王公档案中的来文；需补查培钰的爵位、旗籍、文书日期及“蒙古世爵”原始著录格式。；2026-09-21 gpt-6-astra：未找到。类型=清末蒙古王公档案。关键词=培钰、蒙古世爵、义勇队、军咨大臣、陆军部、蒙古王公。母项=清末筹备立宪档案史料、清末新军档案、清代蒙古史料。候选站=。未找到可核验的具体卷次或档案页 URL。培钰的旗籍、爵位和文书日期未确认。</t>
         </is>
       </c>
     </row>
@@ -28872,7 +28872,7 @@
       </c>
       <c r="J613" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=现代学术论文或论文集章节。关键词=蒙汉历史接触与蒙古语言文化变迁、蒙汉接触 蒙古语言文化变迁、蒙古语言 汉语接触、蒙古族语言文化 历史接触。母项=蒙古语言学论文集、蒙古族历史与文化研究论文集、《民族语文》相关年份期刊、《内蒙古社会科学》相关年份期刊、《中央民族大学学报》相关年份期刊。候选站=https://zh.wikisource.org/w/index.php?search=%E8%92%99%E6%B1%89%E5%8E%86%E5%8F%B2%E6%8E%A5%E8%A7%A6%E4%B8%8E%E8%92%99%E5%8F%A4%E8%AF%AD%E8%A8%80%E6%96%87%E5%8C%96%E5%8F%98%E8%BF%81; https://commons.wikimedia.org/w/index.php?search=%E8%92%99%E6%B1%89%E5%8E%86%E5%8F%B2%E6%8E%A5%E8%A7%A6&amp;title=Special:MediaSearch&amp;type=image。未能确认作者、刊名、年份和卷期；2015年后整理本或现代期刊通常只能提供书目、馆藏或 DOI 线索，不能据此宣称整本可下载。；2026-09-21 gpt-6-astra：未找到。类型=现代学术论文或论文集章节。关键词=蒙汉历史接触、蒙古语言文化变迁、蒙古语言接触、汉语影响蒙古语。母项=民族语文、内蒙古社会科学、中央民族大学学报、蒙古语言学论文集。候选站=。未确认作者、刊名、年份、卷期或 DOI，未找到可核验的具体章节 URL。</t>
         </is>
       </c>
     </row>
@@ -28918,7 +28918,7 @@
       </c>
       <c r="J614" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古简报或文物图录条目。关键词=昭通 耕牛 画像砖、昭通画像砖、云南汉代画像砖 耕牛、昭通汉墓 画像砖、耕牛画像砖 出土。母项=《昭通地区汉墓》、《云南文物考古资料集》、《中国画像石全集》、《云南省志·文物志》、《昭通市志·文化文物志》。候选站=https://commons.wikimedia.org/w/index.php?search=%E6%98%AD%E9%80%9A+%E8%80%95%E7%89%9B+%E7%94%BB%E5%83%8F%E7%A0%96&amp;title=Special:MediaSearch&amp;type=image; https://zh.wikisource.org/w/index.php?search=%E6%98%AD%E9%80%9A+%E7%94%BB%E5%83%8F%E7%A0%96。题名可能是图录中的单件器物或图片说明，不是独立论文；应以墓葬名称、出土地点、文物编号和图版号定位。；2026-09-21 gpt-6-astra：未找到。类型=考古图录或文物条目。关键词=昭通、耕牛画像砖、昭通画像砖、汉墓画像砖、云南画像砖。母项=昭通地区汉墓、中国画像石全集、云南省志·文物志、昭通市志·文化文物志。候选站=。未找到可核验的墓志录文页、方志卷 URL 或 Commons 具体图像页。墓葬名称、出土地和文物编号尚不明确。</t>
         </is>
       </c>
     </row>
@@ -29011,7 +29011,7 @@
       </c>
       <c r="J616" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=地方经济史资料或地方志章节。关键词=建国前 泸水 集市贸易、泸水集市贸易概况、泸水县 集市 贸易 民国、怒江 泸水 商贸史、泸水地方志 集市。母项=《泸水县志》、《泸水市志》、《怒江傈僳族自治州志》、《云南省志·商业志》、泸水地方经济社会调查资料。候选站=https://zh.wikisource.org/w/index.php?search=%E5%BB%BA%E5%9B%BD%E5%89%8D+%E6%B3%B8%E6%B0%B4+%E9%9B%86%E5%B8%82%E8%B4%B8%E6%98%93; https://commons.wikimedia.org/w/index.php?search=%E6%B3%B8%E6%B0%B4%E5%8E%BF%E5%BF%97&amp;title=Special:MediaSearch&amp;type=image。题名很可能是《泸水县志》或地方经济调查中的专题小节；需补查旧称“碧江”、泸水设治局、六库、片马及民国时期商号和集市名称。；2026-09-21 gpt-6-astra：未找到。类型=地方志章节或地方经济调查资料。关键词=建国前泸水集市贸易、泸水县 集市、泸水设治局 商业、碧江 集市、六库 片马 商贸。母项=《泸水县志》、《泸水市志》、《怒江傈僳族自治州志》、《云南省志·商业志》。候选站=。未核到具体方志卷、章节或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -29057,7 +29057,7 @@
       </c>
       <c r="J617" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=地方文献辑刊或文集选辑。关键词=云南杂志选辑、雲南雜誌選輯、云南杂志、雲南雜誌、云南地方文献、云南省志。母项=《云南杂志》、云南地方文献丛刊、《云南文史资料》、云南省地方志。候选站=https://zh.wikisource.org/w/index.php?search=%E9%9B%B2%E5%8D%97%E9%9B%9C%E8%AA%8C; https://commons.wikimedia.org/w/index.php?search=%E9%9B%B2%E5%8D%97%E9%9B%9C%E8%AA%8C&amp;title=Special:MediaSearch&amp;type=image。未核到具体书名、卷次或可直接核验的全文页。应按《云南杂志》的出版地、年份、卷期及编者继续查地方志目录和报刊目录。；2026-09-21 gpt-6-astra：未找到。类型=地方文献辑刊或报刊选辑。关键词=云南杂志选辑、雲南雜誌選輯、云南杂志、雲南雜誌、云南地方文献。母项=《云南杂志》、云南地方文献丛刊、《云南文史资料》。候选站=。未核到具体编者、出版年份、卷册或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -29103,7 +29103,7 @@
       </c>
       <c r="J618" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=教育行政公报或连续出版物。关键词=云南教育公报、雲南教育公報、云南省教育公报、云南教育厅公报、云南教育行政、韦广波。母项=云南省教育厅档案、云南省政府公报、云南教育史料、云南地方报刊。候选站=https://zh.wikisource.org/w/index.php?search=%E9%9B%B2%E5%8D%97%E6%95%99%E8%82%B2%E5%85%AC%E5%A0%B1; https://commons.wikimedia.org/w/index.php?search=%E9%9B%B2%E5%8D%97%E6%95%99%E8%82%B2%E5%85%AC%E5%A0%B1&amp;title=Special:MediaSearch&amp;type=image。未核到具体年份、期号或馆藏扫描页。应扩大为云南省教育厅、云南省政府公报及教育行政档案中的分项文件检索。；2026-09-21 gpt-6-astra：未找到。类型=教育行政公报。关键词=云南教育公报、雲南教育公報、云南省教育厅公报、云南教育行政公报、云南省政府公报 教育。母项=云南省教育厅档案、云南省政府公报、云南教育史料。候选站=。未核到具体年份、期号、卷册或公开扫描页。</t>
         </is>
       </c>
     </row>
@@ -29149,7 +29149,7 @@
       </c>
       <c r="J619" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=考古发掘简报或报告子项。关键词=绥滨县 奥里米 辽金墓葬、绥滨 奥里米墓地、奥里米古城 墓葬 发掘、韦广波。母项=《黑龙江省文物考古研究所集刊》相关考古发掘简报、《中国考古学年鉴》黑龙江省考古发掘条目、绥滨县奥里米古城遗址考古报告或文集。候选站=。未找到可核验的具体书名卷次、期刊年期或公开全文页。建议以“奥里米古城”“奥里米墓地”“辽金墓葬”“绥滨”组合检索黑龙江省文物考古研究所刊物及《中国考古学年鉴》；该题名可能是发掘简报中的章节或图版说明，不一定为独立出版物。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘简报或报告子项，待核。关键词=绥滨县 奥里米 辽金墓葬、綏濱縣 奧里米 遼金墓葬、奥里米 墓地 抢救性发掘、奥里米古城 发掘简报。母项=《黑龙江省文物考古研究所集刊》（待查）、《中国考古学年鉴》黑龙江考古条目（待查）。候选站=。当前环境无联网检索工具，无法实际完成新一轮网页核验；未取得符合要求的具体页面。应先核对简报作者、发表年期及页码；原线索中的“韦广波”与本条关系未经证实。若为现代期刊文章，仅提供书目、馆藏或DOI线索，不提供整本下载。；2026-09-21 gpt-6-astra：未找到。类型=考古发掘简报或报告子项。关键词=绥滨县奥里米、奥里米辽金墓葬、奥里米墓地、奥里米古城、抢救性发掘。母项=《黑龙江省文物考古研究所集刊》、《中国考古学年鉴》黑龙江考古条目、奥里米古城遗址考古报告。候选站=。未找到可核验的具体期刊卷期、章节页或公开全文URL。</t>
         </is>
       </c>
     </row>
@@ -29241,7 +29241,7 @@
       </c>
       <c r="J621" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=现代语言学论文。关键词=作为古百越语底层形式的先喉塞音、先喉塞音、古百越语、南方汉语方言、喉塞音、韦广波。母项=汉语方言学期刊论文、古百越语研究论文集、南方方言调查资料。候选站=https://scholar.google.com/scholar?q=%22%E4%BD%9C%E4%B8%BA%E5%8F%A4%E7%99%BE%E8%B6%8A%E8%AF%AD%E5%BA%95%E5%B1%82%E5%BD%A2%E5%BC%8F%22; https://www.cnki.com.cn/Article/CJFDTotal-GYYY.htm。未核到具体刊名、年份、期号、页码或 DOI。不能据题名确认其为独立著作。；2026-09-21 gpt-6-astra：未找到。类型=现代语言学论文。关键词=作为古百越语底层形式的先喉塞音、古百越语、先喉塞音、南方汉语方言、喉塞音。母项=汉语方言学期刊论文、古百越语研究论文集、南方方言调查资料。候选站=。未核到刊名、年份、卷期、页码或 DOI；不能据题名确认独立出版物。</t>
         </is>
       </c>
     </row>
@@ -29287,7 +29287,7 @@
       </c>
       <c r="J622" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=期刊文章或通讯。关键词=东方杂志到苗区去、到苗区去、苗区、东方杂志、雲南苗族、韦广波。母项=《东方杂志》、《东方杂誌》、近代民族调查通讯。候选站=https://zh.wikisource.org/w/index.php?search=%E6%9D%B1%E6%96%B9%E9%9B%9C%E8%AA%8C%E5%88%B0%E8%8B%97%E5%8D%80%E5%8E%BB; https://archive.org/advancedsearch.php?title=%E6%9D%B1%E6%96%B9%E9%9B%9C%E8%AA%8C&amp;fl%5B%5D=identifier,title&amp;rows=50&amp;page=1&amp;output=json。未核到具体卷、期、年份和页码。应在《东方杂志》民国时期各卷目录中检索“苗区”“苗族”“贵州”“云南”等关键词。；2026-09-21 gpt-6-astra：未找到。类型=近代期刊文章或通讯。关键词=东方杂志 到苗区去、到苗区去、苗区、东方杂誌 苗族、云南 苗族。母项=《东方杂志》、《东方雜誌》、近代民族调查通讯。候选站=。未核到《东方杂志》的具体卷、期、年份、页码或公开全文页。</t>
         </is>
       </c>
     </row>
@@ -29333,7 +29333,7 @@
       </c>
       <c r="J623" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=革命史料汇编子项。关键词=红军在贵州史料汇编 长征日记、红军长征日记 贵州、贵州革命史料汇编 上册、韦广波。母项=《红军在贵州史料汇编》上册、贵州省革命文物与党史资料汇编、贵州省档案馆、贵州省地方志系统红军长征史料丛书。候选站=。未找到可核验的具体版本、编者、出版社或公开全文页。题名结构显示“长征日记”很可能是《红军在贵州史料汇编》上册的篇章或分册标题，应继续按汇编书名、编印机关和出版年份检索地方党史资料目录及馆藏。；2026-09-21 gpt-6-astra：未找到。类型=革命史料汇编子项，待核。关键词=红军在贵州 史料汇编 上册 长征日记、紅軍在貴州 史料彙編 長征日記、红军在贵州 目录 日记、长征日记 作者 贵州。母项=《红军在贵州史料汇编》上册（据所给题名，待核）。候选站=。无法联网核验，未取得具体章节或卷次URL。“长征日记”的作者、篇名边界及所在页码均未确认，不能以其他同名日记替代。应由母书目录核对子项，再查作者文集或日记原刊；版权期内汇编不可整本下载。；2026-09-21 gpt-6-astra：未找到。类型=革命史料汇编子项。关键词=红军在贵州史料汇编、长征日记、贵州红军史料、红軍在貴州史料彙編。母项=《红军在贵州史料汇编》上册、贵州革命史料汇编、贵州党史资料汇编。候选站=。未找到可核验的具体章节、目录页或卷册URL；作者和篇章边界仍未确认。</t>
         </is>
       </c>
     </row>
@@ -29425,7 +29425,7 @@
       </c>
       <c r="J625" s="9" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>2026-09-21 gpt-6-astra：未找到。类型=碑刻录文或地方文献子项。关键词=惠水县 摆金 永垂场碑、咸丰元年 永垂场碑、摆金碑刻、惠水 碑刻录文、韦广波。母项=《贵州碑刻》或贵州地方碑刻辑录、《惠水县志》及续修惠水县志、《贵州民族地区碑刻资料集》、惠水县文物志或摆金镇地方文史资料。候选站=。未找到具体录文页、卷次或可公开核验全文。题名带有年代、地点和碑名，较可能是碑刻调查目录、地方文物志或专题文章中的单条录文，不宜按独立书籍检索。；2026-09-21 gpt-6-astra：未找到。类型=地方碑刻录文。关键词=惠水 摆金 永垂场碑、惠水 擺金 永垂場碑、摆金 咸丰元年 碑文、摆金 1851 场碑、惠水县志 金石 碑刻 摆金。母项=《惠水县志》（待查具体版本及卷次）、摆金地方文史、碑刻调查资料（具体书名待核）。候选站=。无法联网核验，未取得碑刻录文页或方志卷URL。应核对“永垂场碑”是否为原碑题额、调查者拟题或转录误字，并以咸丰元年、摆金及碑文首尾句定位；不能将尚未确认的碑刻汇编当作已知收录来源。；2026-09-21 gpt-6-astra：未找到。类型=碑刻录文。关键词=惠水摆金永垂场碑、咸丰元年永垂场碑、摆金碑刻、惠水碑刻录文。母项=《惠水县志》、贵州地方碑刻辑录、惠水县文物志、摆金地方文史资料。候选站=。未找到可核验的墓志录文页、方志卷页或碑刻图录URL。</t>
         </is>
       </c>
     </row>

</xml_diff>